<commit_message>
BCC tracker: session 2026-09-23
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q234"/>
+  <dimension ref="A1:Q250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4268,7 +4268,21 @@
       <c r="D109" t="n">
         <v>245.96</v>
       </c>
+      <c r="E109" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K109" t="inlineStr"/>
+      <c r="L109" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="M109" t="n">
+        <v>-0.79</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4289,7 +4303,21 @@
       <c r="D110" t="n">
         <v>52.71</v>
       </c>
+      <c r="E110" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K110" t="inlineStr"/>
+      <c r="L110" t="n">
+        <v>-2.16</v>
+      </c>
+      <c r="M110" t="n">
+        <v>-0.87</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4310,7 +4338,21 @@
       <c r="D111" t="n">
         <v>250.54</v>
       </c>
+      <c r="E111" t="n">
+        <v>-5.21</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K111" t="inlineStr"/>
+      <c r="L111" t="n">
+        <v>-7.03</v>
+      </c>
+      <c r="M111" t="n">
+        <v>-2.84</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4331,7 +4373,21 @@
       <c r="D112" t="n">
         <v>490.3</v>
       </c>
+      <c r="E112" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K112" t="inlineStr"/>
+      <c r="L112" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="M112" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4352,7 +4408,21 @@
       <c r="D113" t="n">
         <v>139.82</v>
       </c>
+      <c r="E113" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K113" t="inlineStr"/>
+      <c r="L113" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="M113" t="n">
+        <v>1.15</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4373,7 +4443,21 @@
       <c r="D114" t="n">
         <v>174.34</v>
       </c>
+      <c r="E114" t="n">
+        <v>10</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K114" t="inlineStr"/>
+      <c r="L114" t="n">
+        <v>8.18</v>
+      </c>
+      <c r="M114" t="n">
+        <v>8.890000000000001</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4394,7 +4478,21 @@
       <c r="D115" t="n">
         <v>52.71</v>
       </c>
+      <c r="E115" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K115" t="inlineStr"/>
+      <c r="L115" t="n">
+        <v>-2.16</v>
+      </c>
+      <c r="M115" t="n">
+        <v>-0.87</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4415,7 +4513,21 @@
       <c r="D116" t="n">
         <v>547.4299999999999</v>
       </c>
+      <c r="E116" t="n">
+        <v>-6.76</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K116" t="inlineStr"/>
+      <c r="L116" t="n">
+        <v>-8.58</v>
+      </c>
+      <c r="M116" t="n">
+        <v>-7.39</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4436,7 +4548,21 @@
       <c r="D117" t="n">
         <v>190.28</v>
       </c>
+      <c r="E117" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K117" t="inlineStr"/>
+      <c r="L117" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="M117" t="n">
+        <v>3.34</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4457,7 +4583,21 @@
       <c r="D118" t="n">
         <v>191.58</v>
       </c>
+      <c r="E118" t="n">
+        <v>12.02</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K118" t="inlineStr"/>
+      <c r="L118" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="M118" t="n">
+        <v>11.67</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4478,7 +4618,21 @@
       <c r="D119" t="n">
         <v>104.96</v>
       </c>
+      <c r="E119" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K119" t="inlineStr"/>
+      <c r="L119" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="M119" t="n">
+        <v>2.81</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4499,7 +4653,21 @@
       <c r="D120" t="n">
         <v>229.71</v>
       </c>
+      <c r="E120" t="n">
+        <v>13.58</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K120" t="inlineStr"/>
+      <c r="L120" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="M120" t="n">
+        <v>8.58</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4520,7 +4688,21 @@
       <c r="D121" t="n">
         <v>490.3</v>
       </c>
+      <c r="E121" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K121" t="inlineStr"/>
+      <c r="L121" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4541,7 +4723,21 @@
       <c r="D122" t="n">
         <v>331.02</v>
       </c>
+      <c r="E122" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K122" t="inlineStr"/>
+      <c r="L122" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0.14</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4562,7 +4758,21 @@
       <c r="D123" t="n">
         <v>34.84</v>
       </c>
+      <c r="E123" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K123" t="inlineStr"/>
+      <c r="L123" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="M123" t="n">
+        <v>8.369999999999999</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4583,7 +4793,21 @@
       <c r="D124" t="n">
         <v>332.41</v>
       </c>
+      <c r="E124" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K124" t="inlineStr"/>
+      <c r="L124" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0.55</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4604,7 +4828,21 @@
       <c r="D125" t="n">
         <v>512.5</v>
       </c>
+      <c r="E125" t="n">
+        <v>19.98</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K125" t="inlineStr"/>
+      <c r="L125" t="n">
+        <v>18.16</v>
+      </c>
+      <c r="M125" t="n">
+        <v>15.14</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4625,7 +4863,21 @@
       <c r="D126" t="n">
         <v>270.02</v>
       </c>
+      <c r="E126" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K126" t="inlineStr"/>
+      <c r="L126" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="M126" t="n">
+        <v>-2.92</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4646,7 +4898,21 @@
       <c r="D127" t="n">
         <v>44.95</v>
       </c>
+      <c r="E127" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K127" t="inlineStr"/>
+      <c r="L127" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="M127" t="n">
+        <v>5.45</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4667,7 +4933,21 @@
       <c r="D128" t="n">
         <v>241.36</v>
       </c>
+      <c r="E128" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K128" t="inlineStr"/>
+      <c r="L128" t="n">
+        <v>6.94</v>
+      </c>
+      <c r="M128" t="n">
+        <v>11.11</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4688,7 +4968,21 @@
       <c r="D129" t="n">
         <v>563.29</v>
       </c>
+      <c r="E129" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K129" t="inlineStr"/>
+      <c r="L129" t="n">
+        <v>-4.22</v>
+      </c>
+      <c r="M129" t="n">
+        <v>-3.71</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4709,7 +5003,21 @@
       <c r="D130" t="n">
         <v>119.46</v>
       </c>
+      <c r="E130" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K130" t="inlineStr"/>
+      <c r="L130" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="M130" t="n">
+        <v>4.18</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4730,7 +5038,21 @@
       <c r="D131" t="n">
         <v>324.65</v>
       </c>
+      <c r="E131" t="n">
+        <v>8.57</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K131" t="inlineStr"/>
+      <c r="L131" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="M131" t="n">
+        <v>9.84</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4751,7 +5073,21 @@
       <c r="D132" t="n">
         <v>150.88</v>
       </c>
+      <c r="E132" t="n">
+        <v>-1.64</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K132" t="inlineStr"/>
+      <c r="L132" t="n">
+        <v>-3.46</v>
+      </c>
+      <c r="M132" t="n">
+        <v>-3.61</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4772,7 +5108,21 @@
       <c r="D133" t="n">
         <v>34.84</v>
       </c>
+      <c r="E133" t="n">
+        <v>14.45</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K133" t="inlineStr"/>
+      <c r="L133" t="n">
+        <v>12.63</v>
+      </c>
+      <c r="M133" t="n">
+        <v>8.369999999999999</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4793,7 +5143,21 @@
       <c r="D134" t="n">
         <v>139.82</v>
       </c>
+      <c r="E134" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K134" t="inlineStr"/>
+      <c r="L134" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="M134" t="n">
+        <v>1.15</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4814,7 +5178,21 @@
       <c r="D135" t="n">
         <v>23.17</v>
       </c>
+      <c r="E135" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K135" t="inlineStr"/>
+      <c r="L135" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="M135" t="n">
+        <v>5.81</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4835,7 +5213,21 @@
       <c r="D136" t="n">
         <v>190.28</v>
       </c>
+      <c r="E136" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K136" t="inlineStr"/>
+      <c r="L136" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="M136" t="n">
+        <v>3.34</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6894,6 +7286,342 @@
         <v>1094.58</v>
       </c>
       <c r="K234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>237.49</v>
+      </c>
+      <c r="K235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>500.78</v>
+      </c>
+      <c r="K236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>140.81</v>
+      </c>
+      <c r="K237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>191.77</v>
+      </c>
+      <c r="K238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>197.25</v>
+      </c>
+      <c r="K239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>510.45</v>
+      </c>
+      <c r="K240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>214.61</v>
+      </c>
+      <c r="K241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>EWY</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>185.73</v>
+      </c>
+      <c r="K242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>154.44</v>
+      </c>
+      <c r="K243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>226.42</v>
+      </c>
+      <c r="K244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>225.51</v>
+      </c>
+      <c r="K245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>ALAB</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>360.44</v>
+      </c>
+      <c r="K246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>332.56</v>
+      </c>
+      <c r="K247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>DRAM</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>61.84</v>
+      </c>
+      <c r="K248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>122.71</v>
+      </c>
+      <c r="K249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>1071.43</v>
+      </c>
+      <c r="K250" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7021,22 +7749,22 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>40</v>
+        <v>42.9</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.46</v>
+        <v>-0.18</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.19</v>
+        <v>-1.22</v>
       </c>
       <c r="G2" t="n">
-        <v>40</v>
+        <v>28.6</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.98</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -7052,25 +7780,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C3" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D3" t="n">
-        <v>51.6</v>
+        <v>53.8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08</v>
+        <v>0.45</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.95</v>
+        <v>-0.74</v>
       </c>
       <c r="G3" t="n">
-        <v>38.7</v>
+        <v>41</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.09</v>
+        <v>0.3</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -7086,25 +7814,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C4" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>73.09999999999999</v>
+        <v>76.7</v>
       </c>
       <c r="E4" t="n">
-        <v>3.43</v>
+        <v>3.64</v>
       </c>
       <c r="F4" t="n">
-        <v>2.74</v>
+        <v>2.79</v>
       </c>
       <c r="G4" t="n">
-        <v>61.5</v>
+        <v>63.3</v>
       </c>
       <c r="H4" t="n">
-        <v>3.69</v>
+        <v>3.6</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -7123,22 +7851,22 @@
         <v>18</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
         <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>7.08</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
-        <v>5.64</v>
+        <v>6.51</v>
       </c>
       <c r="G5" t="n">
         <v>100</v>
       </c>
       <c r="H5" t="n">
-        <v>7.77</v>
+        <v>7.84</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -7154,25 +7882,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C6" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D6" t="n">
-        <v>80</v>
+        <v>79.3</v>
       </c>
       <c r="E6" t="n">
-        <v>3.42</v>
+        <v>3.92</v>
       </c>
       <c r="F6" t="n">
-        <v>1.98</v>
+        <v>2.36</v>
       </c>
       <c r="G6" t="n">
-        <v>65</v>
+        <v>65.5</v>
       </c>
       <c r="H6" t="n">
-        <v>4.83</v>
+        <v>4.57</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -7188,25 +7916,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C7" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D7" t="n">
-        <v>44.4</v>
+        <v>54.5</v>
       </c>
       <c r="E7" t="n">
-        <v>-1.03</v>
+        <v>0.14</v>
       </c>
       <c r="F7" t="n">
-        <v>-2.31</v>
+        <v>-1.24</v>
       </c>
       <c r="G7" t="n">
-        <v>22.2</v>
+        <v>31.8</v>
       </c>
       <c r="H7" t="n">
-        <v>0.67</v>
+        <v>1.4</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-09-24
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q256"/>
+  <dimension ref="A1:Q277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,6 +531,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G2" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>-5.69</v>
@@ -538,6 +546,12 @@
       <c r="M2" t="n">
         <v>-6.27</v>
       </c>
+      <c r="N2" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-3.37</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -562,6 +576,14 @@
         <v>-0.79</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -573,6 +595,12 @@
       <c r="M3" t="n">
         <v>-1.92</v>
       </c>
+      <c r="N3" t="n">
+        <v>-3.34</v>
+      </c>
+      <c r="O3" t="n">
+        <v>-3.21</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -636,6 +664,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>3.9</v>
@@ -643,6 +679,12 @@
       <c r="M5" t="n">
         <v>3.71</v>
       </c>
+      <c r="N5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="O5" t="n">
+        <v>5.21</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -667,6 +709,14 @@
         <v>1.08</v>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -678,6 +728,12 @@
       <c r="M6" t="n">
         <v>0.32</v>
       </c>
+      <c r="N6" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.29</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -702,6 +758,14 @@
         <v>5.57</v>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -713,6 +777,12 @@
       <c r="M7" t="n">
         <v>6.01</v>
       </c>
+      <c r="N7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O7" t="n">
+        <v>5.48</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -737,6 +807,14 @@
         <v>6.26</v>
       </c>
       <c r="F8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>16.13</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -748,6 +826,12 @@
       <c r="M8" t="n">
         <v>4.74</v>
       </c>
+      <c r="N8" t="n">
+        <v>14.89</v>
+      </c>
+      <c r="O8" t="n">
+        <v>14.48</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -772,6 +856,14 @@
         <v>-0.6899999999999999</v>
       </c>
       <c r="F9" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -783,6 +875,12 @@
       <c r="M9" t="n">
         <v>-0.79</v>
       </c>
+      <c r="N9" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="O9" t="n">
+        <v>-1.43</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -951,6 +1049,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G14" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>-1.83</v>
@@ -958,6 +1064,12 @@
       <c r="M14" t="n">
         <v>-2.61</v>
       </c>
+      <c r="N14" t="n">
+        <v>-5.54</v>
+      </c>
+      <c r="O14" t="n">
+        <v>-5.67</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -982,6 +1094,14 @@
         <v>-4.5</v>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -993,6 +1113,12 @@
       <c r="M15" t="n">
         <v>-5.6</v>
       </c>
+      <c r="N15" t="n">
+        <v>-1.96</v>
+      </c>
+      <c r="O15" t="n">
+        <v>-1.86</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1017,6 +1143,14 @@
         <v>1.08</v>
       </c>
       <c r="F16" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1028,6 +1162,12 @@
       <c r="M16" t="n">
         <v>0.32</v>
       </c>
+      <c r="N16" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.29</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1091,6 +1231,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G18" t="n">
+        <v>16.13</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>5.63</v>
@@ -1098,6 +1246,12 @@
       <c r="M18" t="n">
         <v>4.74</v>
       </c>
+      <c r="N18" t="n">
+        <v>14.89</v>
+      </c>
+      <c r="O18" t="n">
+        <v>14.48</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1124,6 +1278,14 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -1133,6 +1295,12 @@
       <c r="M19" t="n">
         <v>-5.88</v>
       </c>
+      <c r="N19" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="O19" t="n">
+        <v>2.26</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1231,6 +1399,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G22" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
         <v>-0.11</v>
@@ -1238,6 +1414,12 @@
       <c r="M22" t="n">
         <v>-0.4</v>
       </c>
+      <c r="N22" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="O22" t="n">
+        <v>4.42</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1262,6 +1444,14 @@
         <v>3.19</v>
       </c>
       <c r="F23" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1273,6 +1463,12 @@
       <c r="M23" t="n">
         <v>2.82</v>
       </c>
+      <c r="N23" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="O23" t="n">
+        <v>2.47</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1299,6 +1495,14 @@
       <c r="F24" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -1308,6 +1512,12 @@
       <c r="M24" t="n">
         <v>-3.22</v>
       </c>
+      <c r="N24" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="O24" t="n">
+        <v>6.48</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1332,6 +1542,14 @@
         <v>8.24</v>
       </c>
       <c r="F25" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1343,6 +1561,12 @@
       <c r="M25" t="n">
         <v>6.63</v>
       </c>
+      <c r="N25" t="n">
+        <v>23.66</v>
+      </c>
+      <c r="O25" t="n">
+        <v>23.07</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1367,6 +1591,14 @@
         <v>-1.54</v>
       </c>
       <c r="F26" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>-8.77</v>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -1378,6 +1610,12 @@
       <c r="M26" t="n">
         <v>-8.52</v>
       </c>
+      <c r="N26" t="n">
+        <v>-10.01</v>
+      </c>
+      <c r="O26" t="n">
+        <v>-15.25</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1404,6 +1642,14 @@
       <c r="F27" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -1413,6 +1659,12 @@
       <c r="M27" t="n">
         <v>-5.88</v>
       </c>
+      <c r="N27" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="O27" t="n">
+        <v>2.26</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4338,7 +4590,21 @@
       <c r="D111" t="n">
         <v>250.54</v>
       </c>
+      <c r="E111" t="n">
+        <v>-4.88</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K111" t="inlineStr"/>
+      <c r="L111" t="n">
+        <v>-6.7</v>
+      </c>
+      <c r="M111" t="n">
+        <v>-2.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4499,7 +4765,21 @@
       <c r="D116" t="n">
         <v>547.4299999999999</v>
       </c>
+      <c r="E116" t="n">
+        <v>-6.57</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K116" t="inlineStr"/>
+      <c r="L116" t="n">
+        <v>-8.390000000000001</v>
+      </c>
+      <c r="M116" t="n">
+        <v>-7.2</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4520,7 +4800,21 @@
       <c r="D117" t="n">
         <v>190.28</v>
       </c>
+      <c r="E117" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K117" t="inlineStr"/>
+      <c r="L117" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="M117" t="n">
+        <v>2.02</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4541,7 +4835,21 @@
       <c r="D118" t="n">
         <v>191.58</v>
       </c>
+      <c r="E118" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K118" t="inlineStr"/>
+      <c r="L118" t="n">
+        <v>10.22</v>
+      </c>
+      <c r="M118" t="n">
+        <v>11.69</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4667,7 +4975,21 @@
       <c r="D122" t="n">
         <v>331.02</v>
       </c>
+      <c r="E122" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K122" t="inlineStr"/>
+      <c r="L122" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="M122" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4828,7 +5150,21 @@
       <c r="D127" t="n">
         <v>44.95</v>
       </c>
+      <c r="E127" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K127" t="inlineStr"/>
+      <c r="L127" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="M127" t="n">
+        <v>4.31</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4849,7 +5185,21 @@
       <c r="D128" t="n">
         <v>241.36</v>
       </c>
+      <c r="E128" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K128" t="inlineStr"/>
+      <c r="L128" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="M128" t="n">
+        <v>9.890000000000001</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4905,7 +5255,21 @@
       <c r="D130" t="n">
         <v>119.46</v>
       </c>
+      <c r="E130" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K130" t="inlineStr"/>
+      <c r="L130" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="M130" t="n">
+        <v>2.67</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4926,7 +5290,21 @@
       <c r="D131" t="n">
         <v>324.65</v>
       </c>
+      <c r="E131" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K131" t="inlineStr"/>
+      <c r="L131" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="M131" t="n">
+        <v>11.86</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5052,7 +5430,21 @@
       <c r="D135" t="n">
         <v>23.17</v>
       </c>
+      <c r="E135" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K135" t="inlineStr"/>
+      <c r="L135" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="M135" t="n">
+        <v>5.26</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5073,7 +5465,21 @@
       <c r="D136" t="n">
         <v>190.28</v>
       </c>
+      <c r="E136" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K136" t="inlineStr"/>
+      <c r="L136" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="M136" t="n">
+        <v>2.02</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5115,7 +5521,21 @@
       <c r="D138" t="n">
         <v>497.75</v>
       </c>
+      <c r="E138" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K138" t="inlineStr"/>
+      <c r="L138" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="M138" t="n">
+        <v>-0.18</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5136,7 +5556,21 @@
       <c r="D139" t="n">
         <v>138.47</v>
       </c>
+      <c r="E139" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K139" t="inlineStr"/>
+      <c r="L139" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="M139" t="n">
+        <v>-1.48</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5157,7 +5591,21 @@
       <c r="D140" t="n">
         <v>176.24</v>
       </c>
+      <c r="E140" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K140" t="inlineStr"/>
+      <c r="L140" t="n">
+        <v>8.68</v>
+      </c>
+      <c r="M140" t="n">
+        <v>8.609999999999999</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5178,7 +5626,21 @@
       <c r="D141" t="n">
         <v>52.94</v>
       </c>
+      <c r="E141" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K141" t="inlineStr"/>
+      <c r="L141" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="M141" t="n">
+        <v>-0.19</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5262,7 +5724,21 @@
       <c r="D145" t="n">
         <v>977.5</v>
       </c>
+      <c r="E145" t="n">
+        <v>10.34</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K145" t="inlineStr"/>
+      <c r="L145" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="M145" t="n">
+        <v>9.44</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5283,7 +5759,21 @@
       <c r="D146" t="n">
         <v>138.47</v>
       </c>
+      <c r="E146" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K146" t="inlineStr"/>
+      <c r="L146" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="M146" t="n">
+        <v>-1.48</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5304,7 +5794,21 @@
       <c r="D147" t="n">
         <v>1614.39</v>
       </c>
+      <c r="E147" t="n">
+        <v>8.65</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K147" t="inlineStr"/>
+      <c r="L147" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="M147" t="n">
+        <v>7.82</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5346,7 +5850,21 @@
       <c r="D149" t="n">
         <v>30.37</v>
       </c>
+      <c r="E149" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K149" t="inlineStr"/>
+      <c r="L149" t="n">
+        <v>-3.21</v>
+      </c>
+      <c r="M149" t="n">
+        <v>-3.9</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5367,7 +5885,21 @@
       <c r="D150" t="n">
         <v>38.06</v>
       </c>
+      <c r="E150" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K150" t="inlineStr"/>
+      <c r="L150" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="M150" t="n">
+        <v>-1.47</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5388,7 +5920,21 @@
       <c r="D151" t="n">
         <v>39.65</v>
       </c>
+      <c r="E151" t="n">
+        <v>-3.49</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K151" t="inlineStr"/>
+      <c r="L151" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="M151" t="n">
+        <v>-4.2</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5409,7 +5955,21 @@
       <c r="D152" t="n">
         <v>545.09</v>
       </c>
+      <c r="E152" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K152" t="inlineStr"/>
+      <c r="L152" t="n">
+        <v>14.79</v>
+      </c>
+      <c r="M152" t="n">
+        <v>14.82</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5430,7 +5990,21 @@
       <c r="D153" t="n">
         <v>280.76</v>
       </c>
+      <c r="E153" t="n">
+        <v>-5.07</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K153" t="inlineStr"/>
+      <c r="L153" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="M153" t="n">
+        <v>-6.36</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5493,7 +6067,21 @@
       <c r="D156" t="n">
         <v>588.4</v>
       </c>
+      <c r="E156" t="n">
+        <v>-8.890000000000001</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K156" t="inlineStr"/>
+      <c r="L156" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="M156" t="n">
+        <v>-9.720000000000001</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5535,7 +6123,21 @@
       <c r="D158" t="n">
         <v>38.06</v>
       </c>
+      <c r="E158" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K158" t="inlineStr"/>
+      <c r="L158" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="M158" t="n">
+        <v>-1.47</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5556,7 +6158,21 @@
       <c r="D159" t="n">
         <v>108.8</v>
       </c>
+      <c r="E159" t="n">
+        <v>17.06</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K159" t="inlineStr"/>
+      <c r="L159" t="n">
+        <v>16.45</v>
+      </c>
+      <c r="M159" t="n">
+        <v>15.89</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7594,6 +8210,447 @@
         <v>1071.43</v>
       </c>
       <c r="K256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>238.31</v>
+      </c>
+      <c r="K257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>777.4400000000001</v>
+      </c>
+      <c r="K258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>497.58</v>
+      </c>
+      <c r="K259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>137.78</v>
+      </c>
+      <c r="K260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>192.61</v>
+      </c>
+      <c r="K261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>194.25</v>
+      </c>
+      <c r="K262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>511.46</v>
+      </c>
+      <c r="K263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>214.64</v>
+      </c>
+      <c r="K264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>EWY</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>182.52</v>
+      </c>
+      <c r="K265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>154.1</v>
+      </c>
+      <c r="K266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>120.81</v>
+      </c>
+      <c r="K267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>1183.09</v>
+      </c>
+      <c r="K268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>224.54</v>
+      </c>
+      <c r="K269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>ALAB</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>360.63</v>
+      </c>
+      <c r="K270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>629.02</v>
+      </c>
+      <c r="K271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>306.43</v>
+      </c>
+      <c r="K272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="K273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>127.36</v>
+      </c>
+      <c r="K274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>777.4400000000001</v>
+      </c>
+      <c r="K275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>1078.62</v>
+      </c>
+      <c r="K276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>243.44</v>
+      </c>
+      <c r="K277" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7739,7 +8796,22 @@
         <v>-0.93</v>
       </c>
       <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="n">
         <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-3.35</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-3.29</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -7752,28 +8824,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C3" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D3" t="n">
-        <v>57.1</v>
+        <v>53.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.62</v>
+        <v>0.73</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="G3" t="n">
-        <v>42.9</v>
+        <v>39.5</v>
       </c>
       <c r="H3" t="n">
-        <v>0.38</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="J3" t="n">
+        <v>80</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="M3" t="n">
+        <v>60</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4.81</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -7786,28 +8873,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C4" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D4" t="n">
-        <v>75.90000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="E4" t="n">
-        <v>3.78</v>
+        <v>3.72</v>
       </c>
       <c r="F4" t="n">
-        <v>2.97</v>
+        <v>2.9</v>
       </c>
       <c r="G4" t="n">
-        <v>65.5</v>
+        <v>61.8</v>
       </c>
       <c r="H4" t="n">
-        <v>3.77</v>
+        <v>3.56</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="J4" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="K4" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="M4" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2.32</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -7823,22 +8925,22 @@
         <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E5" t="n">
-        <v>8.02</v>
+        <v>6.3</v>
       </c>
       <c r="F5" t="n">
-        <v>6.53</v>
+        <v>4.99</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="H5" t="n">
-        <v>7.85</v>
+        <v>5.72</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -7854,28 +8956,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C6" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E6" t="n">
-        <v>3.72</v>
+        <v>3.71</v>
       </c>
       <c r="F6" t="n">
-        <v>2.21</v>
+        <v>2.24</v>
       </c>
       <c r="G6" t="n">
-        <v>68</v>
+        <v>68.8</v>
       </c>
       <c r="H6" t="n">
-        <v>4.31</v>
+        <v>4.22</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="J6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="L6" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="M6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.48</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -7888,28 +9005,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C7" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D7" t="n">
-        <v>55</v>
+        <v>62.5</v>
       </c>
       <c r="E7" t="n">
-        <v>0.05</v>
+        <v>1.04</v>
       </c>
       <c r="F7" t="n">
-        <v>-1.29</v>
+        <v>-0.27</v>
       </c>
       <c r="G7" t="n">
-        <v>35</v>
+        <v>41.7</v>
       </c>
       <c r="H7" t="n">
-        <v>1.3</v>
+        <v>1.99</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="L7" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="M7" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3.36</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-09-25
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q277"/>
+  <dimension ref="A1:Q296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,6 +629,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G4" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>1.99</v>
@@ -636,6 +644,12 @@
       <c r="M4" t="n">
         <v>1.94</v>
       </c>
+      <c r="N4" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="O4" t="n">
+        <v>4.76</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -909,6 +923,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G10" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>0.73</v>
@@ -916,6 +938,12 @@
       <c r="M10" t="n">
         <v>0.15</v>
       </c>
+      <c r="N10" t="n">
+        <v>-3.55</v>
+      </c>
+      <c r="O10" t="n">
+        <v>-3.48</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -940,6 +968,14 @@
         <v>7.22</v>
       </c>
       <c r="F11" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -951,6 +987,12 @@
       <c r="M11" t="n">
         <v>7.69</v>
       </c>
+      <c r="N11" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="O11" t="n">
+        <v>4.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -975,6 +1017,14 @@
         <v>11.49</v>
       </c>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -986,6 +1036,12 @@
       <c r="M12" t="n">
         <v>10.82</v>
       </c>
+      <c r="N12" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="O12" t="n">
+        <v>9.27</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1010,6 +1066,14 @@
         <v>17.64</v>
       </c>
       <c r="F13" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>20.72</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1021,6 +1085,12 @@
       <c r="M13" t="n">
         <v>18.01</v>
       </c>
+      <c r="N13" t="n">
+        <v>19.48</v>
+      </c>
+      <c r="O13" t="n">
+        <v>21.1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1196,6 +1266,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G17" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>6.69</v>
@@ -1203,6 +1281,12 @@
       <c r="M17" t="n">
         <v>6.65</v>
       </c>
+      <c r="N17" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="O17" t="n">
+        <v>11.44</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1329,6 +1413,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G20" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
         <v>0.73</v>
@@ -1336,6 +1428,12 @@
       <c r="M20" t="n">
         <v>0.15</v>
       </c>
+      <c r="N20" t="n">
+        <v>-3.55</v>
+      </c>
+      <c r="O20" t="n">
+        <v>-3.48</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1360,6 +1458,14 @@
         <v>7.22</v>
       </c>
       <c r="F21" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1371,6 +1477,12 @@
       <c r="M21" t="n">
         <v>7.69</v>
       </c>
+      <c r="N21" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="O21" t="n">
+        <v>4.99</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1693,6 +1805,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G28" t="n">
+        <v>-2.41</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>-1.32</v>
@@ -1700,6 +1820,12 @@
       <c r="M28" t="n">
         <v>-1.28</v>
       </c>
+      <c r="N28" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="O28" t="n">
+        <v>-2.03</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1763,6 +1889,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G30" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>3.13</v>
@@ -1770,6 +1904,12 @@
       <c r="M30" t="n">
         <v>0.65</v>
       </c>
+      <c r="N30" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="O30" t="n">
+        <v>2.23</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1796,6 +1936,14 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -1805,6 +1953,12 @@
       <c r="M31" t="n">
         <v>-0.76</v>
       </c>
+      <c r="N31" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="O31" t="n">
+        <v>3.73</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1829,6 +1983,14 @@
         <v>2.22</v>
       </c>
       <c r="F32" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1840,6 +2002,12 @@
       <c r="M32" t="n">
         <v>-3.34</v>
       </c>
+      <c r="N32" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="O32" t="n">
+        <v>-3.22</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1864,6 +2032,14 @@
         <v>6.22</v>
       </c>
       <c r="F33" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1875,6 +2051,12 @@
       <c r="M33" t="n">
         <v>4.58</v>
       </c>
+      <c r="N33" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="O33" t="n">
+        <v>11.67</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1901,6 +2083,14 @@
       <c r="F34" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -1910,6 +2100,12 @@
       <c r="M34" t="n">
         <v>-3.69</v>
       </c>
+      <c r="N34" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1.15</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2043,6 +2239,14 @@
           <t>FLAT</t>
         </is>
       </c>
+      <c r="G38" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
         <v>0.76</v>
@@ -2050,6 +2254,12 @@
       <c r="M38" t="n">
         <v>8.039999999999999</v>
       </c>
+      <c r="N38" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="O38" t="n">
+        <v>9.279999999999999</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2074,6 +2284,14 @@
         <v>3.45</v>
       </c>
       <c r="F39" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2085,6 +2303,12 @@
       <c r="M39" t="n">
         <v>13.08</v>
       </c>
+      <c r="N39" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="O39" t="n">
+        <v>21.25</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2111,6 +2335,14 @@
       <c r="F40" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K40" t="inlineStr"/>
@@ -2120,6 +2352,12 @@
       <c r="M40" t="n">
         <v>-0.76</v>
       </c>
+      <c r="N40" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="O40" t="n">
+        <v>3.73</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2144,6 +2382,14 @@
         <v>6.22</v>
       </c>
       <c r="F41" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2155,6 +2401,12 @@
       <c r="M41" t="n">
         <v>4.58</v>
       </c>
+      <c r="N41" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="O41" t="n">
+        <v>11.67</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2179,6 +2431,14 @@
         <v>9.699999999999999</v>
       </c>
       <c r="F42" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2190,6 +2450,12 @@
       <c r="M42" t="n">
         <v>17.66</v>
       </c>
+      <c r="N42" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="O42" t="n">
+        <v>16.73</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2253,6 +2519,14 @@
           <t>FLAT</t>
         </is>
       </c>
+      <c r="G44" t="n">
+        <v>-2.39</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="n">
         <v>0.51</v>
@@ -2260,6 +2534,12 @@
       <c r="M44" t="n">
         <v>-1.21</v>
       </c>
+      <c r="N44" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="O44" t="n">
+        <v>-3.73</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2286,6 +2566,14 @@
       <c r="F45" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -2295,6 +2583,12 @@
       <c r="M45" t="n">
         <v>5.38</v>
       </c>
+      <c r="N45" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="O45" t="n">
+        <v>4.42</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2319,6 +2613,14 @@
         <v>8.460000000000001</v>
       </c>
       <c r="F46" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>22.13</v>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2330,6 +2632,12 @@
       <c r="M46" t="n">
         <v>15.02</v>
       </c>
+      <c r="N46" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="O46" t="n">
+        <v>29.53</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2356,6 +2664,14 @@
       <c r="F47" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
@@ -2365,6 +2681,12 @@
       <c r="M47" t="n">
         <v>5.38</v>
       </c>
+      <c r="N47" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="O47" t="n">
+        <v>4.42</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2389,6 +2711,14 @@
         <v>-3.93</v>
       </c>
       <c r="F48" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -2400,6 +2730,12 @@
       <c r="M48" t="n">
         <v>1.47</v>
       </c>
+      <c r="N48" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="O48" t="n">
+        <v>4.75</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2424,6 +2760,14 @@
         <v>-9.779999999999999</v>
       </c>
       <c r="F49" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -2435,6 +2779,12 @@
       <c r="M49" t="n">
         <v>-0.45</v>
       </c>
+      <c r="N49" t="n">
+        <v>-6.75</v>
+      </c>
+      <c r="O49" t="n">
+        <v>3.92</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2461,6 +2811,14 @@
       <c r="F50" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
@@ -2470,6 +2828,12 @@
       <c r="M50" t="n">
         <v>8.039999999999999</v>
       </c>
+      <c r="N50" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="O50" t="n">
+        <v>9.279999999999999</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2494,6 +2858,14 @@
         <v>-4.04</v>
       </c>
       <c r="F51" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>-6.78</v>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -2505,6 +2877,12 @@
       <c r="M51" t="n">
         <v>6.27</v>
       </c>
+      <c r="N51" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="O51" t="n">
+        <v>3.24</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5500,7 +5878,21 @@
       <c r="D137" t="n">
         <v>242.85</v>
       </c>
+      <c r="E137" t="n">
+        <v>-3.61</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K137" t="inlineStr"/>
+      <c r="L137" t="n">
+        <v>-4.22</v>
+      </c>
+      <c r="M137" t="n">
+        <v>-4.27</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5661,7 +6053,21 @@
       <c r="D142" t="n">
         <v>528.84</v>
       </c>
+      <c r="E142" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K142" t="inlineStr"/>
+      <c r="L142" t="n">
+        <v>-4.23</v>
+      </c>
+      <c r="M142" t="n">
+        <v>-3.47</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5682,7 +6088,21 @@
       <c r="D143" t="n">
         <v>192.53</v>
       </c>
+      <c r="E143" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K143" t="inlineStr"/>
+      <c r="L143" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="M143" t="n">
+        <v>-3.08</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5703,7 +6123,21 @@
       <c r="D144" t="n">
         <v>197.47</v>
       </c>
+      <c r="E144" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K144" t="inlineStr"/>
+      <c r="L144" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="M144" t="n">
+        <v>-3.1</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5829,7 +6263,21 @@
       <c r="D148" t="n">
         <v>192.53</v>
       </c>
+      <c r="E148" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K148" t="inlineStr"/>
+      <c r="L148" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="M148" t="n">
+        <v>-3.08</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6025,7 +6473,21 @@
       <c r="D154" t="n">
         <v>45.32</v>
       </c>
+      <c r="E154" t="n">
+        <v>-1.39</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K154" t="inlineStr"/>
+      <c r="L154" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M154" t="n">
+        <v>-2.2</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6046,7 +6508,21 @@
       <c r="D155" t="n">
         <v>245.7</v>
       </c>
+      <c r="E155" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K155" t="inlineStr"/>
+      <c r="L155" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="M155" t="n">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6102,7 +6578,21 @@
       <c r="D157" t="n">
         <v>120.48</v>
       </c>
+      <c r="E157" t="n">
+        <v>-2.12</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K157" t="inlineStr"/>
+      <c r="L157" t="n">
+        <v>-2.73</v>
+      </c>
+      <c r="M157" t="n">
+        <v>-2.67</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6193,7 +6683,21 @@
       <c r="D160" t="n">
         <v>333.94</v>
       </c>
+      <c r="E160" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K160" t="inlineStr"/>
+      <c r="L160" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="M160" t="n">
+        <v>3.12</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6214,7 +6718,21 @@
       <c r="D161" t="n">
         <v>23.19</v>
       </c>
+      <c r="E161" t="n">
+        <v>-3.51</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K161" t="inlineStr"/>
+      <c r="L161" t="n">
+        <v>-4.12</v>
+      </c>
+      <c r="M161" t="n">
+        <v>-3.36</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6235,7 +6753,21 @@
       <c r="D162" t="n">
         <v>192.53</v>
       </c>
+      <c r="E162" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K162" t="inlineStr"/>
+      <c r="L162" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="M162" t="n">
+        <v>-3.08</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6277,7 +6809,21 @@
       <c r="D164" t="n">
         <v>493.78</v>
       </c>
+      <c r="E164" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K164" t="inlineStr"/>
+      <c r="L164" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="M164" t="n">
+        <v>4.17</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6298,7 +6844,21 @@
       <c r="D165" t="n">
         <v>135.47</v>
       </c>
+      <c r="E165" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K165" t="inlineStr"/>
+      <c r="L165" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="M165" t="n">
+        <v>-0.97</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6319,7 +6879,21 @@
       <c r="D166" t="n">
         <v>177.64</v>
       </c>
+      <c r="E166" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K166" t="inlineStr"/>
+      <c r="L166" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="M166" t="n">
+        <v>6.02</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6403,7 +6977,21 @@
       <c r="D170" t="n">
         <v>223.54</v>
       </c>
+      <c r="E170" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K170" t="inlineStr"/>
+      <c r="L170" t="n">
+        <v>4.96</v>
+      </c>
+      <c r="M170" t="n">
+        <v>4.98</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -6424,7 +7012,21 @@
       <c r="D171" t="n">
         <v>444.57</v>
       </c>
+      <c r="E171" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K171" t="inlineStr"/>
+      <c r="L171" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="M171" t="n">
+        <v>6.28</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6445,7 +7047,21 @@
       <c r="D172" t="n">
         <v>194.25</v>
       </c>
+      <c r="E172" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K172" t="inlineStr"/>
+      <c r="L172" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="M172" t="n">
+        <v>-5.01</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -6466,7 +7082,21 @@
       <c r="D173" t="n">
         <v>91.78</v>
       </c>
+      <c r="E173" t="n">
+        <v>-3.07</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K173" t="inlineStr"/>
+      <c r="L173" t="n">
+        <v>-4.33</v>
+      </c>
+      <c r="M173" t="n">
+        <v>-9.41</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -6529,7 +7159,21 @@
       <c r="D176" t="n">
         <v>336.13</v>
       </c>
+      <c r="E176" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K176" t="inlineStr"/>
+      <c r="L176" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M176" t="n">
+        <v>1.62</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6550,7 +7194,21 @@
       <c r="D177" t="n">
         <v>559.8200000000001</v>
       </c>
+      <c r="E177" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K177" t="inlineStr"/>
+      <c r="L177" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="M177" t="n">
+        <v>7.86</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6571,7 +7229,21 @@
       <c r="D178" t="n">
         <v>275.61</v>
       </c>
+      <c r="E178" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K178" t="inlineStr"/>
+      <c r="L178" t="n">
+        <v>11.42</v>
+      </c>
+      <c r="M178" t="n">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6592,7 +7264,21 @@
       <c r="D179" t="n">
         <v>265.63</v>
       </c>
+      <c r="E179" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K179" t="inlineStr"/>
+      <c r="L179" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="M179" t="n">
+        <v>6.78</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6613,7 +7299,21 @@
       <c r="D180" t="n">
         <v>194.25</v>
       </c>
+      <c r="E180" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K180" t="inlineStr"/>
+      <c r="L180" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="M180" t="n">
+        <v>-5.01</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6676,7 +7376,21 @@
       <c r="D183" t="n">
         <v>18.34</v>
       </c>
+      <c r="E183" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K183" t="inlineStr"/>
+      <c r="L183" t="n">
+        <v>-4.59</v>
+      </c>
+      <c r="M183" t="n">
+        <v>-5.11</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -6697,7 +7411,21 @@
       <c r="D184" t="n">
         <v>317.36</v>
       </c>
+      <c r="E184" t="n">
+        <v>-6.8</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K184" t="inlineStr"/>
+      <c r="L184" t="n">
+        <v>-8.06</v>
+      </c>
+      <c r="M184" t="n">
+        <v>-9.5</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6718,7 +7446,21 @@
       <c r="D185" t="n">
         <v>39.44</v>
       </c>
+      <c r="E185" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K185" t="inlineStr"/>
+      <c r="L185" t="n">
+        <v>-2.48</v>
+      </c>
+      <c r="M185" t="n">
+        <v>-2.77</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6760,7 +7502,21 @@
       <c r="D187" t="n">
         <v>119.82</v>
       </c>
+      <c r="E187" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K187" t="inlineStr"/>
+      <c r="L187" t="n">
+        <v>-1.56</v>
+      </c>
+      <c r="M187" t="n">
+        <v>-4.57</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6781,7 +7537,21 @@
       <c r="D188" t="n">
         <v>1015.8</v>
       </c>
+      <c r="E188" t="n">
+        <v>6.49</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K188" t="inlineStr"/>
+      <c r="L188" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="M188" t="n">
+        <v>3.41</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6823,7 +7593,21 @@
       <c r="D190" t="n">
         <v>177.72</v>
       </c>
+      <c r="E190" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K190" t="inlineStr"/>
+      <c r="L190" t="n">
+        <v>12.37</v>
+      </c>
+      <c r="M190" t="n">
+        <v>11.72</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6844,7 +7628,21 @@
       <c r="D191" t="n">
         <v>152.71</v>
       </c>
+      <c r="E191" t="n">
+        <v>-2.61</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K191" t="inlineStr"/>
+      <c r="L191" t="n">
+        <v>-3.87</v>
+      </c>
+      <c r="M191" t="n">
+        <v>-4</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8651,6 +9449,405 @@
         <v>243.44</v>
       </c>
       <c r="K277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>234.07</v>
+      </c>
+      <c r="K278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>751.9</v>
+      </c>
+      <c r="K279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>516.1</v>
+      </c>
+      <c r="K280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>135.63</v>
+      </c>
+      <c r="K281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>189.66</v>
+      </c>
+      <c r="K282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>201.95</v>
+      </c>
+      <c r="K283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>509.68</v>
+      </c>
+      <c r="K284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>193.03</v>
+      </c>
+      <c r="K285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>156.7</v>
+      </c>
+      <c r="K286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>119.46</v>
+      </c>
+      <c r="K287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>IGV</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>105.98</v>
+      </c>
+      <c r="K288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>237.44</v>
+      </c>
+      <c r="K289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>135.63</v>
+      </c>
+      <c r="K290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>225.08</v>
+      </c>
+      <c r="K291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>ALAB</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>364.46</v>
+      </c>
+      <c r="K292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>310.55</v>
+      </c>
+      <c r="K293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>288.58</v>
+      </c>
+      <c r="K294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>516.1</v>
+      </c>
+      <c r="K295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>1081.69</v>
+      </c>
+      <c r="K296" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8796,22 +9993,22 @@
         <v>-0.93</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="K2" t="n">
-        <v>-2.12</v>
+        <v>-0.3</v>
       </c>
       <c r="L2" t="n">
-        <v>-3.35</v>
+        <v>-1.46</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="N2" t="n">
-        <v>-3.29</v>
+        <v>-0.96</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -8824,43 +10021,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C3" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>53.5</v>
+        <v>52</v>
       </c>
       <c r="E3" t="n">
-        <v>0.73</v>
+        <v>0.62</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.4</v>
+        <v>-0.48</v>
       </c>
       <c r="G3" t="n">
-        <v>39.5</v>
+        <v>38</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.39</v>
       </c>
       <c r="I3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J3" t="n">
-        <v>80</v>
+        <v>83.3</v>
       </c>
       <c r="K3" t="n">
-        <v>5.38</v>
+        <v>4.66</v>
       </c>
       <c r="L3" t="n">
-        <v>4.14</v>
+        <v>3.55</v>
       </c>
       <c r="M3" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="N3" t="n">
-        <v>4.81</v>
+        <v>3.43</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -8873,43 +10070,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C4" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" t="n">
-        <v>73.5</v>
+        <v>72.2</v>
       </c>
       <c r="E4" t="n">
-        <v>3.72</v>
+        <v>3.61</v>
       </c>
       <c r="F4" t="n">
-        <v>2.9</v>
+        <v>2.79</v>
       </c>
       <c r="G4" t="n">
-        <v>61.8</v>
+        <v>61.1</v>
       </c>
       <c r="H4" t="n">
-        <v>3.56</v>
+        <v>3.42</v>
       </c>
       <c r="I4" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="J4" t="n">
-        <v>66.7</v>
+        <v>76.5</v>
       </c>
       <c r="K4" t="n">
-        <v>3.53</v>
+        <v>6.04</v>
       </c>
       <c r="L4" t="n">
-        <v>2.29</v>
+        <v>4.91</v>
       </c>
       <c r="M4" t="n">
-        <v>50</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>2.32</v>
+        <v>6.83</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -8925,25 +10122,40 @@
         <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>90</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>6.3</v>
+        <v>5.34</v>
       </c>
       <c r="F5" t="n">
-        <v>4.99</v>
+        <v>4.05</v>
       </c>
       <c r="G5" t="n">
-        <v>90</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>5.72</v>
+        <v>3.77</v>
       </c>
       <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
         <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>4.42</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -8956,43 +10168,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D6" t="n">
         <v>75</v>
       </c>
       <c r="E6" t="n">
-        <v>3.71</v>
+        <v>3.84</v>
       </c>
       <c r="F6" t="n">
-        <v>2.24</v>
+        <v>2.46</v>
       </c>
       <c r="G6" t="n">
-        <v>68.8</v>
+        <v>67.5</v>
       </c>
       <c r="H6" t="n">
-        <v>4.22</v>
+        <v>3.72</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>4.72</v>
+        <v>6</v>
       </c>
       <c r="L6" t="n">
-        <v>3.49</v>
+        <v>4.95</v>
       </c>
       <c r="M6" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="N6" t="n">
-        <v>4.48</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -9005,43 +10217,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C7" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D7" t="n">
-        <v>62.5</v>
+        <v>52.9</v>
       </c>
       <c r="E7" t="n">
-        <v>1.04</v>
+        <v>0.86</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.27</v>
+        <v>-0.38</v>
       </c>
       <c r="G7" t="n">
-        <v>41.7</v>
+        <v>38.2</v>
       </c>
       <c r="H7" t="n">
-        <v>1.99</v>
+        <v>0.99</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J7" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="K7" t="n">
-        <v>6.59</v>
+        <v>1.45</v>
       </c>
       <c r="L7" t="n">
-        <v>5.35</v>
+        <v>0.38</v>
       </c>
       <c r="M7" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="N7" t="n">
-        <v>3.36</v>
+        <v>4.42</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-09-29
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q347"/>
+  <dimension ref="A1:Q381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4598,6 +4598,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G85" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="n">
         <v>0.53</v>
@@ -4605,6 +4613,12 @@
       <c r="M85" t="n">
         <v>2.67</v>
       </c>
+      <c r="N85" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="O85" t="n">
+        <v>-0.67</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4629,6 +4643,14 @@
         <v>-8.75</v>
       </c>
       <c r="F86" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>-11.83</v>
+      </c>
+      <c r="H86" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -4640,6 +4662,12 @@
       <c r="M86" t="n">
         <v>-7.47</v>
       </c>
+      <c r="N86" t="n">
+        <v>-12.74</v>
+      </c>
+      <c r="O86" t="n">
+        <v>-10.6</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4666,6 +4694,14 @@
       <c r="F87" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K87" t="inlineStr"/>
@@ -4675,6 +4711,12 @@
       <c r="M87" t="n">
         <v>2.18</v>
       </c>
+      <c r="N87" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0.73</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4701,6 +4743,14 @@
       <c r="F88" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K88" t="inlineStr"/>
@@ -4710,6 +4760,12 @@
       <c r="M88" t="n">
         <v>0.91</v>
       </c>
+      <c r="N88" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="O88" t="n">
+        <v>3.15</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4734,6 +4790,14 @@
         <v>-3.45</v>
       </c>
       <c r="F89" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>-8.390000000000001</v>
+      </c>
+      <c r="H89" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -4745,6 +4809,12 @@
       <c r="M89" t="n">
         <v>-1.68</v>
       </c>
+      <c r="N89" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="O89" t="n">
+        <v>-6.72</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4769,6 +4839,14 @@
         <v>1.38</v>
       </c>
       <c r="F90" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="H90" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -4780,6 +4858,12 @@
       <c r="M90" t="n">
         <v>0.95</v>
       </c>
+      <c r="N90" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="O90" t="n">
+        <v>3.83</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4804,6 +4888,14 @@
         <v>7.2</v>
       </c>
       <c r="F91" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="H91" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -4815,6 +4907,12 @@
       <c r="M91" t="n">
         <v>8.470000000000001</v>
       </c>
+      <c r="N91" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="O91" t="n">
+        <v>9.630000000000001</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4841,6 +4939,14 @@
       <c r="F92" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K92" t="inlineStr"/>
@@ -4850,6 +4956,12 @@
       <c r="M92" t="n">
         <v>-1.48</v>
       </c>
+      <c r="N92" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4874,6 +4986,14 @@
         <v>-10.2</v>
       </c>
       <c r="F93" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>-11.6</v>
+      </c>
+      <c r="H93" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -4885,6 +5005,12 @@
       <c r="M93" t="n">
         <v>-10.57</v>
       </c>
+      <c r="N93" t="n">
+        <v>-12.51</v>
+      </c>
+      <c r="O93" t="n">
+        <v>-11.96</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4909,6 +5035,14 @@
         <v>-0.61</v>
       </c>
       <c r="F94" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="H94" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -4920,6 +5054,12 @@
       <c r="M94" t="n">
         <v>1.6</v>
       </c>
+      <c r="N94" t="n">
+        <v>-8.210000000000001</v>
+      </c>
+      <c r="O94" t="n">
+        <v>-5.24</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4946,6 +5086,14 @@
       <c r="F95" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K95" t="inlineStr"/>
@@ -4955,6 +5103,12 @@
       <c r="M95" t="n">
         <v>2.18</v>
       </c>
+      <c r="N95" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.73</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4979,6 +5133,14 @@
         <v>18.34</v>
       </c>
       <c r="F96" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>18.76</v>
+      </c>
+      <c r="H96" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -4990,6 +5152,12 @@
       <c r="M96" t="n">
         <v>15.61</v>
       </c>
+      <c r="N96" t="n">
+        <v>17.84</v>
+      </c>
+      <c r="O96" t="n">
+        <v>16.02</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5016,6 +5184,14 @@
       <c r="F97" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K97" t="inlineStr"/>
@@ -5025,6 +5201,12 @@
       <c r="M97" t="n">
         <v>0.91</v>
       </c>
+      <c r="N97" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="O97" t="n">
+        <v>3.15</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5049,6 +5231,14 @@
         <v>7.2</v>
       </c>
       <c r="F98" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="H98" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -5060,6 +5250,12 @@
       <c r="M98" t="n">
         <v>8.470000000000001</v>
       </c>
+      <c r="N98" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="O98" t="n">
+        <v>9.630000000000001</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5084,6 +5280,14 @@
         <v>-10.2</v>
       </c>
       <c r="F99" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>-11.6</v>
+      </c>
+      <c r="H99" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -5095,6 +5299,12 @@
       <c r="M99" t="n">
         <v>-10.57</v>
       </c>
+      <c r="N99" t="n">
+        <v>-12.51</v>
+      </c>
+      <c r="O99" t="n">
+        <v>-11.96</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5119,6 +5329,14 @@
         <v>22.83</v>
       </c>
       <c r="F100" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>18.56</v>
+      </c>
+      <c r="H100" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -5130,6 +5348,12 @@
       <c r="M100" t="n">
         <v>16.13</v>
       </c>
+      <c r="N100" t="n">
+        <v>17.65</v>
+      </c>
+      <c r="O100" t="n">
+        <v>12.09</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5156,6 +5380,14 @@
       <c r="F101" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K101" t="inlineStr"/>
@@ -5165,6 +5397,12 @@
       <c r="M101" t="n">
         <v>2.07</v>
       </c>
+      <c r="N101" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="O101" t="n">
+        <v>-0.98</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5189,6 +5427,14 @@
         <v>-0.82</v>
       </c>
       <c r="F102" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>-7.78</v>
+      </c>
+      <c r="H102" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -5200,6 +5446,12 @@
       <c r="M102" t="n">
         <v>-1.55</v>
       </c>
+      <c r="N102" t="n">
+        <v>-8.69</v>
+      </c>
+      <c r="O102" t="n">
+        <v>-8.470000000000001</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5226,6 +5478,14 @@
       <c r="F103" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K103" t="inlineStr"/>
@@ -5235,6 +5495,12 @@
       <c r="M103" t="n">
         <v>3.28</v>
       </c>
+      <c r="N103" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="O103" t="n">
+        <v>1.61</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5259,6 +5525,14 @@
         <v>3.12</v>
       </c>
       <c r="F104" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="H104" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -5270,6 +5544,12 @@
       <c r="M104" t="n">
         <v>5.45</v>
       </c>
+      <c r="N104" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="O104" t="n">
+        <v>10.8</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5296,6 +5576,14 @@
       <c r="F105" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K105" t="inlineStr"/>
@@ -5305,6 +5593,12 @@
       <c r="M105" t="n">
         <v>-0.95</v>
       </c>
+      <c r="N105" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="O105" t="n">
+        <v>-2.62</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5331,6 +5625,14 @@
       <c r="F106" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K106" t="inlineStr"/>
@@ -5340,6 +5642,12 @@
       <c r="M106" t="n">
         <v>2.08</v>
       </c>
+      <c r="N106" t="n">
+        <v>-1.68</v>
+      </c>
+      <c r="O106" t="n">
+        <v>0.13</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5364,6 +5672,14 @@
         <v>-6.84</v>
       </c>
       <c r="F107" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>-11.41</v>
+      </c>
+      <c r="H107" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -5375,6 +5691,12 @@
       <c r="M107" t="n">
         <v>-3.89</v>
       </c>
+      <c r="N107" t="n">
+        <v>-12.32</v>
+      </c>
+      <c r="O107" t="n">
+        <v>-8.609999999999999</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5399,6 +5721,14 @@
         <v>7.88</v>
       </c>
       <c r="F108" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="H108" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -5410,6 +5740,12 @@
       <c r="M108" t="n">
         <v>8.84</v>
       </c>
+      <c r="N108" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="O108" t="n">
+        <v>8.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5436,6 +5772,14 @@
       <c r="F109" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K109" t="inlineStr"/>
@@ -5445,6 +5789,12 @@
       <c r="M109" t="n">
         <v>2.18</v>
       </c>
+      <c r="N109" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0.73</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5469,6 +5819,14 @@
         <v>-3.45</v>
       </c>
       <c r="F110" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>-8.390000000000001</v>
+      </c>
+      <c r="H110" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -5480,6 +5838,12 @@
       <c r="M110" t="n">
         <v>-1.68</v>
       </c>
+      <c r="N110" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="O110" t="n">
+        <v>-6.72</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5506,6 +5870,14 @@
       <c r="F111" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K111" t="inlineStr"/>
@@ -5515,6 +5887,12 @@
       <c r="M111" t="n">
         <v>3.42</v>
       </c>
+      <c r="N111" t="n">
+        <v>-1.57</v>
+      </c>
+      <c r="O111" t="n">
+        <v>1.14</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5539,6 +5917,14 @@
         <v>-0.61</v>
       </c>
       <c r="F112" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="H112" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -5550,6 +5936,12 @@
       <c r="M112" t="n">
         <v>1.6</v>
       </c>
+      <c r="N112" t="n">
+        <v>-8.210000000000001</v>
+      </c>
+      <c r="O112" t="n">
+        <v>-5.24</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9735,7 +10127,21 @@
       <c r="D232" t="n">
         <v>340</v>
       </c>
+      <c r="E232" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K232" t="inlineStr"/>
+      <c r="L232" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="M232" t="n">
+        <v>-0.87</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -9756,7 +10162,21 @@
       <c r="D233" t="n">
         <v>233.28</v>
       </c>
+      <c r="E233" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K233" t="inlineStr"/>
+      <c r="L233" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="M233" t="n">
+        <v>-3.94</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -9777,7 +10197,21 @@
       <c r="D234" t="n">
         <v>498</v>
       </c>
+      <c r="E234" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K234" t="inlineStr"/>
+      <c r="L234" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="M234" t="n">
+        <v>1.55</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -9798,7 +10232,21 @@
       <c r="D235" t="n">
         <v>137</v>
       </c>
+      <c r="E235" t="n">
+        <v>-5.12</v>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K235" t="inlineStr"/>
+      <c r="L235" t="n">
+        <v>-3.94</v>
+      </c>
+      <c r="M235" t="n">
+        <v>-5.37</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -9819,7 +10267,21 @@
       <c r="D236" t="n">
         <v>27.93</v>
       </c>
+      <c r="E236" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K236" t="inlineStr"/>
+      <c r="L236" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="M236" t="n">
+        <v>2.64</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -9840,7 +10302,21 @@
       <c r="D237" t="n">
         <v>184.99</v>
       </c>
+      <c r="E237" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K237" t="inlineStr"/>
+      <c r="L237" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="M237" t="n">
+        <v>0.27</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -9861,7 +10337,21 @@
       <c r="D238" t="n">
         <v>198.27</v>
       </c>
+      <c r="E238" t="n">
+        <v>-7.1</v>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K238" t="inlineStr"/>
+      <c r="L238" t="n">
+        <v>-5.93</v>
+      </c>
+      <c r="M238" t="n">
+        <v>-7.83</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -9882,7 +10372,21 @@
       <c r="D239" t="n">
         <v>501.3</v>
       </c>
+      <c r="E239" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K239" t="inlineStr"/>
+      <c r="L239" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="M239" t="n">
+        <v>-1.64</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -9903,7 +10407,21 @@
       <c r="D240" t="n">
         <v>188.65</v>
       </c>
+      <c r="E240" t="n">
+        <v>-6.73</v>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K240" t="inlineStr"/>
+      <c r="L240" t="n">
+        <v>-5.55</v>
+      </c>
+      <c r="M240" t="n">
+        <v>-7.5</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -9924,7 +10442,21 @@
       <c r="D241" t="n">
         <v>210.18</v>
       </c>
+      <c r="E241" t="n">
+        <v>-5.61</v>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K241" t="inlineStr"/>
+      <c r="L241" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="M241" t="n">
+        <v>-6.96</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -9945,7 +10477,21 @@
       <c r="D242" t="n">
         <v>159.69</v>
       </c>
+      <c r="E242" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K242" t="inlineStr"/>
+      <c r="L242" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="M242" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -9966,7 +10512,21 @@
       <c r="D243" t="n">
         <v>106.75</v>
       </c>
+      <c r="E243" t="n">
+        <v>-1.41</v>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K243" t="inlineStr"/>
+      <c r="L243" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="M243" t="n">
+        <v>-1.8</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -9987,7 +10547,21 @@
       <c r="D244" t="n">
         <v>363.46</v>
       </c>
+      <c r="E244" t="n">
+        <v>-1.57</v>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K244" t="inlineStr"/>
+      <c r="L244" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="M244" t="n">
+        <v>-1.9</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -10008,7 +10582,21 @@
       <c r="D245" t="n">
         <v>623.77</v>
       </c>
+      <c r="E245" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K245" t="inlineStr"/>
+      <c r="L245" t="n">
+        <v>-1.39</v>
+      </c>
+      <c r="M245" t="n">
+        <v>-2.31</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -10029,7 +10617,21 @@
       <c r="D246" t="n">
         <v>333.2</v>
       </c>
+      <c r="E246" t="n">
+        <v>-11.86</v>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K246" t="inlineStr"/>
+      <c r="L246" t="n">
+        <v>-10.69</v>
+      </c>
+      <c r="M246" t="n">
+        <v>-11.59</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -10050,7 +10652,21 @@
       <c r="D247" t="n">
         <v>8.619999999999999</v>
       </c>
+      <c r="E247" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K247" t="inlineStr"/>
+      <c r="L247" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="M247" t="n">
+        <v>1.3</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -10071,7 +10687,21 @@
       <c r="D248" t="n">
         <v>123.86</v>
       </c>
+      <c r="E248" t="n">
+        <v>-6.36</v>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K248" t="inlineStr"/>
+      <c r="L248" t="n">
+        <v>-5.19</v>
+      </c>
+      <c r="M248" t="n">
+        <v>-6.47</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -10092,7 +10722,21 @@
       <c r="D249" t="n">
         <v>310.39</v>
       </c>
+      <c r="E249" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K249" t="inlineStr"/>
+      <c r="L249" t="n">
+        <v>-4.65</v>
+      </c>
+      <c r="M249" t="n">
+        <v>-6.45</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -10113,7 +10757,21 @@
       <c r="D250" t="n">
         <v>945.67</v>
       </c>
+      <c r="E250" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K250" t="inlineStr"/>
+      <c r="L250" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="M250" t="n">
+        <v>2.69</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -10134,7 +10792,21 @@
       <c r="D251" t="n">
         <v>182.56</v>
       </c>
+      <c r="E251" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K251" t="inlineStr"/>
+      <c r="L251" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="M251" t="n">
+        <v>10.79</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -12151,6 +12823,720 @@
         <v>40.89</v>
       </c>
       <c r="K347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>233.18</v>
+      </c>
+      <c r="K348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>225.41</v>
+      </c>
+      <c r="K349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>739.02</v>
+      </c>
+      <c r="K350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>129.99</v>
+      </c>
+      <c r="K351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>28.73</v>
+      </c>
+      <c r="K352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>186.97</v>
+      </c>
+      <c r="K353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>184.19</v>
+      </c>
+      <c r="K354" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>493.52</v>
+      </c>
+      <c r="K355" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>198.39</v>
+      </c>
+      <c r="K356" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>78.15000000000001</v>
+      </c>
+      <c r="K357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>291.22</v>
+      </c>
+      <c r="K358" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>539.6900000000001</v>
+      </c>
+      <c r="K359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>158.72</v>
+      </c>
+      <c r="K360" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>116.24</v>
+      </c>
+      <c r="K361" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>IGV</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>105.24</v>
+      </c>
+      <c r="K362" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>1065.4</v>
+      </c>
+      <c r="K363" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>10.37</v>
+      </c>
+      <c r="K364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>129.99</v>
+      </c>
+      <c r="K365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>227.3</v>
+      </c>
+      <c r="K366" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>184.19</v>
+      </c>
+      <c r="K367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>1729.75</v>
+      </c>
+      <c r="K368" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>913.59</v>
+      </c>
+      <c r="K369" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>175.96</v>
+      </c>
+      <c r="K370" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>VIAV</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>41.83</v>
+      </c>
+      <c r="K371" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>512.15</v>
+      </c>
+      <c r="K372" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>1834.86</v>
+      </c>
+      <c r="K373" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>78.15000000000001</v>
+      </c>
+      <c r="K374" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>291.22</v>
+      </c>
+      <c r="K375" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>203.38</v>
+      </c>
+      <c r="K376" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>263.28</v>
+      </c>
+      <c r="K377" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>739.02</v>
+      </c>
+      <c r="K378" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>ONTO</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>304.56</v>
+      </c>
+      <c r="K379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="K380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>VIAV</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>41.83</v>
+      </c>
+      <c r="K381" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12278,40 +13664,40 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>42.9</v>
+        <v>37.5</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.18</v>
+        <v>-0.34</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.23</v>
+        <v>-1.11</v>
       </c>
       <c r="G2" t="n">
-        <v>28.6</v>
+        <v>25</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.93</v>
       </c>
       <c r="I2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.36</v>
+        <v>-0.43</v>
       </c>
       <c r="L2" t="n">
-        <v>-1.52</v>
+        <v>-1.53</v>
       </c>
       <c r="M2" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="N2" t="n">
-        <v>-1.03</v>
+        <v>-0.96</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -12324,43 +13710,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C3" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="D3" t="n">
-        <v>53.6</v>
+        <v>51.3</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4</v>
+        <v>0.06</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.46</v>
+        <v>-0.57</v>
       </c>
       <c r="G3" t="n">
-        <v>39.1</v>
+        <v>38.5</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.01</v>
+        <v>-0.38</v>
       </c>
       <c r="I3" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="J3" t="n">
-        <v>65.40000000000001</v>
+        <v>60</v>
       </c>
       <c r="K3" t="n">
-        <v>1.34</v>
+        <v>0.31</v>
       </c>
       <c r="L3" t="n">
-        <v>0.43</v>
+        <v>-0.6</v>
       </c>
       <c r="M3" t="n">
-        <v>57.7</v>
+        <v>51.4</v>
       </c>
       <c r="N3" t="n">
-        <v>0.73</v>
+        <v>0.06</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -12373,43 +13759,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C4" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D4" t="n">
-        <v>71.8</v>
+        <v>68.3</v>
       </c>
       <c r="E4" t="n">
-        <v>3.22</v>
+        <v>3.01</v>
       </c>
       <c r="F4" t="n">
-        <v>2.54</v>
+        <v>2.42</v>
       </c>
       <c r="G4" t="n">
-        <v>59</v>
+        <v>58.5</v>
       </c>
       <c r="H4" t="n">
-        <v>3.04</v>
+        <v>2.82</v>
       </c>
       <c r="I4" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="J4" t="n">
-        <v>71.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="K4" t="n">
-        <v>6.38</v>
+        <v>5.83</v>
       </c>
       <c r="L4" t="n">
-        <v>5.33</v>
+        <v>4.8</v>
       </c>
       <c r="M4" t="n">
-        <v>66.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>6.7</v>
+        <v>6.09</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -12443,22 +13829,22 @@
         <v>1.97</v>
       </c>
       <c r="I5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
-        <v>83.3</v>
+        <v>85.7</v>
       </c>
       <c r="K5" t="n">
-        <v>2.86</v>
+        <v>5.1</v>
       </c>
       <c r="L5" t="n">
-        <v>2.2</v>
+        <v>4.41</v>
       </c>
       <c r="M5" t="n">
-        <v>66.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="N5" t="n">
-        <v>4.75</v>
+        <v>5.8</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -12471,43 +13857,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C6" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D6" t="n">
-        <v>72.3</v>
+        <v>67.3</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="F6" t="n">
-        <v>1.93</v>
+        <v>1.45</v>
       </c>
       <c r="G6" t="n">
-        <v>61.7</v>
+        <v>57.7</v>
       </c>
       <c r="H6" t="n">
-        <v>3.17</v>
+        <v>2.46</v>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J6" t="n">
-        <v>83.3</v>
+        <v>65</v>
       </c>
       <c r="K6" t="n">
-        <v>6.43</v>
+        <v>3.62</v>
       </c>
       <c r="L6" t="n">
-        <v>5.64</v>
+        <v>2.78</v>
       </c>
       <c r="M6" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="N6" t="n">
-        <v>8.4</v>
+        <v>5.07</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -12520,43 +13906,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C7" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D7" t="n">
-        <v>54.2</v>
+        <v>54.9</v>
       </c>
       <c r="E7" t="n">
-        <v>1.5</v>
+        <v>1.58</v>
       </c>
       <c r="F7" t="n">
-        <v>0.74</v>
+        <v>0.93</v>
       </c>
       <c r="G7" t="n">
-        <v>41.7</v>
+        <v>43.1</v>
       </c>
       <c r="H7" t="n">
-        <v>1.69</v>
+        <v>1.73</v>
       </c>
       <c r="I7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J7" t="n">
-        <v>50</v>
+        <v>38.9</v>
       </c>
       <c r="K7" t="n">
-        <v>1.14</v>
+        <v>-0.04</v>
       </c>
       <c r="L7" t="n">
-        <v>0.33</v>
+        <v>-0.87</v>
       </c>
       <c r="M7" t="n">
-        <v>50</v>
+        <v>38.9</v>
       </c>
       <c r="N7" t="n">
-        <v>2.84</v>
+        <v>1.65</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-09-30
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q379"/>
+  <dimension ref="A1:Q411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5970,6 +5970,14 @@
           <t>UP</t>
         </is>
       </c>
+      <c r="G113" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="n">
         <v>-0.48</v>
@@ -5977,6 +5985,12 @@
       <c r="M113" t="n">
         <v>-0.82</v>
       </c>
+      <c r="N113" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="O113" t="n">
+        <v>-0.91</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6001,6 +6015,14 @@
         <v>-0.38</v>
       </c>
       <c r="F114" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H114" t="inlineStr">
         <is>
           <t>FLAT</t>
         </is>
@@ -6012,6 +6034,12 @@
       <c r="M114" t="n">
         <v>-0.9</v>
       </c>
+      <c r="N114" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="O114" t="n">
+        <v>-0.88</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6036,6 +6064,14 @@
         <v>-5.17</v>
       </c>
       <c r="F115" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>-8.369999999999999</v>
+      </c>
+      <c r="H115" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -6047,6 +6083,12 @@
       <c r="M115" t="n">
         <v>-2.8</v>
       </c>
+      <c r="N115" t="n">
+        <v>-9.48</v>
+      </c>
+      <c r="O115" t="n">
+        <v>-6.08</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6071,6 +6113,14 @@
         <v>2.1</v>
       </c>
       <c r="F116" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="H116" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6082,6 +6132,12 @@
       <c r="M116" t="n">
         <v>0.46</v>
       </c>
+      <c r="N116" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="O116" t="n">
+        <v>2.95</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6108,6 +6164,14 @@
       <c r="F117" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K117" t="inlineStr"/>
@@ -6117,6 +6181,12 @@
       <c r="M117" t="n">
         <v>1.13</v>
       </c>
+      <c r="N117" t="n">
+        <v>-5.27</v>
+      </c>
+      <c r="O117" t="n">
+        <v>-3.74</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6141,6 +6211,14 @@
         <v>2.62</v>
       </c>
       <c r="F118" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H118" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6152,6 +6230,12 @@
       <c r="M118" t="n">
         <v>1.93</v>
       </c>
+      <c r="N118" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="O118" t="n">
+        <v>3.19</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6176,6 +6260,14 @@
         <v>10.01</v>
       </c>
       <c r="F119" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="H119" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6187,6 +6279,12 @@
       <c r="M119" t="n">
         <v>8.9</v>
       </c>
+      <c r="N119" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="O119" t="n">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6211,6 +6309,14 @@
         <v>-0.38</v>
       </c>
       <c r="F120" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H120" t="inlineStr">
         <is>
           <t>FLAT</t>
         </is>
@@ -6222,6 +6328,12 @@
       <c r="M120" t="n">
         <v>-0.9</v>
       </c>
+      <c r="N120" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="O120" t="n">
+        <v>-0.88</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6246,6 +6358,14 @@
         <v>-6.76</v>
       </c>
       <c r="F121" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>-10.97</v>
+      </c>
+      <c r="H121" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -6257,6 +6377,12 @@
       <c r="M121" t="n">
         <v>-7.4</v>
       </c>
+      <c r="N121" t="n">
+        <v>-12.09</v>
+      </c>
+      <c r="O121" t="n">
+        <v>-11.58</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6283,6 +6409,14 @@
       <c r="F122" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>-5.84</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K122" t="inlineStr"/>
@@ -6292,6 +6426,12 @@
       <c r="M122" t="n">
         <v>3.32</v>
       </c>
+      <c r="N122" t="n">
+        <v>-6.95</v>
+      </c>
+      <c r="O122" t="n">
+        <v>-5.11</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6316,6 +6456,14 @@
         <v>11.94</v>
       </c>
       <c r="F123" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="H123" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6327,6 +6475,12 @@
       <c r="M123" t="n">
         <v>11.59</v>
       </c>
+      <c r="N123" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="O123" t="n">
+        <v>3.72</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6351,6 +6505,14 @@
         <v>2.99</v>
       </c>
       <c r="F124" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="H124" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6362,6 +6524,12 @@
       <c r="M124" t="n">
         <v>2.77</v>
       </c>
+      <c r="N124" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="O124" t="n">
+        <v>1.18</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6386,6 +6554,14 @@
         <v>13.58</v>
       </c>
       <c r="F125" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G125" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="H125" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6397,6 +6573,12 @@
       <c r="M125" t="n">
         <v>8.58</v>
       </c>
+      <c r="N125" t="n">
+        <v>13.91</v>
+      </c>
+      <c r="O125" t="n">
+        <v>9.960000000000001</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6421,6 +6603,14 @@
         <v>2.1</v>
       </c>
       <c r="F126" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="H126" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6432,6 +6622,12 @@
       <c r="M126" t="n">
         <v>0.46</v>
       </c>
+      <c r="N126" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="O126" t="n">
+        <v>2.95</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6456,6 +6652,14 @@
         <v>1.14</v>
       </c>
       <c r="F127" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="H127" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6467,6 +6671,12 @@
       <c r="M127" t="n">
         <v>0.14</v>
       </c>
+      <c r="N127" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="O127" t="n">
+        <v>1.63</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6491,6 +6701,14 @@
         <v>14.47</v>
       </c>
       <c r="F128" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="H128" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6502,6 +6720,12 @@
       <c r="M128" t="n">
         <v>8.390000000000001</v>
       </c>
+      <c r="N128" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="O128" t="n">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6528,6 +6752,14 @@
       <c r="F129" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K129" t="inlineStr"/>
@@ -6537,6 +6769,12 @@
       <c r="M129" t="n">
         <v>0.57</v>
       </c>
+      <c r="N129" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="O129" t="n">
+        <v>-0.63</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6561,6 +6799,14 @@
         <v>19.92</v>
       </c>
       <c r="F130" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>19.36</v>
+      </c>
+      <c r="H130" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6572,6 +6818,12 @@
       <c r="M130" t="n">
         <v>15.08</v>
       </c>
+      <c r="N130" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="O130" t="n">
+        <v>14.54</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6596,6 +6848,14 @@
         <v>1.91</v>
       </c>
       <c r="F131" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="H131" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6607,6 +6867,12 @@
       <c r="M131" t="n">
         <v>-2.91</v>
       </c>
+      <c r="N131" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="O131" t="n">
+        <v>-2.29</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6631,6 +6897,14 @@
         <v>4.83</v>
       </c>
       <c r="F132" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="H132" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6642,6 +6916,12 @@
       <c r="M132" t="n">
         <v>5.43</v>
       </c>
+      <c r="N132" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="O132" t="n">
+        <v>3.3</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6666,6 +6946,14 @@
         <v>8.75</v>
       </c>
       <c r="F133" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="H133" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6677,6 +6965,12 @@
       <c r="M133" t="n">
         <v>11.11</v>
       </c>
+      <c r="N133" t="n">
+        <v>8.57</v>
+      </c>
+      <c r="O133" t="n">
+        <v>12.05</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6701,6 +6995,14 @@
         <v>-2.39</v>
       </c>
       <c r="F134" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>-4.43</v>
+      </c>
+      <c r="H134" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -6712,6 +7014,12 @@
       <c r="M134" t="n">
         <v>-3.71</v>
       </c>
+      <c r="N134" t="n">
+        <v>-5.55</v>
+      </c>
+      <c r="O134" t="n">
+        <v>-5.72</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6736,6 +7044,14 @@
         <v>3.86</v>
       </c>
       <c r="F135" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="H135" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6747,6 +7063,12 @@
       <c r="M135" t="n">
         <v>4.2</v>
       </c>
+      <c r="N135" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O135" t="n">
+        <v>1.65</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6771,6 +7093,14 @@
         <v>8.529999999999999</v>
       </c>
       <c r="F136" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="H136" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6782,6 +7112,12 @@
       <c r="M136" t="n">
         <v>9.800000000000001</v>
       </c>
+      <c r="N136" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="O136" t="n">
+        <v>8.23</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6808,6 +7144,14 @@
       <c r="F137" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K137" t="inlineStr"/>
@@ -6817,6 +7161,12 @@
       <c r="M137" t="n">
         <v>-3.64</v>
       </c>
+      <c r="N137" t="n">
+        <v>-1.07</v>
+      </c>
+      <c r="O137" t="n">
+        <v>-1.96</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6841,6 +7191,14 @@
         <v>14.47</v>
       </c>
       <c r="F138" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="H138" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6852,6 +7210,12 @@
       <c r="M138" t="n">
         <v>8.390000000000001</v>
       </c>
+      <c r="N138" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="O138" t="n">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6878,6 +7242,14 @@
       <c r="F139" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K139" t="inlineStr"/>
@@ -6887,6 +7259,12 @@
       <c r="M139" t="n">
         <v>1.13</v>
       </c>
+      <c r="N139" t="n">
+        <v>-5.27</v>
+      </c>
+      <c r="O139" t="n">
+        <v>-3.74</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6911,6 +7289,14 @@
         <v>4.01</v>
       </c>
       <c r="F140" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="H140" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -6922,6 +7308,12 @@
       <c r="M140" t="n">
         <v>5.83</v>
       </c>
+      <c r="N140" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="O140" t="n">
+        <v>4.43</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6948,6 +7340,14 @@
       <c r="F141" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>-5.84</v>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K141" t="inlineStr"/>
@@ -6957,6 +7357,12 @@
       <c r="M141" t="n">
         <v>3.32</v>
       </c>
+      <c r="N141" t="n">
+        <v>-6.95</v>
+      </c>
+      <c r="O141" t="n">
+        <v>-5.11</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -10827,7 +11233,21 @@
       <c r="D252" t="n">
         <v>237.58</v>
       </c>
+      <c r="E252" t="n">
+        <v>-3.37</v>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K252" t="inlineStr"/>
+      <c r="L252" t="n">
+        <v>-2.67</v>
+      </c>
+      <c r="M252" t="n">
+        <v>-4.7</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -10848,7 +11268,21 @@
       <c r="D253" t="n">
         <v>500.59</v>
       </c>
+      <c r="E253" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K253" t="inlineStr"/>
+      <c r="L253" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="M253" t="n">
+        <v>3.51</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -10869,7 +11303,21 @@
       <c r="D254" t="n">
         <v>140.78</v>
       </c>
+      <c r="E254" t="n">
+        <v>-4.81</v>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K254" t="inlineStr"/>
+      <c r="L254" t="n">
+        <v>-4.11</v>
+      </c>
+      <c r="M254" t="n">
+        <v>-4.31</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -10890,7 +11338,21 @@
       <c r="D255" t="n">
         <v>28.18</v>
       </c>
+      <c r="E255" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K255" t="inlineStr"/>
+      <c r="L255" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="M255" t="n">
+        <v>1.07</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -10911,7 +11373,21 @@
       <c r="D256" t="n">
         <v>191.79</v>
       </c>
+      <c r="E256" t="n">
+        <v>-2.48</v>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K256" t="inlineStr"/>
+      <c r="L256" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="M256" t="n">
+        <v>-1.24</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -10932,7 +11408,21 @@
       <c r="D257" t="n">
         <v>197.24</v>
       </c>
+      <c r="E257" t="n">
+        <v>-6.68</v>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K257" t="inlineStr"/>
+      <c r="L257" t="n">
+        <v>-5.98</v>
+      </c>
+      <c r="M257" t="n">
+        <v>-6.47</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -10953,7 +11443,21 @@
       <c r="D258" t="n">
         <v>510.4</v>
       </c>
+      <c r="E258" t="n">
+        <v>-4.52</v>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K258" t="inlineStr"/>
+      <c r="L258" t="n">
+        <v>-3.82</v>
+      </c>
+      <c r="M258" t="n">
+        <v>-3.59</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -10974,7 +11478,21 @@
       <c r="D259" t="n">
         <v>214.45</v>
       </c>
+      <c r="E259" t="n">
+        <v>-7.05</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K259" t="inlineStr"/>
+      <c r="L259" t="n">
+        <v>-6.35</v>
+      </c>
+      <c r="M259" t="n">
+        <v>-6.72</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -10995,7 +11513,21 @@
       <c r="D260" t="n">
         <v>154.48</v>
       </c>
+      <c r="E260" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K260" t="inlineStr"/>
+      <c r="L260" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="M260" t="n">
+        <v>2.05</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -11016,7 +11548,21 @@
       <c r="D261" t="n">
         <v>226.61</v>
       </c>
+      <c r="E261" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K261" t="inlineStr"/>
+      <c r="L261" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="M261" t="n">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -11037,7 +11583,21 @@
       <c r="D262" t="n">
         <v>225.51</v>
       </c>
+      <c r="E262" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K262" t="inlineStr"/>
+      <c r="L262" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="M262" t="n">
+        <v>2.7</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -11058,7 +11618,21 @@
       <c r="D263" t="n">
         <v>360.46</v>
       </c>
+      <c r="E263" t="n">
+        <v>-1.25</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K263" t="inlineStr"/>
+      <c r="L263" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="M263" t="n">
+        <v>1.49</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -11079,7 +11653,21 @@
       <c r="D264" t="n">
         <v>332.56</v>
       </c>
+      <c r="E264" t="n">
+        <v>-12.87</v>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K264" t="inlineStr"/>
+      <c r="L264" t="n">
+        <v>-12.17</v>
+      </c>
+      <c r="M264" t="n">
+        <v>-9.33</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -11100,7 +11688,21 @@
       <c r="D265" t="n">
         <v>61.9</v>
       </c>
+      <c r="E265" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K265" t="inlineStr"/>
+      <c r="L265" t="n">
+        <v>-1.76</v>
+      </c>
+      <c r="M265" t="n">
+        <v>-0.9399999999999999</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -11121,7 +11723,21 @@
       <c r="D266" t="n">
         <v>122.7</v>
       </c>
+      <c r="E266" t="n">
+        <v>-8.300000000000001</v>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K266" t="inlineStr"/>
+      <c r="L266" t="n">
+        <v>-7.6</v>
+      </c>
+      <c r="M266" t="n">
+        <v>-5.94</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -11142,7 +11758,21 @@
       <c r="D267" t="n">
         <v>182.11</v>
       </c>
+      <c r="E267" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K267" t="inlineStr"/>
+      <c r="L267" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="M267" t="n">
+        <v>6.48</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -11163,7 +11793,21 @@
       <c r="D268" t="n">
         <v>1071.88</v>
       </c>
+      <c r="E268" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K268" t="inlineStr"/>
+      <c r="L268" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="M268" t="n">
+        <v>1.59</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -13495,6 +14139,678 @@
         <v>41.83</v>
       </c>
       <c r="K379" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>240.04</v>
+      </c>
+      <c r="K380" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>229.57</v>
+      </c>
+      <c r="K381" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>725.29</v>
+      </c>
+      <c r="K382" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>134.01</v>
+      </c>
+      <c r="K383" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>28.53</v>
+      </c>
+      <c r="K384" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>187.04</v>
+      </c>
+      <c r="K385" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>184.06</v>
+      </c>
+      <c r="K386" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>487.35</v>
+      </c>
+      <c r="K387" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>199.34</v>
+      </c>
+      <c r="K388" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>333.01</v>
+      </c>
+      <c r="K389" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>99.58</v>
+      </c>
+      <c r="K390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>276.96</v>
+      </c>
+      <c r="K391" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>538.3200000000001</v>
+      </c>
+      <c r="K392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>153.75</v>
+      </c>
+      <c r="K393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>344.13</v>
+      </c>
+      <c r="K394" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>112.52</v>
+      </c>
+      <c r="K395" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="K396" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>134.01</v>
+      </c>
+      <c r="K397" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>184.06</v>
+      </c>
+      <c r="K398" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>1739.99</v>
+      </c>
+      <c r="K399" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>339.78</v>
+      </c>
+      <c r="K400" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>179.17</v>
+      </c>
+      <c r="K401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>ZETA</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>31.57</v>
+      </c>
+      <c r="K402" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>99.58</v>
+      </c>
+      <c r="K403" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>77.41</v>
+      </c>
+      <c r="K404" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>276.96</v>
+      </c>
+      <c r="K405" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>CAMT</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>155.25</v>
+      </c>
+      <c r="K406" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>971.46</v>
+      </c>
+      <c r="K407" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>192.48</v>
+      </c>
+      <c r="K408" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>236</v>
+      </c>
+      <c r="K409" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>ONTO</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>307.81</v>
+      </c>
+      <c r="K410" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>40.34</v>
+      </c>
+      <c r="K411" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13640,22 +14956,22 @@
         <v>-0.93</v>
       </c>
       <c r="I2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J2" t="n">
-        <v>20</v>
+        <v>28.6</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.43</v>
+        <v>-0.18</v>
       </c>
       <c r="L2" t="n">
-        <v>-1.53</v>
+        <v>-1.29</v>
       </c>
       <c r="M2" t="n">
-        <v>20</v>
+        <v>28.6</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.96</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -13668,43 +14984,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="C3" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="D3" t="n">
-        <v>51.3</v>
+        <v>48.8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.05</v>
+        <v>-0.24</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.58</v>
+        <v>-0.75</v>
       </c>
       <c r="G3" t="n">
-        <v>38.5</v>
+        <v>37.2</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.38</v>
+        <v>-0.61</v>
       </c>
       <c r="I3" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="J3" t="n">
-        <v>60</v>
+        <v>56.8</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3</v>
+        <v>0.02</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.61</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>51.4</v>
+        <v>50</v>
       </c>
       <c r="N3" t="n">
-        <v>0.06</v>
+        <v>-0.21</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -13717,43 +15033,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="C4" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D4" t="n">
-        <v>68.3</v>
+        <v>68.2</v>
       </c>
       <c r="E4" t="n">
-        <v>3.02</v>
+        <v>2.92</v>
       </c>
       <c r="F4" t="n">
         <v>2.42</v>
       </c>
       <c r="G4" t="n">
-        <v>58.5</v>
+        <v>61.4</v>
       </c>
       <c r="H4" t="n">
-        <v>2.82</v>
+        <v>2.78</v>
       </c>
       <c r="I4" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J4" t="n">
-        <v>69.2</v>
+        <v>73.3</v>
       </c>
       <c r="K4" t="n">
-        <v>5.83</v>
+        <v>5.84</v>
       </c>
       <c r="L4" t="n">
         <v>4.8</v>
       </c>
       <c r="M4" t="n">
-        <v>65.40000000000001</v>
+        <v>70</v>
       </c>
       <c r="N4" t="n">
-        <v>6.09</v>
+        <v>5.8</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -13787,22 +15103,22 @@
         <v>1.96</v>
       </c>
       <c r="I5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>85.7</v>
+        <v>87.5</v>
       </c>
       <c r="K5" t="n">
-        <v>5.1</v>
+        <v>5.39</v>
       </c>
       <c r="L5" t="n">
-        <v>4.4</v>
+        <v>4.63</v>
       </c>
       <c r="M5" t="n">
-        <v>71.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="N5" t="n">
-        <v>5.79</v>
+        <v>5.28</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -13815,43 +15131,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C6" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D6" t="n">
-        <v>67.3</v>
+        <v>64.8</v>
       </c>
       <c r="E6" t="n">
-        <v>2.3</v>
+        <v>1.95</v>
       </c>
       <c r="F6" t="n">
-        <v>1.45</v>
+        <v>1.16</v>
       </c>
       <c r="G6" t="n">
-        <v>57.7</v>
+        <v>55.6</v>
       </c>
       <c r="H6" t="n">
-        <v>2.46</v>
+        <v>2.22</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J6" t="n">
-        <v>65</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>3.61</v>
+        <v>3.82</v>
       </c>
       <c r="L6" t="n">
-        <v>2.77</v>
+        <v>2.89</v>
       </c>
       <c r="M6" t="n">
-        <v>55</v>
+        <v>58.6</v>
       </c>
       <c r="N6" t="n">
-        <v>5.06</v>
+        <v>4.5</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -13864,43 +15180,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C7" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D7" t="n">
-        <v>54.9</v>
+        <v>52.7</v>
       </c>
       <c r="E7" t="n">
-        <v>1.58</v>
+        <v>1.37</v>
       </c>
       <c r="F7" t="n">
-        <v>0.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>43.1</v>
+        <v>43.6</v>
       </c>
       <c r="H7" t="n">
-        <v>1.73</v>
+        <v>1.62</v>
       </c>
       <c r="I7" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J7" t="n">
-        <v>38.9</v>
+        <v>40.9</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.88</v>
+        <v>-0.92</v>
       </c>
       <c r="M7" t="n">
-        <v>38.9</v>
+        <v>40.9</v>
       </c>
       <c r="N7" t="n">
-        <v>1.64</v>
+        <v>1.22</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-01
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q412"/>
+  <dimension ref="A1:Q443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7391,6 +7391,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G142" t="n">
+        <v>-2.53</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K142" t="inlineStr"/>
       <c r="L142" t="n">
         <v>-2.51</v>
@@ -7398,6 +7406,12 @@
       <c r="M142" t="n">
         <v>-2.57</v>
       </c>
+      <c r="N142" t="n">
+        <v>-2.72</v>
+      </c>
+      <c r="O142" t="n">
+        <v>-3.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7424,6 +7438,14 @@
       <c r="F143" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G143" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K143" t="inlineStr"/>
@@ -7433,6 +7455,12 @@
       <c r="M143" t="n">
         <v>-0.11</v>
       </c>
+      <c r="N143" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="O143" t="n">
+        <v>2.94</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7457,6 +7485,14 @@
         <v>-0.5</v>
       </c>
       <c r="F144" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G144" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="H144" t="inlineStr">
         <is>
           <t>FLAT</t>
         </is>
@@ -7468,6 +7504,12 @@
       <c r="M144" t="n">
         <v>-1.48</v>
       </c>
+      <c r="N144" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="O144" t="n">
+        <v>-1.47</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7492,6 +7534,14 @@
         <v>2.79</v>
       </c>
       <c r="F145" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G145" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="H145" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -7503,6 +7553,12 @@
       <c r="M145" t="n">
         <v>2.69</v>
       </c>
+      <c r="N145" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="O145" t="n">
+        <v>1.64</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7527,6 +7583,14 @@
         <v>9.279999999999999</v>
       </c>
       <c r="F146" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G146" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="H146" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -7538,6 +7602,12 @@
       <c r="M146" t="n">
         <v>8.6</v>
       </c>
+      <c r="N146" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="O146" t="n">
+        <v>7.14</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7564,6 +7634,14 @@
       <c r="F147" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G147" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K147" t="inlineStr"/>
@@ -7573,6 +7651,12 @@
       <c r="M147" t="n">
         <v>-0.19</v>
       </c>
+      <c r="N147" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7597,6 +7681,14 @@
         <v>-3.3</v>
       </c>
       <c r="F148" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G148" t="n">
+        <v>-7.1</v>
+      </c>
+      <c r="H148" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -7608,6 +7700,12 @@
       <c r="M148" t="n">
         <v>-3.14</v>
       </c>
+      <c r="N148" t="n">
+        <v>-7.29</v>
+      </c>
+      <c r="O148" t="n">
+        <v>-6.95</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7634,6 +7732,14 @@
       <c r="F149" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G149" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K149" t="inlineStr"/>
@@ -7643,6 +7749,12 @@
       <c r="M149" t="n">
         <v>-0.54</v>
       </c>
+      <c r="N149" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="O149" t="n">
+        <v>-1.95</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7667,6 +7779,14 @@
         <v>8.69</v>
       </c>
       <c r="F150" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G150" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H150" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -7678,6 +7798,12 @@
       <c r="M150" t="n">
         <v>7.76</v>
       </c>
+      <c r="N150" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="O150" t="n">
+        <v>-0.21</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7702,6 +7828,14 @@
         <v>10.54</v>
       </c>
       <c r="F151" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G151" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="H151" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -7713,6 +7847,12 @@
       <c r="M151" t="n">
         <v>9.630000000000001</v>
       </c>
+      <c r="N151" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="O151" t="n">
+        <v>11.37</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7737,6 +7877,14 @@
         <v>-0.5</v>
       </c>
       <c r="F152" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G152" t="n">
+        <v>-0.49</v>
+      </c>
+      <c r="H152" t="inlineStr">
         <is>
           <t>FLAT</t>
         </is>
@@ -7748,6 +7896,12 @@
       <c r="M152" t="n">
         <v>-1.48</v>
       </c>
+      <c r="N152" t="n">
+        <v>-0.68</v>
+      </c>
+      <c r="O152" t="n">
+        <v>-1.47</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7772,6 +7926,14 @@
         <v>8.619999999999999</v>
       </c>
       <c r="F153" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G153" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="H153" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -7783,6 +7945,12 @@
       <c r="M153" t="n">
         <v>7.8</v>
       </c>
+      <c r="N153" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="O153" t="n">
+        <v>9.85</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7809,6 +7977,14 @@
       <c r="F154" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G154" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K154" t="inlineStr"/>
@@ -7818,6 +7994,12 @@
       <c r="M154" t="n">
         <v>-0.54</v>
       </c>
+      <c r="N154" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="O154" t="n">
+        <v>-1.95</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7844,6 +8026,14 @@
       <c r="F155" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G155" t="n">
+        <v>6.77</v>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K155" t="inlineStr"/>
@@ -7853,6 +8043,12 @@
       <c r="M155" t="n">
         <v>-3.94</v>
       </c>
+      <c r="N155" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="O155" t="n">
+        <v>5.35</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7879,6 +8075,14 @@
       <c r="F156" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G156" t="n">
+        <v>-1.87</v>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K156" t="inlineStr"/>
@@ -7888,6 +8092,12 @@
       <c r="M156" t="n">
         <v>-1.49</v>
       </c>
+      <c r="N156" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="O156" t="n">
+        <v>-5.54</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7912,6 +8122,14 @@
         <v>-3.43</v>
       </c>
       <c r="F157" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G157" t="n">
+        <v>-8.880000000000001</v>
+      </c>
+      <c r="H157" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -7923,6 +8141,12 @@
       <c r="M157" t="n">
         <v>-4.14</v>
       </c>
+      <c r="N157" t="n">
+        <v>-9.06</v>
+      </c>
+      <c r="O157" t="n">
+        <v>-9.550000000000001</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7947,6 +8171,14 @@
         <v>15.44</v>
       </c>
       <c r="F158" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G158" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="H158" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -7958,6 +8190,12 @@
       <c r="M158" t="n">
         <v>14.86</v>
       </c>
+      <c r="N158" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="O158" t="n">
+        <v>12.37</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7982,6 +8220,14 @@
         <v>-5.03</v>
       </c>
       <c r="F159" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G159" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="H159" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -7993,6 +8239,12 @@
       <c r="M159" t="n">
         <v>-6.31</v>
       </c>
+      <c r="N159" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="O159" t="n">
+        <v>-2.48</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -8017,6 +8269,14 @@
         <v>2.93</v>
       </c>
       <c r="F160" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G160" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="H160" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8028,6 +8288,12 @@
       <c r="M160" t="n">
         <v>2.09</v>
       </c>
+      <c r="N160" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="O160" t="n">
+        <v>1.72</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8052,6 +8318,14 @@
         <v>5.69</v>
       </c>
       <c r="F161" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G161" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="H161" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8063,6 +8337,12 @@
       <c r="M161" t="n">
         <v>5.04</v>
       </c>
+      <c r="N161" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="O161" t="n">
+        <v>7.67</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8087,6 +8367,14 @@
         <v>-8.9</v>
       </c>
       <c r="F162" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G162" t="n">
+        <v>-7.94</v>
+      </c>
+      <c r="H162" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -8098,6 +8386,12 @@
       <c r="M162" t="n">
         <v>-9.73</v>
       </c>
+      <c r="N162" t="n">
+        <v>-8.119999999999999</v>
+      </c>
+      <c r="O162" t="n">
+        <v>-8.77</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8122,6 +8416,14 @@
         <v>1.41</v>
       </c>
       <c r="F163" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G163" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="H163" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8133,6 +8435,12 @@
       <c r="M163" t="n">
         <v>0.85</v>
       </c>
+      <c r="N163" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="O163" t="n">
+        <v>0.41</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8159,6 +8467,14 @@
       <c r="F164" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G164" t="n">
+        <v>-1.87</v>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K164" t="inlineStr"/>
@@ -8168,6 +8484,12 @@
       <c r="M164" t="n">
         <v>-1.49</v>
       </c>
+      <c r="N164" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="O164" t="n">
+        <v>-5.54</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8192,6 +8514,14 @@
         <v>17.09</v>
       </c>
       <c r="F165" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G165" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="H165" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8203,6 +8533,12 @@
       <c r="M165" t="n">
         <v>15.92</v>
       </c>
+      <c r="N165" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="O165" t="n">
+        <v>9.15</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8227,6 +8563,14 @@
         <v>7.45</v>
       </c>
       <c r="F166" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G166" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="H166" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8238,6 +8582,12 @@
       <c r="M166" t="n">
         <v>6.06</v>
       </c>
+      <c r="N166" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="O166" t="n">
+        <v>3.75</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8262,6 +8612,14 @@
         <v>3.41</v>
       </c>
       <c r="F167" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G167" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="H167" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8273,6 +8631,12 @@
       <c r="M167" t="n">
         <v>3.57</v>
       </c>
+      <c r="N167" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="O167" t="n">
+        <v>6.51</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8299,6 +8663,14 @@
       <c r="F168" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G168" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K168" t="inlineStr"/>
@@ -8308,6 +8680,12 @@
       <c r="M168" t="n">
         <v>-0.54</v>
       </c>
+      <c r="N168" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="O168" t="n">
+        <v>-1.95</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11828,7 +12206,21 @@
       <c r="D269" t="n">
         <v>238.22</v>
       </c>
+      <c r="E269" t="n">
+        <v>-0.64</v>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K269" t="inlineStr"/>
+      <c r="L269" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="M269" t="n">
+        <v>-0.24</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -11849,7 +12241,21 @@
       <c r="D270" t="n">
         <v>777.59</v>
       </c>
+      <c r="E270" t="n">
+        <v>-6.62</v>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K270" t="inlineStr"/>
+      <c r="L270" t="n">
+        <v>-6.21</v>
+      </c>
+      <c r="M270" t="n">
+        <v>-5.66</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -11870,7 +12276,21 @@
       <c r="D271" t="n">
         <v>497.93</v>
       </c>
+      <c r="E271" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K271" t="inlineStr"/>
+      <c r="L271" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="M271" t="n">
+        <v>2.72</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -11891,7 +12311,21 @@
       <c r="D272" t="n">
         <v>137.78</v>
       </c>
+      <c r="E272" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K272" t="inlineStr"/>
+      <c r="L272" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M272" t="n">
+        <v>0.29</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -11912,7 +12346,21 @@
       <c r="D273" t="n">
         <v>28.41</v>
       </c>
+      <c r="E273" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K273" t="inlineStr"/>
+      <c r="L273" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="M273" t="n">
+        <v>-1.26</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -11933,7 +12381,21 @@
       <c r="D274" t="n">
         <v>192.59</v>
       </c>
+      <c r="E274" t="n">
+        <v>-1.34</v>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K274" t="inlineStr"/>
+      <c r="L274" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="M274" t="n">
+        <v>-1.51</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -11954,7 +12416,21 @@
       <c r="D275" t="n">
         <v>194.26</v>
       </c>
+      <c r="E275" t="n">
+        <v>-6.3</v>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K275" t="inlineStr"/>
+      <c r="L275" t="n">
+        <v>-5.88</v>
+      </c>
+      <c r="M275" t="n">
+        <v>-6.77</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -11975,7 +12451,21 @@
       <c r="D276" t="n">
         <v>511.38</v>
       </c>
+      <c r="E276" t="n">
+        <v>-3.93</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K276" t="inlineStr"/>
+      <c r="L276" t="n">
+        <v>-3.52</v>
+      </c>
+      <c r="M276" t="n">
+        <v>-3.72</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -11996,7 +12486,21 @@
       <c r="D277" t="n">
         <v>214.64</v>
       </c>
+      <c r="E277" t="n">
+        <v>-7.39</v>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K277" t="inlineStr"/>
+      <c r="L277" t="n">
+        <v>-6.98</v>
+      </c>
+      <c r="M277" t="n">
+        <v>-3.6</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -12017,7 +12521,21 @@
       <c r="D278" t="n">
         <v>154.15</v>
       </c>
+      <c r="E278" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K278" t="inlineStr"/>
+      <c r="L278" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="M278" t="n">
+        <v>2.78</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -12038,7 +12556,21 @@
       <c r="D279" t="n">
         <v>120.82</v>
       </c>
+      <c r="E279" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K279" t="inlineStr"/>
+      <c r="L279" t="n">
+        <v>-7.58</v>
+      </c>
+      <c r="M279" t="n">
+        <v>-8.710000000000001</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -12059,7 +12591,21 @@
       <c r="D280" t="n">
         <v>107.15</v>
       </c>
+      <c r="E280" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K280" t="inlineStr"/>
+      <c r="L280" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="M280" t="n">
+        <v>0.53</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -12080,7 +12626,21 @@
       <c r="D281" t="n">
         <v>224.58</v>
       </c>
+      <c r="E281" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K281" t="inlineStr"/>
+      <c r="L281" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="M281" t="n">
+        <v>2.49</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -12101,7 +12661,21 @@
       <c r="D282" t="n">
         <v>360.51</v>
       </c>
+      <c r="E282" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K282" t="inlineStr"/>
+      <c r="L282" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="M282" t="n">
+        <v>-2.81</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -12122,7 +12696,21 @@
       <c r="D283" t="n">
         <v>629.26</v>
       </c>
+      <c r="E283" t="n">
+        <v>-2.16</v>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K283" t="inlineStr"/>
+      <c r="L283" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="M283" t="n">
+        <v>-3.08</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -12143,7 +12731,21 @@
       <c r="D284" t="n">
         <v>306.34</v>
       </c>
+      <c r="E284" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K284" t="inlineStr"/>
+      <c r="L284" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="M284" t="n">
+        <v>-8.31</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -12164,7 +12766,21 @@
       <c r="D285" t="n">
         <v>127.39</v>
       </c>
+      <c r="E285" t="n">
+        <v>-5.83</v>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K285" t="inlineStr"/>
+      <c r="L285" t="n">
+        <v>-5.42</v>
+      </c>
+      <c r="M285" t="n">
+        <v>-5.52</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -12185,7 +12801,21 @@
       <c r="D286" t="n">
         <v>8.73</v>
       </c>
+      <c r="E286" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K286" t="inlineStr"/>
+      <c r="L286" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="M286" t="n">
+        <v>4.76</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -12206,7 +12836,21 @@
       <c r="D287" t="n">
         <v>777.59</v>
       </c>
+      <c r="E287" t="n">
+        <v>-6.62</v>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K287" t="inlineStr"/>
+      <c r="L287" t="n">
+        <v>-6.21</v>
+      </c>
+      <c r="M287" t="n">
+        <v>-5.66</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -12227,7 +12871,21 @@
       <c r="D288" t="n">
         <v>194.82</v>
       </c>
+      <c r="E288" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K288" t="inlineStr"/>
+      <c r="L288" t="n">
+        <v>-2.62</v>
+      </c>
+      <c r="M288" t="n">
+        <v>-3.39</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -12248,7 +12906,21 @@
       <c r="D289" t="n">
         <v>1080.53</v>
       </c>
+      <c r="E289" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K289" t="inlineStr"/>
+      <c r="L289" t="n">
+        <v>2</v>
+      </c>
+      <c r="M289" t="n">
+        <v>0.07000000000000001</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -12269,7 +12941,21 @@
       <c r="D290" t="n">
         <v>243.48</v>
       </c>
+      <c r="E290" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K290" t="inlineStr"/>
+      <c r="L290" t="n">
+        <v>-4.19</v>
+      </c>
+      <c r="M290" t="n">
+        <v>-5.52</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -12290,7 +12976,21 @@
       <c r="D291" t="n">
         <v>41.37</v>
       </c>
+      <c r="E291" t="n">
+        <v>-1.31</v>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K291" t="inlineStr"/>
+      <c r="L291" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="M291" t="n">
+        <v>-2.79</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -12311,7 +13011,21 @@
       <c r="D292" t="n">
         <v>192.59</v>
       </c>
+      <c r="E292" t="n">
+        <v>-1.34</v>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K292" t="inlineStr"/>
+      <c r="L292" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="M292" t="n">
+        <v>-1.51</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -14832,6 +15546,657 @@
         <v>40.34</v>
       </c>
       <c r="K412" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>241.27</v>
+      </c>
+      <c r="K413" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>236.7</v>
+      </c>
+      <c r="K414" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>726.09</v>
+      </c>
+      <c r="K415" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>137.79</v>
+      </c>
+      <c r="K416" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>28.12</v>
+      </c>
+      <c r="K417" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>190</v>
+      </c>
+      <c r="K418" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>182.03</v>
+      </c>
+      <c r="K419" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>491.28</v>
+      </c>
+      <c r="K420" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>198.78</v>
+      </c>
+      <c r="K421" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>330.48</v>
+      </c>
+      <c r="K422" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>101.64</v>
+      </c>
+      <c r="K423" t="inlineStr"/>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>277.56</v>
+      </c>
+      <c r="K424" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>236.7</v>
+      </c>
+      <c r="K425" t="inlineStr"/>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>541.7</v>
+      </c>
+      <c r="K426" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>160.49</v>
+      </c>
+      <c r="K427" t="inlineStr"/>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>111.16</v>
+      </c>
+      <c r="K428" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="K429" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>137.79</v>
+      </c>
+      <c r="K430" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>54.96</v>
+      </c>
+      <c r="K431" t="inlineStr"/>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>28.12</v>
+      </c>
+      <c r="K432" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>182.03</v>
+      </c>
+      <c r="K433" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>1786.91</v>
+      </c>
+      <c r="K434" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>FOTO</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="K435" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>AEHR</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>101.64</v>
+      </c>
+      <c r="K436" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="K437" t="inlineStr"/>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>FOTO</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="K438" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>COHR</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>319.3</v>
+      </c>
+      <c r="K439" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>1045.61</v>
+      </c>
+      <c r="K440" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>268.01</v>
+      </c>
+      <c r="K441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>ONTO</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>314.71</v>
+      </c>
+      <c r="K442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>1786.91</v>
+      </c>
+      <c r="K443" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15005,43 +16370,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="C3" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D3" t="n">
-        <v>48.8</v>
+        <v>46.3</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.25</v>
+        <v>-0.48</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.75</v>
+        <v>-0.9</v>
       </c>
       <c r="G3" t="n">
-        <v>37.2</v>
+        <v>35.8</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.61</v>
+        <v>-0.76</v>
       </c>
       <c r="I3" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="J3" t="n">
-        <v>56.8</v>
+        <v>56.6</v>
       </c>
       <c r="K3" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.77</v>
       </c>
       <c r="M3" t="n">
-        <v>50</v>
+        <v>50.9</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.21</v>
+        <v>-0.2</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -15054,43 +16419,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="C4" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D4" t="n">
-        <v>68.2</v>
+        <v>68.8</v>
       </c>
       <c r="E4" t="n">
-        <v>2.92</v>
+        <v>2.68</v>
       </c>
       <c r="F4" t="n">
-        <v>2.42</v>
+        <v>2.25</v>
       </c>
       <c r="G4" t="n">
-        <v>61.4</v>
+        <v>62.5</v>
       </c>
       <c r="H4" t="n">
-        <v>2.78</v>
+        <v>2.48</v>
       </c>
       <c r="I4" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="J4" t="n">
-        <v>73.3</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>5.84</v>
+        <v>5.81</v>
       </c>
       <c r="L4" t="n">
-        <v>4.8</v>
+        <v>4.89</v>
       </c>
       <c r="M4" t="n">
-        <v>70</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="N4" t="n">
-        <v>5.8</v>
+        <v>5.63</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -15103,7 +16468,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="n">
         <v>20</v>
@@ -15124,22 +16489,22 @@
         <v>1.96</v>
       </c>
       <c r="I5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J5" t="n">
-        <v>87.5</v>
+        <v>70</v>
       </c>
       <c r="K5" t="n">
-        <v>5.4</v>
+        <v>3.24</v>
       </c>
       <c r="L5" t="n">
-        <v>4.64</v>
+        <v>2.6</v>
       </c>
       <c r="M5" t="n">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="N5" t="n">
-        <v>5.29</v>
+        <v>2.72</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -15152,43 +16517,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C6" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D6" t="n">
-        <v>64.8</v>
+        <v>60.3</v>
       </c>
       <c r="E6" t="n">
-        <v>1.95</v>
+        <v>1.58</v>
       </c>
       <c r="F6" t="n">
-        <v>1.16</v>
+        <v>0.87</v>
       </c>
       <c r="G6" t="n">
-        <v>55.6</v>
+        <v>51.7</v>
       </c>
       <c r="H6" t="n">
-        <v>2.22</v>
+        <v>1.73</v>
       </c>
       <c r="I6" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="J6" t="n">
-        <v>72.40000000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>3.81</v>
+        <v>3.61</v>
       </c>
       <c r="L6" t="n">
-        <v>2.89</v>
+        <v>2.81</v>
       </c>
       <c r="M6" t="n">
-        <v>58.6</v>
+        <v>60</v>
       </c>
       <c r="N6" t="n">
-        <v>4.5</v>
+        <v>4.04</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -15201,43 +16566,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C7" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D7" t="n">
-        <v>52.7</v>
+        <v>50</v>
       </c>
       <c r="E7" t="n">
-        <v>1.37</v>
+        <v>1.05</v>
       </c>
       <c r="F7" t="n">
-        <v>0.82</v>
+        <v>0.61</v>
       </c>
       <c r="G7" t="n">
-        <v>43.6</v>
+        <v>41.9</v>
       </c>
       <c r="H7" t="n">
-        <v>1.62</v>
+        <v>1.22</v>
       </c>
       <c r="I7" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J7" t="n">
-        <v>40.9</v>
+        <v>44.4</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.04</v>
+        <v>0.65</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.93</v>
+        <v>-0.1</v>
       </c>
       <c r="M7" t="n">
-        <v>40.9</v>
+        <v>44.4</v>
       </c>
       <c r="N7" t="n">
-        <v>1.22</v>
+        <v>1.43</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-02
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q441"/>
+  <dimension ref="A1:Q460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8714,6 +8714,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G169" t="n">
+        <v>-1.38</v>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="n">
         <v>-2.91</v>
@@ -8721,6 +8729,12 @@
       <c r="M169" t="n">
         <v>-2.51</v>
       </c>
+      <c r="N169" t="n">
+        <v>-2.43</v>
+      </c>
+      <c r="O169" t="n">
+        <v>-2.25</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8745,6 +8759,14 @@
         <v>4.53</v>
       </c>
       <c r="F170" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G170" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="H170" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8756,6 +8778,12 @@
       <c r="M170" t="n">
         <v>4.19</v>
       </c>
+      <c r="N170" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="O170" t="n">
+        <v>4.53</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8782,6 +8810,14 @@
       <c r="F171" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G171" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K171" t="inlineStr"/>
@@ -8791,6 +8827,12 @@
       <c r="M171" t="n">
         <v>-0.98</v>
       </c>
+      <c r="N171" t="n">
+        <v>-1.86</v>
+      </c>
+      <c r="O171" t="n">
+        <v>-1.89</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8817,6 +8859,14 @@
       <c r="F172" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G172" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K172" t="inlineStr"/>
@@ -8826,6 +8876,12 @@
       <c r="M172" t="n">
         <v>3.59</v>
       </c>
+      <c r="N172" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="O172" t="n">
+        <v>0.42</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8850,6 +8906,14 @@
         <v>6.77</v>
       </c>
       <c r="F173" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G173" t="n">
+        <v>6.28</v>
+      </c>
+      <c r="H173" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -8861,6 +8925,12 @@
       <c r="M173" t="n">
         <v>6.02</v>
       </c>
+      <c r="N173" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="O173" t="n">
+        <v>5.53</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8887,6 +8957,14 @@
       <c r="F174" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G174" t="n">
+        <v>-7.17</v>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K174" t="inlineStr"/>
@@ -8896,6 +8974,12 @@
       <c r="M174" t="n">
         <v>0.12</v>
       </c>
+      <c r="N174" t="n">
+        <v>-8.220000000000001</v>
+      </c>
+      <c r="O174" t="n">
+        <v>-7.17</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8920,6 +9004,14 @@
         <v>-2.23</v>
       </c>
       <c r="F175" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G175" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="H175" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -8931,6 +9023,12 @@
       <c r="M175" t="n">
         <v>-3.56</v>
       </c>
+      <c r="N175" t="n">
+        <v>-3.25</v>
+      </c>
+      <c r="O175" t="n">
+        <v>-3.53</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8957,6 +9055,14 @@
       <c r="F176" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G176" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K176" t="inlineStr"/>
@@ -8966,6 +9072,12 @@
       <c r="M176" t="n">
         <v>-2.1</v>
       </c>
+      <c r="N176" t="n">
+        <v>-1.43</v>
+      </c>
+      <c r="O176" t="n">
+        <v>-0.31</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8990,6 +9102,14 @@
         <v>6.17</v>
       </c>
       <c r="F177" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G177" t="n">
+        <v>8.619999999999999</v>
+      </c>
+      <c r="H177" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9001,6 +9121,12 @@
       <c r="M177" t="n">
         <v>4.93</v>
       </c>
+      <c r="N177" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="O177" t="n">
+        <v>7.36</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -9025,6 +9151,14 @@
         <v>9.09</v>
       </c>
       <c r="F178" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G178" t="n">
+        <v>21.47</v>
+      </c>
+      <c r="H178" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9036,6 +9170,12 @@
       <c r="M178" t="n">
         <v>6.27</v>
       </c>
+      <c r="N178" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="O178" t="n">
+        <v>18.34</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -9062,6 +9202,14 @@
       <c r="F179" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G179" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K179" t="inlineStr"/>
@@ -9071,6 +9219,12 @@
       <c r="M179" t="n">
         <v>-5.01</v>
       </c>
+      <c r="N179" t="n">
+        <v>-6.84</v>
+      </c>
+      <c r="O179" t="n">
+        <v>-10.91</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -9095,6 +9249,14 @@
         <v>-3.03</v>
       </c>
       <c r="F180" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G180" t="n">
+        <v>-11.51</v>
+      </c>
+      <c r="H180" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -9106,6 +9268,12 @@
       <c r="M180" t="n">
         <v>-9.369999999999999</v>
       </c>
+      <c r="N180" t="n">
+        <v>-12.55</v>
+      </c>
+      <c r="O180" t="n">
+        <v>-17.3</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -9130,6 +9298,14 @@
         <v>9.19</v>
       </c>
       <c r="F181" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G181" t="n">
+        <v>24.39</v>
+      </c>
+      <c r="H181" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9141,6 +9317,12 @@
       <c r="M181" t="n">
         <v>5.65</v>
       </c>
+      <c r="N181" t="n">
+        <v>23.34</v>
+      </c>
+      <c r="O181" t="n">
+        <v>20.37</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -9167,6 +9349,14 @@
       <c r="F182" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G182" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K182" t="inlineStr"/>
@@ -9176,6 +9366,12 @@
       <c r="M182" t="n">
         <v>2.42</v>
       </c>
+      <c r="N182" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="O182" t="n">
+        <v>-5.16</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9202,6 +9398,14 @@
       <c r="F183" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G183" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K183" t="inlineStr"/>
@@ -9211,6 +9415,12 @@
       <c r="M183" t="n">
         <v>1.63</v>
       </c>
+      <c r="N183" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="O183" t="n">
+        <v>-0.54</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -9235,6 +9445,14 @@
         <v>12.65</v>
       </c>
       <c r="F184" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G184" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="H184" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9246,6 +9464,12 @@
       <c r="M184" t="n">
         <v>7.91</v>
       </c>
+      <c r="N184" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="O184" t="n">
+        <v>8.44</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9270,6 +9494,14 @@
         <v>12.59</v>
       </c>
       <c r="F185" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G185" t="n">
+        <v>11.56</v>
+      </c>
+      <c r="H185" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9281,6 +9513,12 @@
       <c r="M185" t="n">
         <v>5.32</v>
       </c>
+      <c r="N185" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="O185" t="n">
+        <v>4.35</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -9305,6 +9543,14 @@
         <v>8.69</v>
       </c>
       <c r="F186" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G186" t="n">
+        <v>8.880000000000001</v>
+      </c>
+      <c r="H186" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9316,6 +9562,12 @@
       <c r="M186" t="n">
         <v>6.83</v>
       </c>
+      <c r="N186" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="O186" t="n">
+        <v>7.02</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -9342,6 +9594,14 @@
       <c r="F187" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G187" t="n">
+        <v>-5.79</v>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K187" t="inlineStr"/>
@@ -9351,6 +9611,12 @@
       <c r="M187" t="n">
         <v>-5.01</v>
       </c>
+      <c r="N187" t="n">
+        <v>-6.84</v>
+      </c>
+      <c r="O187" t="n">
+        <v>-10.91</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -9375,6 +9641,14 @@
         <v>6.09</v>
       </c>
       <c r="F188" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G188" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="H188" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9386,6 +9660,12 @@
       <c r="M188" t="n">
         <v>8.76</v>
       </c>
+      <c r="N188" t="n">
+        <v>12.59</v>
+      </c>
+      <c r="O188" t="n">
+        <v>16.5</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -9410,6 +9690,14 @@
         <v>0.83</v>
       </c>
       <c r="F189" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G189" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="H189" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9421,6 +9709,12 @@
       <c r="M189" t="n">
         <v>0.03</v>
       </c>
+      <c r="N189" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="O189" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -9445,6 +9739,14 @@
         <v>-3.33</v>
       </c>
       <c r="F190" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G190" t="n">
+        <v>-14.29</v>
+      </c>
+      <c r="H190" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -9456,6 +9758,12 @@
       <c r="M190" t="n">
         <v>-5.11</v>
       </c>
+      <c r="N190" t="n">
+        <v>-15.33</v>
+      </c>
+      <c r="O190" t="n">
+        <v>-15.88</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -9482,6 +9790,14 @@
       <c r="F191" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G191" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K191" t="inlineStr"/>
@@ -9491,6 +9807,12 @@
       <c r="M191" t="n">
         <v>-9.49</v>
       </c>
+      <c r="N191" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="O191" t="n">
+        <v>3.17</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -9517,6 +9839,14 @@
       <c r="F192" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G192" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K192" t="inlineStr"/>
@@ -9526,6 +9856,12 @@
       <c r="M192" t="n">
         <v>-2.75</v>
       </c>
+      <c r="N192" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="O192" t="n">
+        <v>0.66</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -9552,6 +9888,14 @@
       <c r="F193" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G193" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K193" t="inlineStr"/>
@@ -9561,6 +9905,12 @@
       <c r="M193" t="n">
         <v>-0.65</v>
       </c>
+      <c r="N193" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="O193" t="n">
+        <v>3.23</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9587,6 +9937,14 @@
       <c r="F194" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G194" t="n">
+        <v>-5.91</v>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K194" t="inlineStr"/>
@@ -9596,6 +9954,12 @@
       <c r="M194" t="n">
         <v>-4.61</v>
       </c>
+      <c r="N194" t="n">
+        <v>-6.96</v>
+      </c>
+      <c r="O194" t="n">
+        <v>-9.94</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9620,6 +9984,14 @@
         <v>29.11</v>
       </c>
       <c r="F195" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G195" t="n">
+        <v>23.29</v>
+      </c>
+      <c r="H195" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9631,6 +10003,12 @@
       <c r="M195" t="n">
         <v>23.39</v>
       </c>
+      <c r="N195" t="n">
+        <v>22.24</v>
+      </c>
+      <c r="O195" t="n">
+        <v>17.82</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -9655,6 +10033,14 @@
         <v>6.54</v>
       </c>
       <c r="F196" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G196" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="H196" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9666,6 +10052,12 @@
       <c r="M196" t="n">
         <v>3.47</v>
       </c>
+      <c r="N196" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="O196" t="n">
+        <v>2.7</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -9690,6 +10082,14 @@
         <v>7.86</v>
       </c>
       <c r="F197" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="H197" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9701,6 +10101,12 @@
       <c r="M197" t="n">
         <v>6.63</v>
       </c>
+      <c r="N197" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="O197" t="n">
+        <v>6.56</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -9725,6 +10131,14 @@
         <v>13.65</v>
       </c>
       <c r="F198" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="H198" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -9736,6 +10150,12 @@
       <c r="M198" t="n">
         <v>11.73</v>
       </c>
+      <c r="N198" t="n">
+        <v>3</v>
+      </c>
+      <c r="O198" t="n">
+        <v>2.28</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -9762,6 +10182,14 @@
       <c r="F199" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K199" t="inlineStr"/>
@@ -9771,6 +10199,12 @@
       <c r="M199" t="n">
         <v>-4.03</v>
       </c>
+      <c r="N199" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="O199" t="n">
+        <v>2.62</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13046,7 +13480,21 @@
       <c r="D293" t="n">
         <v>234.02</v>
       </c>
+      <c r="E293" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K293" t="inlineStr"/>
+      <c r="L293" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="M293" t="n">
+        <v>4.2</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -13067,7 +13515,21 @@
       <c r="D294" t="n">
         <v>751.66</v>
       </c>
+      <c r="E294" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K294" t="inlineStr"/>
+      <c r="L294" t="n">
+        <v>-2.92</v>
+      </c>
+      <c r="M294" t="n">
+        <v>-3.03</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -13088,7 +13550,21 @@
       <c r="D295" t="n">
         <v>516.17</v>
       </c>
+      <c r="E295" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K295" t="inlineStr"/>
+      <c r="L295" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M295" t="n">
+        <v>2.35</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -13109,7 +13585,21 @@
       <c r="D296" t="n">
         <v>135.62</v>
       </c>
+      <c r="E296" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K296" t="inlineStr"/>
+      <c r="L296" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="M296" t="n">
+        <v>3.42</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -13130,7 +13620,21 @@
       <c r="D297" t="n">
         <v>28.67</v>
       </c>
+      <c r="E297" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K297" t="inlineStr"/>
+      <c r="L297" t="n">
+        <v>-2.83</v>
+      </c>
+      <c r="M297" t="n">
+        <v>-2.98</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -13151,7 +13655,21 @@
       <c r="D298" t="n">
         <v>189.67</v>
       </c>
+      <c r="E298" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K298" t="inlineStr"/>
+      <c r="L298" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="M298" t="n">
+        <v>1.27</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -13172,7 +13690,21 @@
       <c r="D299" t="n">
         <v>201.97</v>
       </c>
+      <c r="E299" t="n">
+        <v>-8.449999999999999</v>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K299" t="inlineStr"/>
+      <c r="L299" t="n">
+        <v>-8.23</v>
+      </c>
+      <c r="M299" t="n">
+        <v>-7.26</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -13193,7 +13725,21 @@
       <c r="D300" t="n">
         <v>510.01</v>
       </c>
+      <c r="E300" t="n">
+        <v>-7.28</v>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K300" t="inlineStr"/>
+      <c r="L300" t="n">
+        <v>-7.06</v>
+      </c>
+      <c r="M300" t="n">
+        <v>-6.83</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -13214,7 +13760,21 @@
       <c r="D301" t="n">
         <v>193.05</v>
       </c>
+      <c r="E301" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K301" t="inlineStr"/>
+      <c r="L301" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="M301" t="n">
+        <v>3.96</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -13235,7 +13795,21 @@
       <c r="D302" t="n">
         <v>156.74</v>
       </c>
+      <c r="E302" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K302" t="inlineStr"/>
+      <c r="L302" t="n">
+        <v>5</v>
+      </c>
+      <c r="M302" t="n">
+        <v>6.36</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -13256,7 +13830,21 @@
       <c r="D303" t="n">
         <v>119.4</v>
       </c>
+      <c r="E303" t="n">
+        <v>-5.58</v>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K303" t="inlineStr"/>
+      <c r="L303" t="n">
+        <v>-5.36</v>
+      </c>
+      <c r="M303" t="n">
+        <v>-4.58</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -13277,7 +13865,21 @@
       <c r="D304" t="n">
         <v>106.01</v>
       </c>
+      <c r="E304" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K304" t="inlineStr"/>
+      <c r="L304" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="M304" t="n">
+        <v>4.36</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -13298,7 +13900,21 @@
       <c r="D305" t="n">
         <v>135.62</v>
       </c>
+      <c r="E305" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K305" t="inlineStr"/>
+      <c r="L305" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="M305" t="n">
+        <v>3.42</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -13319,7 +13935,21 @@
       <c r="D306" t="n">
         <v>225.07</v>
       </c>
+      <c r="E306" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K306" t="inlineStr"/>
+      <c r="L306" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="M306" t="n">
+        <v>1.75</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -13340,7 +13970,21 @@
       <c r="D307" t="n">
         <v>335.94</v>
       </c>
+      <c r="E307" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K307" t="inlineStr"/>
+      <c r="L307" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="M307" t="n">
+        <v>6.47</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -13361,7 +14005,21 @@
       <c r="D308" t="n">
         <v>187.74</v>
       </c>
+      <c r="E308" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K308" t="inlineStr"/>
+      <c r="L308" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="M308" t="n">
+        <v>3.02</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -13382,7 +14040,21 @@
       <c r="D309" t="n">
         <v>104.39</v>
       </c>
+      <c r="E309" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K309" t="inlineStr"/>
+      <c r="L309" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="M309" t="n">
+        <v>5.57</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -13403,7 +14075,21 @@
       <c r="D310" t="n">
         <v>364.62</v>
       </c>
+      <c r="E310" t="n">
+        <v>-3.92</v>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K310" t="inlineStr"/>
+      <c r="L310" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="M310" t="n">
+        <v>-1.78</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -13424,7 +14110,21 @@
       <c r="D311" t="n">
         <v>310.32</v>
       </c>
+      <c r="E311" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K311" t="inlineStr"/>
+      <c r="L311" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="M311" t="n">
+        <v>0.43</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -13445,7 +14145,21 @@
       <c r="D312" t="n">
         <v>78.94</v>
       </c>
+      <c r="E312" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K312" t="inlineStr"/>
+      <c r="L312" t="n">
+        <v>9</v>
+      </c>
+      <c r="M312" t="n">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -13466,7 +14180,21 @@
       <c r="D313" t="n">
         <v>288.7</v>
       </c>
+      <c r="E313" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K313" t="inlineStr"/>
+      <c r="L313" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M313" t="n">
+        <v>2.28</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -13487,7 +14215,21 @@
       <c r="D314" t="n">
         <v>198.88</v>
       </c>
+      <c r="E314" t="n">
+        <v>-4.51</v>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K314" t="inlineStr"/>
+      <c r="L314" t="n">
+        <v>-4.29</v>
+      </c>
+      <c r="M314" t="n">
+        <v>-2.79</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -13508,7 +14250,21 @@
       <c r="D315" t="n">
         <v>751.66</v>
       </c>
+      <c r="E315" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K315" t="inlineStr"/>
+      <c r="L315" t="n">
+        <v>-2.92</v>
+      </c>
+      <c r="M315" t="n">
+        <v>-3.03</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -13529,7 +14285,21 @@
       <c r="D316" t="n">
         <v>516.17</v>
       </c>
+      <c r="E316" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K316" t="inlineStr"/>
+      <c r="L316" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="M316" t="n">
+        <v>2.35</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -13550,7 +14320,21 @@
       <c r="D317" t="n">
         <v>1082.28</v>
       </c>
+      <c r="E317" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K317" t="inlineStr"/>
+      <c r="L317" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="M317" t="n">
+        <v>-0.26</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -13571,7 +14355,21 @@
       <c r="D318" t="n">
         <v>43.72</v>
       </c>
+      <c r="E318" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K318" t="inlineStr"/>
+      <c r="L318" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="M318" t="n">
+        <v>1.39</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -16155,6 +16953,405 @@
         <v>44.83</v>
       </c>
       <c r="K441" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>237.72</v>
+      </c>
+      <c r="K442" t="inlineStr"/>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>234.64</v>
+      </c>
+      <c r="K443" t="inlineStr"/>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>728.0700000000001</v>
+      </c>
+      <c r="K444" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>134.37</v>
+      </c>
+      <c r="K445" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="K446" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>188.79</v>
+      </c>
+      <c r="K447" t="inlineStr"/>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>184.91</v>
+      </c>
+      <c r="K448" t="inlineStr"/>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>472.9</v>
+      </c>
+      <c r="K449" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>196.56</v>
+      </c>
+      <c r="K450" t="inlineStr"/>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>333.79</v>
+      </c>
+      <c r="K451" t="inlineStr"/>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>289.23</v>
+      </c>
+      <c r="K452" t="inlineStr"/>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>562.22</v>
+      </c>
+      <c r="K453" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>184.91</v>
+      </c>
+      <c r="K454" t="inlineStr"/>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>341.02</v>
+      </c>
+      <c r="K455" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>196.56</v>
+      </c>
+      <c r="K456" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D457" t="n">
+        <v>61.39</v>
+      </c>
+      <c r="K457" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D458" t="n">
+        <v>46.92</v>
+      </c>
+      <c r="K458" t="inlineStr"/>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D459" t="n">
+        <v>122.97</v>
+      </c>
+      <c r="K459" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D460" t="n">
+        <v>25.06</v>
+      </c>
+      <c r="K460" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16328,43 +17525,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="C3" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="D3" t="n">
-        <v>46.3</v>
+        <v>45.2</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.48</v>
+        <v>-0.64</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.9</v>
+        <v>-1</v>
       </c>
       <c r="G3" t="n">
-        <v>35.8</v>
+        <v>35.6</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.76</v>
+        <v>-0.74</v>
       </c>
       <c r="I3" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="J3" t="n">
-        <v>56.6</v>
+        <v>54.1</v>
       </c>
       <c r="K3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.77</v>
+        <v>-0.82</v>
       </c>
       <c r="M3" t="n">
-        <v>50.9</v>
+        <v>47.5</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.2</v>
+        <v>-0.25</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -16377,43 +17574,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C4" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D4" t="n">
-        <v>68.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>2.68</v>
+        <v>2.44</v>
       </c>
       <c r="F4" t="n">
-        <v>2.25</v>
+        <v>2.1</v>
       </c>
       <c r="G4" t="n">
-        <v>62.5</v>
+        <v>63.6</v>
       </c>
       <c r="H4" t="n">
-        <v>2.48</v>
+        <v>2.55</v>
       </c>
       <c r="I4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J4" t="n">
-        <v>71.40000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="K4" t="n">
-        <v>5.81</v>
+        <v>5.88</v>
       </c>
       <c r="L4" t="n">
-        <v>4.88</v>
+        <v>4.96</v>
       </c>
       <c r="M4" t="n">
-        <v>68.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>5.63</v>
+        <v>5.68</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -16426,7 +17623,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" t="n">
         <v>20</v>
@@ -16447,22 +17644,22 @@
         <v>1.96</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J5" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="K5" t="n">
-        <v>3.25</v>
+        <v>3.99</v>
       </c>
       <c r="L5" t="n">
-        <v>2.6</v>
+        <v>3.22</v>
       </c>
       <c r="M5" t="n">
-        <v>60</v>
+        <v>53.3</v>
       </c>
       <c r="N5" t="n">
-        <v>2.73</v>
+        <v>2.17</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -16475,43 +17672,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D6" t="n">
-        <v>60.3</v>
+        <v>59.4</v>
       </c>
       <c r="E6" t="n">
-        <v>1.58</v>
+        <v>1.47</v>
       </c>
       <c r="F6" t="n">
-        <v>0.87</v>
+        <v>0.84</v>
       </c>
       <c r="G6" t="n">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="H6" t="n">
-        <v>1.72</v>
+        <v>1.81</v>
       </c>
       <c r="I6" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J6" t="n">
-        <v>68.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="K6" t="n">
-        <v>3.61</v>
+        <v>4.08</v>
       </c>
       <c r="L6" t="n">
-        <v>2.81</v>
+        <v>3.24</v>
       </c>
       <c r="M6" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N6" t="n">
-        <v>4.04</v>
+        <v>4.06</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -16524,43 +17721,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C7" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D7" t="n">
         <v>50</v>
       </c>
       <c r="E7" t="n">
-        <v>1.04</v>
+        <v>0.95</v>
       </c>
       <c r="F7" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="G7" t="n">
-        <v>41.9</v>
+        <v>42.4</v>
       </c>
       <c r="H7" t="n">
-        <v>1.21</v>
+        <v>1.14</v>
       </c>
       <c r="I7" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="J7" t="n">
-        <v>44.4</v>
+        <v>55.3</v>
       </c>
       <c r="K7" t="n">
-        <v>0.65</v>
+        <v>1.59</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.11</v>
+        <v>0.75</v>
       </c>
       <c r="M7" t="n">
-        <v>44.4</v>
+        <v>55.3</v>
       </c>
       <c r="N7" t="n">
-        <v>1.43</v>
+        <v>1.5</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-05
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q465"/>
+  <dimension ref="A1:Q487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10233,6 +10233,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G200" t="n">
+        <v>-2.79</v>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K200" t="inlineStr"/>
       <c r="L200" t="n">
         <v>-2.85</v>
@@ -10240,6 +10248,12 @@
       <c r="M200" t="n">
         <v>-5.99</v>
       </c>
+      <c r="N200" t="n">
+        <v>-2.97</v>
+      </c>
+      <c r="O200" t="n">
+        <v>-4.93</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -10264,6 +10278,14 @@
         <v>1.52</v>
       </c>
       <c r="F201" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="H201" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -10275,6 +10297,12 @@
       <c r="M201" t="n">
         <v>0.27</v>
       </c>
+      <c r="N201" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="O201" t="n">
+        <v>3.48</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -10299,6 +10327,14 @@
         <v>-4.52</v>
       </c>
       <c r="F202" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G202" t="n">
+        <v>-1.13</v>
+      </c>
+      <c r="H202" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10310,6 +10346,12 @@
       <c r="M202" t="n">
         <v>-7.42</v>
       </c>
+      <c r="N202" t="n">
+        <v>-1.32</v>
+      </c>
+      <c r="O202" t="n">
+        <v>-4.13</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -10336,6 +10378,14 @@
       <c r="F203" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G203" t="n">
+        <v>-1.19</v>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K203" t="inlineStr"/>
@@ -10345,6 +10395,12 @@
       <c r="M203" t="n">
         <v>3.43</v>
       </c>
+      <c r="N203" t="n">
+        <v>-1.38</v>
+      </c>
+      <c r="O203" t="n">
+        <v>-1.29</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -10369,6 +10425,14 @@
         <v>2.4</v>
       </c>
       <c r="F204" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G204" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="H204" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -10380,6 +10444,12 @@
       <c r="M204" t="n">
         <v>1.17</v>
       </c>
+      <c r="N204" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="O204" t="n">
+        <v>2.23</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -10404,6 +10474,14 @@
         <v>-3.73</v>
       </c>
       <c r="F205" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G205" t="n">
+        <v>-6.53</v>
+      </c>
+      <c r="H205" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10415,6 +10493,12 @@
       <c r="M205" t="n">
         <v>-4.5</v>
       </c>
+      <c r="N205" t="n">
+        <v>-6.72</v>
+      </c>
+      <c r="O205" t="n">
+        <v>-7.28</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -10441,6 +10525,14 @@
       <c r="F206" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G206" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K206" t="inlineStr"/>
@@ -10450,6 +10542,12 @@
       <c r="M206" t="n">
         <v>-10.83</v>
       </c>
+      <c r="N206" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="O206" t="n">
+        <v>-1.74</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -10474,6 +10572,14 @@
         <v>-3.74</v>
       </c>
       <c r="F207" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G207" t="n">
+        <v>-2.51</v>
+      </c>
+      <c r="H207" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10485,6 +10591,12 @@
       <c r="M207" t="n">
         <v>-5.16</v>
       </c>
+      <c r="N207" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="O207" t="n">
+        <v>-3.94</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -10511,6 +10623,14 @@
       <c r="F208" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G208" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K208" t="inlineStr"/>
@@ -10520,6 +10640,12 @@
       <c r="M208" t="n">
         <v>-3.69</v>
       </c>
+      <c r="N208" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O208" t="n">
+        <v>1.25</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -10546,6 +10672,14 @@
       <c r="F209" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G209" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K209" t="inlineStr"/>
@@ -10555,6 +10689,12 @@
       <c r="M209" t="n">
         <v>-2.74</v>
       </c>
+      <c r="N209" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O209" t="n">
+        <v>1.29</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -10579,6 +10719,14 @@
         <v>0.65</v>
       </c>
       <c r="F210" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G210" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="H210" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -10590,6 +10738,12 @@
       <c r="M210" t="n">
         <v>0.79</v>
       </c>
+      <c r="N210" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="O210" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -10616,6 +10770,14 @@
       <c r="F211" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G211" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K211" t="inlineStr"/>
@@ -10625,6 +10787,12 @@
       <c r="M211" t="n">
         <v>0.11</v>
       </c>
+      <c r="N211" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="O211" t="n">
+        <v>4.08</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -10649,6 +10817,14 @@
         <v>-12.25</v>
       </c>
       <c r="F212" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G212" t="n">
+        <v>-6.15</v>
+      </c>
+      <c r="H212" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10660,6 +10836,12 @@
       <c r="M212" t="n">
         <v>-11.4</v>
       </c>
+      <c r="N212" t="n">
+        <v>-6.34</v>
+      </c>
+      <c r="O212" t="n">
+        <v>-5.23</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -10686,6 +10868,14 @@
       <c r="F213" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G213" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K213" t="inlineStr"/>
@@ -10695,6 +10885,12 @@
       <c r="M213" t="n">
         <v>-0.85</v>
       </c>
+      <c r="N213" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="O213" t="n">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -10719,6 +10915,14 @@
         <v>-4.72</v>
       </c>
       <c r="F214" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G214" t="n">
+        <v>-4.52</v>
+      </c>
+      <c r="H214" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10730,6 +10934,12 @@
       <c r="M214" t="n">
         <v>-3.53</v>
       </c>
+      <c r="N214" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="O214" t="n">
+        <v>-3.32</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -10756,6 +10966,14 @@
       <c r="F215" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G215" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K215" t="inlineStr"/>
@@ -10765,6 +10983,12 @@
       <c r="M215" t="n">
         <v>-2.26</v>
       </c>
+      <c r="N215" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="O215" t="n">
+        <v>1.38</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -10789,6 +11013,14 @@
         <v>3.1</v>
       </c>
       <c r="F216" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G216" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="H216" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -10800,6 +11032,12 @@
       <c r="M216" t="n">
         <v>4.77</v>
       </c>
+      <c r="N216" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="O216" t="n">
+        <v>8.1</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -10826,6 +11064,14 @@
       <c r="F217" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G217" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K217" t="inlineStr"/>
@@ -10835,6 +11081,12 @@
       <c r="M217" t="n">
         <v>0.11</v>
       </c>
+      <c r="N217" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="O217" t="n">
+        <v>4.08</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -10859,6 +11111,14 @@
         <v>-12.25</v>
       </c>
       <c r="F218" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G218" t="n">
+        <v>-6.15</v>
+      </c>
+      <c r="H218" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10870,6 +11130,12 @@
       <c r="M218" t="n">
         <v>-11.4</v>
       </c>
+      <c r="N218" t="n">
+        <v>-6.34</v>
+      </c>
+      <c r="O218" t="n">
+        <v>-5.23</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -10896,6 +11162,14 @@
       <c r="F219" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G219" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K219" t="inlineStr"/>
@@ -10905,6 +11179,12 @@
       <c r="M219" t="n">
         <v>-3.98</v>
       </c>
+      <c r="N219" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="O219" t="n">
+        <v>13.05</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -10929,6 +11209,14 @@
         <v>-4.72</v>
       </c>
       <c r="F220" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G220" t="n">
+        <v>-4.52</v>
+      </c>
+      <c r="H220" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -10940,6 +11228,12 @@
       <c r="M220" t="n">
         <v>-3.53</v>
       </c>
+      <c r="N220" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="O220" t="n">
+        <v>-3.32</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -10966,6 +11260,14 @@
       <c r="F221" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G221" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K221" t="inlineStr"/>
@@ -10975,6 +11277,12 @@
       <c r="M221" t="n">
         <v>-2.26</v>
       </c>
+      <c r="N221" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="O221" t="n">
+        <v>1.38</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -10999,6 +11307,14 @@
         <v>-11.43</v>
       </c>
       <c r="F222" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G222" t="n">
+        <v>-17.94</v>
+      </c>
+      <c r="H222" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -11010,6 +11326,12 @@
       <c r="M222" t="n">
         <v>-9.66</v>
       </c>
+      <c r="N222" t="n">
+        <v>-18.12</v>
+      </c>
+      <c r="O222" t="n">
+        <v>-16.31</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -11036,6 +11358,14 @@
       <c r="F223" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G223" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K223" t="inlineStr"/>
@@ -11045,6 +11375,12 @@
       <c r="M223" t="n">
         <v>-9.07</v>
       </c>
+      <c r="N223" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="O223" t="n">
+        <v>7.45</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -11069,6 +11405,14 @@
         <v>3.97</v>
       </c>
       <c r="F224" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G224" t="n">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="H224" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -11080,6 +11424,12 @@
       <c r="M224" t="n">
         <v>4.35</v>
       </c>
+      <c r="N224" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="O224" t="n">
+        <v>9.789999999999999</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -11106,6 +11456,14 @@
       <c r="F225" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G225" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K225" t="inlineStr"/>
@@ -11115,6 +11473,12 @@
       <c r="M225" t="n">
         <v>-1.93</v>
       </c>
+      <c r="N225" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="O225" t="n">
+        <v>1.25</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -11141,6 +11505,14 @@
       <c r="F226" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G226" t="n">
+        <v>14.47</v>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K226" t="inlineStr"/>
@@ -11150,6 +11522,12 @@
       <c r="M226" t="n">
         <v>-1.79</v>
       </c>
+      <c r="N226" t="n">
+        <v>14.28</v>
+      </c>
+      <c r="O226" t="n">
+        <v>16.49</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -11174,6 +11552,14 @@
         <v>14.07</v>
       </c>
       <c r="F227" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H227" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -11185,6 +11571,12 @@
       <c r="M227" t="n">
         <v>16.98</v>
       </c>
+      <c r="N227" t="n">
+        <v>17.32</v>
+      </c>
+      <c r="O227" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -11209,6 +11601,14 @@
         <v>0.96</v>
       </c>
       <c r="F228" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H228" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -11220,6 +11620,12 @@
       <c r="M228" t="n">
         <v>1.95</v>
       </c>
+      <c r="N228" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="O228" t="n">
+        <v>2.89</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -11244,6 +11650,14 @@
         <v>0.66</v>
       </c>
       <c r="F229" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="H229" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -11255,6 +11669,12 @@
       <c r="M229" t="n">
         <v>0.33</v>
       </c>
+      <c r="N229" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="O229" t="n">
+        <v>1.93</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -11279,6 +11699,14 @@
         <v>-7.5</v>
       </c>
       <c r="F230" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>-6.67</v>
+      </c>
+      <c r="H230" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -11290,6 +11718,12 @@
       <c r="M230" t="n">
         <v>-4.27</v>
       </c>
+      <c r="N230" t="n">
+        <v>-6.86</v>
+      </c>
+      <c r="O230" t="n">
+        <v>-3.41</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -11316,6 +11750,14 @@
       <c r="F231" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K231" t="inlineStr"/>
@@ -11325,6 +11767,12 @@
       <c r="M231" t="n">
         <v>-6.02</v>
       </c>
+      <c r="N231" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="O231" t="n">
+        <v>5.11</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -13194,26 +13642,26 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>127.39</v>
+        <v>8.73</v>
       </c>
       <c r="E285" t="n">
-        <v>-5.8</v>
+        <v>5.15</v>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="K285" t="inlineStr"/>
       <c r="L285" t="n">
-        <v>-5.39</v>
+        <v>5.57</v>
       </c>
       <c r="M285" t="n">
-        <v>-5.49</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="286">
@@ -13224,31 +13672,31 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>8.73</v>
+        <v>127.39</v>
       </c>
       <c r="E286" t="n">
-        <v>5.15</v>
+        <v>-5.8</v>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K286" t="inlineStr"/>
       <c r="L286" t="n">
-        <v>5.57</v>
+        <v>-5.39</v>
       </c>
       <c r="M286" t="n">
-        <v>4.81</v>
+        <v>-5.49</v>
       </c>
     </row>
     <row r="287">
@@ -14390,7 +14838,21 @@
       <c r="D319" t="n">
         <v>231.01</v>
       </c>
+      <c r="E319" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K319" t="inlineStr"/>
+      <c r="L319" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="M319" t="n">
+        <v>3.29</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -14411,7 +14873,21 @@
       <c r="D320" t="n">
         <v>227.27</v>
       </c>
+      <c r="E320" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K320" t="inlineStr"/>
+      <c r="L320" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="M320" t="n">
+        <v>1.03</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -14432,7 +14908,21 @@
       <c r="D321" t="n">
         <v>715.62</v>
       </c>
+      <c r="E321" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K321" t="inlineStr"/>
+      <c r="L321" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="M321" t="n">
+        <v>2.27</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -14453,7 +14943,21 @@
       <c r="D322" t="n">
         <v>509.22</v>
       </c>
+      <c r="E322" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K322" t="inlineStr"/>
+      <c r="L322" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="M322" t="n">
+        <v>3.28</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -14474,7 +14978,21 @@
       <c r="D323" t="n">
         <v>131.45</v>
       </c>
+      <c r="E323" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K323" t="inlineStr"/>
+      <c r="L323" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="M323" t="n">
+        <v>3.94</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -14495,7 +15013,21 @@
       <c r="D324" t="n">
         <v>28.72</v>
       </c>
+      <c r="E324" t="n">
+        <v>-4.56</v>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K324" t="inlineStr"/>
+      <c r="L324" t="n">
+        <v>-5.78</v>
+      </c>
+      <c r="M324" t="n">
+        <v>-4.26</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -14516,7 +15048,21 @@
       <c r="D325" t="n">
         <v>187.48</v>
       </c>
+      <c r="E325" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K325" t="inlineStr"/>
+      <c r="L325" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="M325" t="n">
+        <v>1.02</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -14537,7 +15083,21 @@
       <c r="D326" t="n">
         <v>187.48</v>
       </c>
+      <c r="E326" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K326" t="inlineStr"/>
+      <c r="L326" t="n">
+        <v>-4.76</v>
+      </c>
+      <c r="M326" t="n">
+        <v>-4.66</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -14558,7 +15118,21 @@
       <c r="D327" t="n">
         <v>497.51</v>
       </c>
+      <c r="E327" t="n">
+        <v>-2.91</v>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K327" t="inlineStr"/>
+      <c r="L327" t="n">
+        <v>-4.13</v>
+      </c>
+      <c r="M327" t="n">
+        <v>-3.45</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -14579,7 +15153,21 @@
       <c r="D328" t="n">
         <v>199.39</v>
       </c>
+      <c r="E328" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K328" t="inlineStr"/>
+      <c r="L328" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M328" t="n">
+        <v>1.88</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -14600,7 +15188,21 @@
       <c r="D329" t="n">
         <v>73.67</v>
       </c>
+      <c r="E329" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K329" t="inlineStr"/>
+      <c r="L329" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="M329" t="n">
+        <v>13.05</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -14621,7 +15223,21 @@
       <c r="D330" t="n">
         <v>262.87</v>
       </c>
+      <c r="E330" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K330" t="inlineStr"/>
+      <c r="L330" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="M330" t="n">
+        <v>4.98</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -14642,7 +15258,21 @@
       <c r="D331" t="n">
         <v>116.46</v>
       </c>
+      <c r="E331" t="n">
+        <v>-1.99</v>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K331" t="inlineStr"/>
+      <c r="L331" t="n">
+        <v>-3.21</v>
+      </c>
+      <c r="M331" t="n">
+        <v>-4.05</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -14663,7 +15293,21 @@
       <c r="D332" t="n">
         <v>105.43</v>
       </c>
+      <c r="E332" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K332" t="inlineStr"/>
+      <c r="L332" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="M332" t="n">
+        <v>4.64</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -14684,7 +15328,21 @@
       <c r="D333" t="n">
         <v>131.45</v>
       </c>
+      <c r="E333" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K333" t="inlineStr"/>
+      <c r="L333" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="M333" t="n">
+        <v>3.94</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -14705,7 +15363,21 @@
       <c r="D334" t="n">
         <v>187.48</v>
       </c>
+      <c r="E334" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K334" t="inlineStr"/>
+      <c r="L334" t="n">
+        <v>-4.76</v>
+      </c>
+      <c r="M334" t="n">
+        <v>-4.66</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -14726,7 +15398,21 @@
       <c r="D335" t="n">
         <v>1712.89</v>
       </c>
+      <c r="E335" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K335" t="inlineStr"/>
+      <c r="L335" t="n">
+        <v>-1.73</v>
+      </c>
+      <c r="M335" t="n">
+        <v>-2.39</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -14747,7 +15433,21 @@
       <c r="D336" t="n">
         <v>178.54</v>
       </c>
+      <c r="E336" t="n">
+        <v>10.19</v>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K336" t="inlineStr"/>
+      <c r="L336" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="M336" t="n">
+        <v>10.59</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -14768,7 +15468,21 @@
       <c r="D337" t="n">
         <v>8.800000000000001</v>
       </c>
+      <c r="E337" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K337" t="inlineStr"/>
+      <c r="L337" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="M337" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -14789,7 +15503,21 @@
       <c r="D338" t="n">
         <v>98.48999999999999</v>
       </c>
+      <c r="E338" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K338" t="inlineStr"/>
+      <c r="L338" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="M338" t="n">
+        <v>2.37</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -14810,7 +15538,21 @@
       <c r="D339" t="n">
         <v>351.31</v>
       </c>
+      <c r="E339" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K339" t="inlineStr"/>
+      <c r="L339" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="M339" t="n">
+        <v>2.82</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -14831,7 +15573,21 @@
       <c r="D340" t="n">
         <v>8.800000000000001</v>
       </c>
+      <c r="E340" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K340" t="inlineStr"/>
+      <c r="L340" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="M340" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -14852,7 +15608,21 @@
       <c r="D341" t="n">
         <v>197.28</v>
       </c>
+      <c r="E341" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K341" t="inlineStr"/>
+      <c r="L341" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="M341" t="n">
+        <v>2.65</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -14873,7 +15643,21 @@
       <c r="D342" t="n">
         <v>1053.98</v>
       </c>
+      <c r="E342" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K342" t="inlineStr"/>
+      <c r="L342" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="M342" t="n">
+        <v>-1.3</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -14894,7 +15678,21 @@
       <c r="D343" t="n">
         <v>40.9</v>
       </c>
+      <c r="E343" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K343" t="inlineStr"/>
+      <c r="L343" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="M343" t="n">
+        <v>4.97</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -14915,7 +15713,21 @@
       <c r="D344" t="n">
         <v>600.01</v>
       </c>
+      <c r="E344" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K344" t="inlineStr"/>
+      <c r="L344" t="n">
+        <v>4.46</v>
+      </c>
+      <c r="M344" t="n">
+        <v>4.02</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -14936,7 +15748,21 @@
       <c r="D345" t="n">
         <v>921.51</v>
       </c>
+      <c r="E345" t="n">
+        <v>-3.76</v>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K345" t="inlineStr"/>
+      <c r="L345" t="n">
+        <v>-4.98</v>
+      </c>
+      <c r="M345" t="n">
+        <v>-6.1</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -14957,7 +15783,21 @@
       <c r="D346" t="n">
         <v>40.87</v>
       </c>
+      <c r="E346" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K346" t="inlineStr"/>
+      <c r="L346" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="M346" t="n">
+        <v>11.9</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -15560,11 +16400,11 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>263.27</v>
+        <v>203.46</v>
       </c>
       <c r="K375" t="inlineStr"/>
     </row>
@@ -15576,16 +16416,16 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>149.42</v>
+        <v>263.27</v>
       </c>
       <c r="K376" t="inlineStr"/>
     </row>
@@ -15602,11 +16442,11 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>196.53</v>
+        <v>149.42</v>
       </c>
       <c r="K377" t="inlineStr"/>
     </row>
@@ -15623,11 +16463,11 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>203.46</v>
+        <v>196.53</v>
       </c>
       <c r="K378" t="inlineStr"/>
     </row>
@@ -16316,11 +17156,11 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>235.88</v>
+        <v>512.9</v>
       </c>
       <c r="K411" t="inlineStr"/>
     </row>
@@ -16337,11 +17177,11 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>307.82</v>
+        <v>235.88</v>
       </c>
       <c r="K412" t="inlineStr"/>
     </row>
@@ -16358,32 +17198,32 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>40.34</v>
+        <v>307.82</v>
       </c>
       <c r="K413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Golden Cross</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>241.28</v>
+        <v>40.34</v>
       </c>
       <c r="K414" t="inlineStr"/>
     </row>
@@ -16400,11 +17240,11 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>236.69</v>
+        <v>241.28</v>
       </c>
       <c r="K415" t="inlineStr"/>
     </row>
@@ -16421,11 +17261,11 @@
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D416" t="n">
-        <v>725.9299999999999</v>
+        <v>236.69</v>
       </c>
       <c r="K416" t="inlineStr"/>
     </row>
@@ -16442,11 +17282,11 @@
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>137.76</v>
+        <v>725.9299999999999</v>
       </c>
       <c r="K417" t="inlineStr"/>
     </row>
@@ -16463,11 +17303,11 @@
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>28.12</v>
+        <v>137.76</v>
       </c>
       <c r="K418" t="inlineStr"/>
     </row>
@@ -16484,11 +17324,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>190.04</v>
+        <v>28.12</v>
       </c>
       <c r="K419" t="inlineStr"/>
     </row>
@@ -16505,11 +17345,11 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>182.09</v>
+        <v>190.04</v>
       </c>
       <c r="K420" t="inlineStr"/>
     </row>
@@ -16526,11 +17366,11 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>SPOT</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>491.4</v>
+        <v>182.09</v>
       </c>
       <c r="K421" t="inlineStr"/>
     </row>
@@ -16547,11 +17387,11 @@
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>SPOT</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>198.78</v>
+        <v>491.4</v>
       </c>
       <c r="K422" t="inlineStr"/>
     </row>
@@ -16563,16 +17403,16 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Bull Flag Watch</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>330.32</v>
+        <v>198.78</v>
       </c>
       <c r="K423" t="inlineStr"/>
     </row>
@@ -16589,11 +17429,11 @@
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>101.6</v>
+        <v>330.32</v>
       </c>
       <c r="K424" t="inlineStr"/>
     </row>
@@ -16610,11 +17450,11 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>277.58</v>
+        <v>101.6</v>
       </c>
       <c r="K425" t="inlineStr"/>
     </row>
@@ -16631,11 +17471,11 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="D426" t="n">
-        <v>236.69</v>
+        <v>277.58</v>
       </c>
       <c r="K426" t="inlineStr"/>
     </row>
@@ -16652,11 +17492,11 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>541.74</v>
+        <v>236.69</v>
       </c>
       <c r="K427" t="inlineStr"/>
     </row>
@@ -16673,11 +17513,11 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>160.42</v>
+        <v>541.74</v>
       </c>
       <c r="K428" t="inlineStr"/>
     </row>
@@ -16694,11 +17534,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>10.37</v>
+        <v>160.42</v>
       </c>
       <c r="K429" t="inlineStr"/>
     </row>
@@ -16715,11 +17555,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>137.76</v>
+        <v>10.37</v>
       </c>
       <c r="K430" t="inlineStr"/>
     </row>
@@ -16736,11 +17576,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>182.09</v>
+        <v>137.76</v>
       </c>
       <c r="K431" t="inlineStr"/>
     </row>
@@ -16757,11 +17597,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>1787.69</v>
+        <v>182.09</v>
       </c>
       <c r="K432" t="inlineStr"/>
     </row>
@@ -16773,16 +17613,16 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Breakout Watch (EOD)</t>
+          <t>Bull Flag Watch</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="D433" t="n">
-        <v>319.19</v>
+        <v>1787.69</v>
       </c>
       <c r="K433" t="inlineStr"/>
     </row>
@@ -16799,11 +17639,11 @@
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>FOTO</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="D434" t="n">
-        <v>19.24</v>
+        <v>319.19</v>
       </c>
       <c r="K434" t="inlineStr"/>
     </row>
@@ -16815,16 +17655,16 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Breakout Watch (EOD)</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>FOTO</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>101.6</v>
+        <v>19.24</v>
       </c>
       <c r="K435" t="inlineStr"/>
     </row>
@@ -16841,11 +17681,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>AXTI</t>
+          <t>AEHR</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>81.81</v>
+        <v>101.6</v>
       </c>
       <c r="K436" t="inlineStr"/>
     </row>
@@ -16862,11 +17702,11 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>FOTO</t>
+          <t>AXTI</t>
         </is>
       </c>
       <c r="D437" t="n">
-        <v>19.24</v>
+        <v>81.81</v>
       </c>
       <c r="K437" t="inlineStr"/>
     </row>
@@ -16883,11 +17723,11 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>FOTO</t>
         </is>
       </c>
       <c r="D438" t="n">
-        <v>1045.78</v>
+        <v>19.24</v>
       </c>
       <c r="K438" t="inlineStr"/>
     </row>
@@ -16904,11 +17744,11 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D439" t="n">
-        <v>1097.39</v>
+        <v>1045.78</v>
       </c>
       <c r="K439" t="inlineStr"/>
     </row>
@@ -17030,11 +17870,11 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>VIAV</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="D445" t="n">
-        <v>44.78</v>
+        <v>1787.69</v>
       </c>
       <c r="K445" t="inlineStr"/>
     </row>
@@ -17051,32 +17891,32 @@
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>ZETA</t>
+          <t>VIAV</t>
         </is>
       </c>
       <c r="D446" t="n">
-        <v>32.4</v>
+        <v>44.78</v>
       </c>
       <c r="K446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>Golden Cross</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ZETA</t>
         </is>
       </c>
       <c r="D447" t="n">
-        <v>237.72</v>
+        <v>32.4</v>
       </c>
       <c r="K447" t="inlineStr"/>
     </row>
@@ -17093,11 +17933,11 @@
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="D448" t="n">
-        <v>234.64</v>
+        <v>237.72</v>
       </c>
       <c r="K448" t="inlineStr"/>
     </row>
@@ -17114,11 +17954,11 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>728.0700000000001</v>
+        <v>234.64</v>
       </c>
       <c r="K449" t="inlineStr"/>
     </row>
@@ -17135,11 +17975,11 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D450" t="n">
-        <v>134.37</v>
+        <v>728.0700000000001</v>
       </c>
       <c r="K450" t="inlineStr"/>
     </row>
@@ -17156,11 +17996,11 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>PFE</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>27.8</v>
+        <v>134.37</v>
       </c>
       <c r="K451" t="inlineStr"/>
     </row>
@@ -17177,11 +18017,11 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="D452" t="n">
-        <v>188.79</v>
+        <v>27.8</v>
       </c>
       <c r="K452" t="inlineStr"/>
     </row>
@@ -17198,11 +18038,11 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D453" t="n">
-        <v>184.91</v>
+        <v>188.79</v>
       </c>
       <c r="K453" t="inlineStr"/>
     </row>
@@ -17219,11 +18059,11 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>SPOT</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D454" t="n">
-        <v>472.9</v>
+        <v>184.91</v>
       </c>
       <c r="K454" t="inlineStr"/>
     </row>
@@ -17240,11 +18080,11 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>SPOT</t>
         </is>
       </c>
       <c r="D455" t="n">
-        <v>196.56</v>
+        <v>472.9</v>
       </c>
       <c r="K455" t="inlineStr"/>
     </row>
@@ -17256,16 +18096,16 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Bull Flag Watch</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="D456" t="n">
-        <v>333.79</v>
+        <v>196.56</v>
       </c>
       <c r="K456" t="inlineStr"/>
     </row>
@@ -17282,11 +18122,11 @@
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D457" t="n">
-        <v>289.23</v>
+        <v>333.79</v>
       </c>
       <c r="K457" t="inlineStr"/>
     </row>
@@ -17303,11 +18143,11 @@
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="D458" t="n">
-        <v>562.22</v>
+        <v>289.23</v>
       </c>
       <c r="K458" t="inlineStr"/>
     </row>
@@ -17324,11 +18164,11 @@
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="D459" t="n">
-        <v>184.91</v>
+        <v>562.22</v>
       </c>
       <c r="K459" t="inlineStr"/>
     </row>
@@ -17345,11 +18185,11 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D460" t="n">
-        <v>341.02</v>
+        <v>184.91</v>
       </c>
       <c r="K460" t="inlineStr"/>
     </row>
@@ -17366,11 +18206,11 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="D461" t="n">
-        <v>196.56</v>
+        <v>341.02</v>
       </c>
       <c r="K461" t="inlineStr"/>
     </row>
@@ -17382,16 +18222,16 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>Breakout Watch (EOD)</t>
+          <t>Bull Flag Watch</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="D462" t="n">
-        <v>61.39</v>
+        <v>196.56</v>
       </c>
       <c r="K462" t="inlineStr"/>
     </row>
@@ -17403,16 +18243,16 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Breakout Watch (EOD)</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>BUG</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D463" t="n">
-        <v>46.92</v>
+        <v>61.39</v>
       </c>
       <c r="K463" t="inlineStr"/>
     </row>
@@ -17429,11 +18269,11 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>HACK</t>
+          <t>BUG</t>
         </is>
       </c>
       <c r="D464" t="n">
-        <v>122.97</v>
+        <v>46.92</v>
       </c>
       <c r="K464" t="inlineStr"/>
     </row>
@@ -17445,18 +18285,480 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>122.97</v>
+      </c>
+      <c r="K465" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
           <t>Performance: Buy</t>
         </is>
       </c>
-      <c r="C465" t="inlineStr">
+      <c r="C466" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D465" t="n">
+      <c r="D466" t="n">
         <v>25.06</v>
       </c>
-      <c r="K465" t="inlineStr"/>
+      <c r="K466" t="inlineStr"/>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>238.81</v>
+      </c>
+      <c r="K467" t="inlineStr"/>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>229.83</v>
+      </c>
+      <c r="K468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>742.1900000000001</v>
+      </c>
+      <c r="K469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>136.12</v>
+      </c>
+      <c r="K470" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>27.41</v>
+      </c>
+      <c r="K471" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>189.43</v>
+      </c>
+      <c r="K472" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>180.84</v>
+      </c>
+      <c r="K473" t="inlineStr"/>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>483.01</v>
+      </c>
+      <c r="K474" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>201.94</v>
+      </c>
+      <c r="K475" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D476" t="n">
+        <v>333.13</v>
+      </c>
+      <c r="K476" t="inlineStr"/>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>286.68</v>
+      </c>
+      <c r="K477" t="inlineStr"/>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>552.22</v>
+      </c>
+      <c r="K478" t="inlineStr"/>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>10.21</v>
+      </c>
+      <c r="K479" t="inlineStr"/>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>136.12</v>
+      </c>
+      <c r="K480" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>180.84</v>
+      </c>
+      <c r="K481" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D482" t="n">
+        <v>201.94</v>
+      </c>
+      <c r="K482" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>BOT</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>31.79</v>
+      </c>
+      <c r="K483" t="inlineStr"/>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>47.76</v>
+      </c>
+      <c r="K484" t="inlineStr"/>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>BOT</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>31.79</v>
+      </c>
+      <c r="K485" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>124.91</v>
+      </c>
+      <c r="K486" t="inlineStr"/>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>25.43</v>
+      </c>
+      <c r="K487" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17630,43 +18932,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C3" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="D3" t="n">
-        <v>44.2</v>
+        <v>46.5</v>
       </c>
       <c r="E3" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.97</v>
+      </c>
+      <c r="G3" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="H3" t="n">
         <v>-0.64</v>
       </c>
-      <c r="F3" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-0.74</v>
-      </c>
       <c r="I3" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="J3" t="n">
-        <v>54.1</v>
+        <v>52.2</v>
       </c>
       <c r="K3" t="n">
-        <v>0.04</v>
+        <v>-0.04</v>
       </c>
       <c r="L3" t="n">
         <v>-0.82</v>
       </c>
       <c r="M3" t="n">
-        <v>47.5</v>
+        <v>46.4</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.25</v>
+        <v>-0.48</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -17679,43 +18981,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C4" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="D4" t="n">
-        <v>69.09999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="E4" t="n">
-        <v>2.44</v>
+        <v>2.75</v>
       </c>
       <c r="F4" t="n">
-        <v>2.1</v>
+        <v>2.29</v>
       </c>
       <c r="G4" t="n">
-        <v>63.6</v>
+        <v>63.5</v>
       </c>
       <c r="H4" t="n">
-        <v>2.54</v>
+        <v>2.64</v>
       </c>
       <c r="I4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="J4" t="n">
-        <v>72.2</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="K4" t="n">
-        <v>5.88</v>
+        <v>5.63</v>
       </c>
       <c r="L4" t="n">
-        <v>4.96</v>
+        <v>4.76</v>
       </c>
       <c r="M4" t="n">
-        <v>69.40000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="N4" t="n">
-        <v>5.68</v>
+        <v>5.44</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -17728,43 +19030,43 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" t="n">
+        <v>21</v>
+      </c>
+      <c r="D5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="G5" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="I5" t="n">
         <v>20</v>
-      </c>
-      <c r="D5" t="n">
-        <v>65</v>
-      </c>
-      <c r="E5" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="G5" t="n">
-        <v>65</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="I5" t="n">
-        <v>15</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
       </c>
       <c r="K5" t="n">
-        <v>3.99</v>
+        <v>2.72</v>
       </c>
       <c r="L5" t="n">
-        <v>3.21</v>
+        <v>2.09</v>
       </c>
       <c r="M5" t="n">
-        <v>53.3</v>
+        <v>50</v>
       </c>
       <c r="N5" t="n">
-        <v>2.17</v>
+        <v>1.57</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -17777,43 +19079,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C6" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D6" t="n">
-        <v>59.4</v>
+        <v>62.3</v>
       </c>
       <c r="E6" t="n">
-        <v>1.47</v>
+        <v>1.66</v>
       </c>
       <c r="F6" t="n">
-        <v>0.85</v>
+        <v>1.02</v>
       </c>
       <c r="G6" t="n">
-        <v>51.6</v>
+        <v>55.1</v>
       </c>
       <c r="H6" t="n">
-        <v>1.81</v>
+        <v>1.9</v>
       </c>
       <c r="I6" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="J6" t="n">
-        <v>68.3</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>4.08</v>
+        <v>3.71</v>
       </c>
       <c r="L6" t="n">
-        <v>3.24</v>
+        <v>2.95</v>
       </c>
       <c r="M6" t="n">
-        <v>61</v>
+        <v>59.6</v>
       </c>
       <c r="N6" t="n">
-        <v>4.06</v>
+        <v>3.92</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -17826,43 +19128,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C7" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>51.4</v>
       </c>
       <c r="E7" t="n">
-        <v>0.95</v>
+        <v>1.19</v>
       </c>
       <c r="F7" t="n">
-        <v>0.55</v>
+        <v>0.72</v>
       </c>
       <c r="G7" t="n">
-        <v>42.4</v>
+        <v>42.9</v>
       </c>
       <c r="H7" t="n">
-        <v>1.15</v>
+        <v>1.21</v>
       </c>
       <c r="I7" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="J7" t="n">
-        <v>55.3</v>
+        <v>60.4</v>
       </c>
       <c r="K7" t="n">
-        <v>1.59</v>
+        <v>1.92</v>
       </c>
       <c r="L7" t="n">
-        <v>0.75</v>
+        <v>1.21</v>
       </c>
       <c r="M7" t="n">
-        <v>55.3</v>
+        <v>58.3</v>
       </c>
       <c r="N7" t="n">
-        <v>1.5</v>
+        <v>2.14</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-06
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q492"/>
+  <dimension ref="A1:Q522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11850,6 +11850,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G233" t="n">
+        <v>-2.56</v>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K233" t="inlineStr"/>
       <c r="L233" t="n">
         <v>-0.29</v>
@@ -11857,6 +11865,12 @@
       <c r="M233" t="n">
         <v>-0.88</v>
       </c>
+      <c r="N233" t="n">
+        <v>-3.31</v>
+      </c>
+      <c r="O233" t="n">
+        <v>-1.97</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -11881,6 +11895,14 @@
         <v>-3.42</v>
       </c>
       <c r="F234" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>-3.56</v>
+      </c>
+      <c r="H234" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -11892,6 +11914,12 @@
       <c r="M234" t="n">
         <v>-3.99</v>
       </c>
+      <c r="N234" t="n">
+        <v>-4.31</v>
+      </c>
+      <c r="O234" t="n">
+        <v>-4.13</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -11916,6 +11944,14 @@
         <v>2.2</v>
       </c>
       <c r="F235" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="H235" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -11927,6 +11963,12 @@
       <c r="M235" t="n">
         <v>1.54</v>
       </c>
+      <c r="N235" t="n">
+        <v>5.58</v>
+      </c>
+      <c r="O235" t="n">
+        <v>5.64</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -11953,6 +11995,14 @@
       <c r="F236" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G236" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K236" t="inlineStr"/>
@@ -11962,6 +12012,12 @@
       <c r="M236" t="n">
         <v>-5.41</v>
       </c>
+      <c r="N236" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0.46</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -11988,6 +12044,14 @@
       <c r="F237" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G237" t="n">
+        <v>-1.59</v>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K237" t="inlineStr"/>
@@ -11997,6 +12061,12 @@
       <c r="M237" t="n">
         <v>2.62</v>
       </c>
+      <c r="N237" t="n">
+        <v>-2.34</v>
+      </c>
+      <c r="O237" t="n">
+        <v>-1.8</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -12021,6 +12091,14 @@
         <v>1.07</v>
       </c>
       <c r="F238" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G238" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="H238" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -12032,6 +12110,12 @@
       <c r="M238" t="n">
         <v>0.27</v>
       </c>
+      <c r="N238" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="O238" t="n">
+        <v>3.01</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -12056,6 +12140,14 @@
         <v>-7.15</v>
       </c>
       <c r="F239" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>-8.69</v>
+      </c>
+      <c r="H239" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -12067,6 +12159,12 @@
       <c r="M239" t="n">
         <v>-7.87</v>
       </c>
+      <c r="N239" t="n">
+        <v>-9.43</v>
+      </c>
+      <c r="O239" t="n">
+        <v>-9.4</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -12091,6 +12189,14 @@
         <v>-1.52</v>
       </c>
       <c r="F240" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G240" t="n">
+        <v>-2.64</v>
+      </c>
+      <c r="H240" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -12102,6 +12208,12 @@
       <c r="M240" t="n">
         <v>-1.61</v>
       </c>
+      <c r="N240" t="n">
+        <v>-3.39</v>
+      </c>
+      <c r="O240" t="n">
+        <v>-2.73</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -12128,6 +12240,14 @@
       <c r="F241" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G241" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K241" t="inlineStr"/>
@@ -12137,6 +12257,12 @@
       <c r="M241" t="n">
         <v>-7.5</v>
       </c>
+      <c r="N241" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="O241" t="n">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -12163,6 +12289,14 @@
       <c r="F242" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G242" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K242" t="inlineStr"/>
@@ -12172,6 +12306,12 @@
       <c r="M242" t="n">
         <v>-6.98</v>
       </c>
+      <c r="N242" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="O242" t="n">
+        <v>-0.38</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -12198,6 +12338,14 @@
       <c r="F243" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G243" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K243" t="inlineStr"/>
@@ -12207,6 +12355,12 @@
       <c r="M243" t="n">
         <v>-1.01</v>
       </c>
+      <c r="N243" t="n">
+        <v>5.08</v>
+      </c>
+      <c r="O243" t="n">
+        <v>5.41</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -12233,6 +12387,14 @@
       <c r="F244" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G244" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K244" t="inlineStr"/>
@@ -12242,6 +12404,12 @@
       <c r="M244" t="n">
         <v>-1.82</v>
       </c>
+      <c r="N244" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="O244" t="n">
+        <v>3.68</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -12268,6 +12436,14 @@
       <c r="F245" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G245" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K245" t="inlineStr"/>
@@ -12277,6 +12453,12 @@
       <c r="M245" t="n">
         <v>-1.88</v>
       </c>
+      <c r="N245" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="O245" t="n">
+        <v>6.92</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -12303,6 +12485,14 @@
       <c r="F246" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G246" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K246" t="inlineStr"/>
@@ -12312,6 +12502,12 @@
       <c r="M246" t="n">
         <v>-2.34</v>
       </c>
+      <c r="N246" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="O246" t="n">
+        <v>4.41</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -12336,6 +12532,14 @@
         <v>-11.86</v>
       </c>
       <c r="F247" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G247" t="n">
+        <v>-9.16</v>
+      </c>
+      <c r="H247" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -12347,6 +12551,12 @@
       <c r="M247" t="n">
         <v>-11.59</v>
       </c>
+      <c r="N247" t="n">
+        <v>-9.9</v>
+      </c>
+      <c r="O247" t="n">
+        <v>-8.869999999999999</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -12371,6 +12581,14 @@
         <v>1.16</v>
       </c>
       <c r="F248" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G248" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="H248" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -12382,6 +12600,12 @@
       <c r="M248" t="n">
         <v>1.3</v>
       </c>
+      <c r="N248" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="O248" t="n">
+        <v>11.35</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -12406,6 +12630,14 @@
         <v>-6.4</v>
       </c>
       <c r="F249" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G249" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="H249" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -12417,6 +12649,12 @@
       <c r="M249" t="n">
         <v>-6.51</v>
       </c>
+      <c r="N249" t="n">
+        <v>-9.949999999999999</v>
+      </c>
+      <c r="O249" t="n">
+        <v>-9.31</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -12443,6 +12681,14 @@
       <c r="F250" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G250" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K250" t="inlineStr"/>
@@ -12452,6 +12698,12 @@
       <c r="M250" t="n">
         <v>-6.48</v>
       </c>
+      <c r="N250" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="O250" t="n">
+        <v>8.300000000000001</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -12476,6 +12728,14 @@
         <v>2.94</v>
       </c>
       <c r="F251" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>19.86</v>
+      </c>
+      <c r="H251" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -12487,6 +12747,12 @@
       <c r="M251" t="n">
         <v>2.75</v>
       </c>
+      <c r="N251" t="n">
+        <v>19.11</v>
+      </c>
+      <c r="O251" t="n">
+        <v>19.64</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -12511,6 +12777,14 @@
         <v>11.45</v>
       </c>
       <c r="F252" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G252" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="H252" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -12522,6 +12796,12 @@
       <c r="M252" t="n">
         <v>10.83</v>
       </c>
+      <c r="N252" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="O252" t="n">
+        <v>2.09</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -15937,7 +16217,21 @@
       <c r="D350" t="n">
         <v>233.17</v>
       </c>
+      <c r="E350" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K350" t="inlineStr"/>
+      <c r="L350" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="M350" t="n">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -15958,7 +16252,21 @@
       <c r="D351" t="n">
         <v>225.31</v>
       </c>
+      <c r="E351" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K351" t="inlineStr"/>
+      <c r="L351" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="M351" t="n">
+        <v>-0.29</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -15979,7 +16287,21 @@
       <c r="D352" t="n">
         <v>738.79</v>
       </c>
+      <c r="E352" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K352" t="inlineStr"/>
+      <c r="L352" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="M352" t="n">
+        <v>1.12</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -16000,7 +16322,21 @@
       <c r="D353" t="n">
         <v>129.94</v>
       </c>
+      <c r="E353" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K353" t="inlineStr"/>
+      <c r="L353" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="M353" t="n">
+        <v>6.25</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -16021,7 +16357,21 @@
       <c r="D354" t="n">
         <v>28.72</v>
       </c>
+      <c r="E354" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K354" t="inlineStr"/>
+      <c r="L354" t="n">
+        <v>-6.26</v>
+      </c>
+      <c r="M354" t="n">
+        <v>-4.63</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -16042,7 +16392,21 @@
       <c r="D355" t="n">
         <v>186.97</v>
       </c>
+      <c r="E355" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K355" t="inlineStr"/>
+      <c r="L355" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="M355" t="n">
+        <v>2.12</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -16063,7 +16427,21 @@
       <c r="D356" t="n">
         <v>184.1</v>
       </c>
+      <c r="E356" t="n">
+        <v>-1.66</v>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K356" t="inlineStr"/>
+      <c r="L356" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="M356" t="n">
+        <v>-2.18</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -16084,7 +16462,21 @@
       <c r="D357" t="n">
         <v>493.66</v>
       </c>
+      <c r="E357" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K357" t="inlineStr"/>
+      <c r="L357" t="n">
+        <v>-3.09</v>
+      </c>
+      <c r="M357" t="n">
+        <v>-0.78</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -16105,7 +16497,21 @@
       <c r="D358" t="n">
         <v>198.35</v>
       </c>
+      <c r="E358" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K358" t="inlineStr"/>
+      <c r="L358" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="M358" t="n">
+        <v>6.71</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -16126,7 +16532,21 @@
       <c r="D359" t="n">
         <v>78.18000000000001</v>
       </c>
+      <c r="E359" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K359" t="inlineStr"/>
+      <c r="L359" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="M359" t="n">
+        <v>5.24</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -16147,7 +16567,21 @@
       <c r="D360" t="n">
         <v>291.25</v>
       </c>
+      <c r="E360" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K360" t="inlineStr"/>
+      <c r="L360" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="M360" t="n">
+        <v>-0.17</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -16168,7 +16602,21 @@
       <c r="D361" t="n">
         <v>539.59</v>
       </c>
+      <c r="E361" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K361" t="inlineStr"/>
+      <c r="L361" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="M361" t="n">
+        <v>4.9</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -16189,7 +16637,21 @@
       <c r="D362" t="n">
         <v>158.71</v>
       </c>
+      <c r="E362" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K362" t="inlineStr"/>
+      <c r="L362" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="M362" t="n">
+        <v>6.52</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -16210,7 +16672,21 @@
       <c r="D363" t="n">
         <v>116.22</v>
       </c>
+      <c r="E363" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K363" t="inlineStr"/>
+      <c r="L363" t="n">
+        <v>-5.58</v>
+      </c>
+      <c r="M363" t="n">
+        <v>-8.75</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -16231,7 +16707,21 @@
       <c r="D364" t="n">
         <v>105.22</v>
       </c>
+      <c r="E364" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K364" t="inlineStr"/>
+      <c r="L364" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="M364" t="n">
+        <v>5.11</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -16252,7 +16742,21 @@
       <c r="D365" t="n">
         <v>10.36</v>
       </c>
+      <c r="E365" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K365" t="inlineStr"/>
+      <c r="L365" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="M365" t="n">
+        <v>5.88</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -16273,7 +16777,21 @@
       <c r="D366" t="n">
         <v>129.94</v>
       </c>
+      <c r="E366" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K366" t="inlineStr"/>
+      <c r="L366" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="M366" t="n">
+        <v>6.25</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -16294,7 +16812,21 @@
       <c r="D367" t="n">
         <v>227.21</v>
       </c>
+      <c r="E367" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K367" t="inlineStr"/>
+      <c r="L367" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="M367" t="n">
+        <v>4.22</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -16315,7 +16847,21 @@
       <c r="D368" t="n">
         <v>184.1</v>
       </c>
+      <c r="E368" t="n">
+        <v>-1.66</v>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K368" t="inlineStr"/>
+      <c r="L368" t="n">
+        <v>-3.62</v>
+      </c>
+      <c r="M368" t="n">
+        <v>-2.18</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -16336,7 +16882,21 @@
       <c r="D369" t="n">
         <v>1729.76</v>
       </c>
+      <c r="E369" t="n">
+        <v>-4.02</v>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K369" t="inlineStr"/>
+      <c r="L369" t="n">
+        <v>-5.97</v>
+      </c>
+      <c r="M369" t="n">
+        <v>-4.12</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -16357,7 +16917,21 @@
       <c r="D370" t="n">
         <v>175.96</v>
       </c>
+      <c r="E370" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K370" t="inlineStr"/>
+      <c r="L370" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="M370" t="n">
+        <v>9.869999999999999</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -16378,7 +16952,21 @@
       <c r="D371" t="n">
         <v>41.82</v>
       </c>
+      <c r="E371" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K371" t="inlineStr"/>
+      <c r="L371" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="M371" t="n">
+        <v>14.93</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -16399,7 +16987,21 @@
       <c r="D372" t="n">
         <v>100.78</v>
       </c>
+      <c r="E372" t="n">
+        <v>-8.56</v>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K372" t="inlineStr"/>
+      <c r="L372" t="n">
+        <v>-10.51</v>
+      </c>
+      <c r="M372" t="n">
+        <v>-8.99</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -16420,7 +17022,21 @@
       <c r="D373" t="n">
         <v>512.01</v>
       </c>
+      <c r="E373" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K373" t="inlineStr"/>
+      <c r="L373" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="M373" t="n">
+        <v>3.1</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -16441,7 +17057,21 @@
       <c r="D374" t="n">
         <v>1834.39</v>
       </c>
+      <c r="E374" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K374" t="inlineStr"/>
+      <c r="L374" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="M374" t="n">
+        <v>0.19</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -16462,7 +17092,21 @@
       <c r="D375" t="n">
         <v>78.18000000000001</v>
       </c>
+      <c r="E375" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K375" t="inlineStr"/>
+      <c r="L375" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="M375" t="n">
+        <v>5.24</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -16483,7 +17127,21 @@
       <c r="D376" t="n">
         <v>291.25</v>
       </c>
+      <c r="E376" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K376" t="inlineStr"/>
+      <c r="L376" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="M376" t="n">
+        <v>-0.17</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -16504,7 +17162,21 @@
       <c r="D377" t="n">
         <v>738.79</v>
       </c>
+      <c r="E377" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K377" t="inlineStr"/>
+      <c r="L377" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="M377" t="n">
+        <v>1.12</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -16525,7 +17197,21 @@
       <c r="D378" t="n">
         <v>203.46</v>
       </c>
+      <c r="E378" t="n">
+        <v>-7.88</v>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K378" t="inlineStr"/>
+      <c r="L378" t="n">
+        <v>-9.83</v>
+      </c>
+      <c r="M378" t="n">
+        <v>0.37</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -16546,7 +17232,21 @@
       <c r="D379" t="n">
         <v>263.27</v>
       </c>
+      <c r="E379" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K379" t="inlineStr"/>
+      <c r="L379" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="M379" t="n">
+        <v>8.42</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -16567,7 +17267,21 @@
       <c r="D380" t="n">
         <v>149.42</v>
       </c>
+      <c r="E380" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K380" t="inlineStr"/>
+      <c r="L380" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="M380" t="n">
+        <v>5.61</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -16588,7 +17302,21 @@
       <c r="D381" t="n">
         <v>196.53</v>
       </c>
+      <c r="E381" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K381" t="inlineStr"/>
+      <c r="L381" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="M381" t="n">
+        <v>0.6899999999999999</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -16609,7 +17337,21 @@
       <c r="D382" t="n">
         <v>304.69</v>
       </c>
+      <c r="E382" t="n">
+        <v>3</v>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K382" t="inlineStr"/>
+      <c r="L382" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="M382" t="n">
+        <v>2.84</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -16630,7 +17372,21 @@
       <c r="D383" t="n">
         <v>40</v>
       </c>
+      <c r="E383" t="n">
+        <v>12.27</v>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K383" t="inlineStr"/>
+      <c r="L383" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="M383" t="n">
+        <v>11.9</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -16651,7 +17407,21 @@
       <c r="D384" t="n">
         <v>41.82</v>
       </c>
+      <c r="E384" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K384" t="inlineStr"/>
+      <c r="L384" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="M384" t="n">
+        <v>14.93</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -18920,6 +19690,636 @@
         <v>25.43</v>
       </c>
       <c r="K492" t="inlineStr"/>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Uptrend MA50</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>805.46</v>
+      </c>
+      <c r="K493" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>238.13</v>
+      </c>
+      <c r="K494" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>224.97</v>
+      </c>
+      <c r="K495" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>739.1900000000001</v>
+      </c>
+      <c r="K496" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>137.99</v>
+      </c>
+      <c r="K497" t="inlineStr"/>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="K498" t="inlineStr"/>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>192.08</v>
+      </c>
+      <c r="K499" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>181.04</v>
+      </c>
+      <c r="K500" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>488.05</v>
+      </c>
+      <c r="K501" t="inlineStr"/>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>212.4</v>
+      </c>
+      <c r="K502" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>333.66</v>
+      </c>
+      <c r="K503" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>573.83</v>
+      </c>
+      <c r="K504" t="inlineStr"/>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>EWY</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>186.41</v>
+      </c>
+      <c r="K505" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>137.99</v>
+      </c>
+      <c r="K506" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>181.04</v>
+      </c>
+      <c r="K507" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>1660.26</v>
+      </c>
+      <c r="K508" t="inlineStr"/>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>335.85</v>
+      </c>
+      <c r="K509" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>193.99</v>
+      </c>
+      <c r="K510" t="inlineStr"/>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>CEG</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>300.16</v>
+      </c>
+      <c r="K511" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>443.66</v>
+      </c>
+      <c r="K512" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>287.19</v>
+      </c>
+      <c r="K513" t="inlineStr"/>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>64.36</v>
+      </c>
+      <c r="K514" t="inlineStr"/>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>160.48</v>
+      </c>
+      <c r="K515" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>48.73</v>
+      </c>
+      <c r="K516" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D517" t="n">
+        <v>127.61</v>
+      </c>
+      <c r="K517" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>BOT</t>
+        </is>
+      </c>
+      <c r="D518" t="n">
+        <v>30.66</v>
+      </c>
+      <c r="K518" t="inlineStr"/>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>CIEN</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>443.66</v>
+      </c>
+      <c r="K519" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>287.19</v>
+      </c>
+      <c r="K520" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>64.36</v>
+      </c>
+      <c r="K521" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="K522" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19044,7 +20444,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
         <v>8</v>
@@ -19065,22 +20465,22 @@
         <v>-0.93</v>
       </c>
       <c r="I2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
-        <v>28.6</v>
+        <v>25</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.17</v>
+        <v>-0.47</v>
       </c>
       <c r="L2" t="n">
-        <v>-1.28</v>
+        <v>-1.54</v>
       </c>
       <c r="M2" t="n">
-        <v>28.6</v>
+        <v>25</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.93</v>
+        <v>-1.06</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -19093,43 +20493,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="C3" t="n">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="D3" t="n">
-        <v>46.5</v>
+        <v>47.2</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.53</v>
+        <v>-0.4</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.97</v>
+        <v>-0.95</v>
       </c>
       <c r="G3" t="n">
-        <v>36.8</v>
+        <v>37.4</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.64</v>
+        <v>-0.51</v>
       </c>
       <c r="I3" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="J3" t="n">
-        <v>52.2</v>
+        <v>52.6</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.04</v>
+        <v>-0.06</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.82</v>
+        <v>-0.83</v>
       </c>
       <c r="M3" t="n">
-        <v>46.4</v>
+        <v>46.2</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.48</v>
+        <v>-0.52</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -19142,43 +20542,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="C4" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="D4" t="n">
-        <v>68.3</v>
+        <v>69.7</v>
       </c>
       <c r="E4" t="n">
-        <v>2.75</v>
+        <v>3.08</v>
       </c>
       <c r="F4" t="n">
-        <v>2.29</v>
+        <v>2.37</v>
       </c>
       <c r="G4" t="n">
-        <v>63.5</v>
+        <v>64.5</v>
       </c>
       <c r="H4" t="n">
-        <v>2.64</v>
+        <v>2.81</v>
       </c>
       <c r="I4" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J4" t="n">
-        <v>74.40000000000001</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>5.63</v>
+        <v>5.6</v>
       </c>
       <c r="L4" t="n">
-        <v>4.76</v>
+        <v>4.74</v>
       </c>
       <c r="M4" t="n">
-        <v>71.8</v>
+        <v>73.2</v>
       </c>
       <c r="N4" t="n">
-        <v>5.44</v>
+        <v>5.4</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -19191,7 +20591,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C5" t="n">
         <v>21</v>
@@ -19240,43 +20640,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C6" t="n">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D6" t="n">
         <v>62</v>
       </c>
       <c r="E6" t="n">
-        <v>1.66</v>
+        <v>1.56</v>
       </c>
       <c r="F6" t="n">
-        <v>1.02</v>
+        <v>0.79</v>
       </c>
       <c r="G6" t="n">
-        <v>54.9</v>
+        <v>53.2</v>
       </c>
       <c r="H6" t="n">
-        <v>1.89</v>
+        <v>1.82</v>
       </c>
       <c r="I6" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="J6" t="n">
-        <v>68.09999999999999</v>
+        <v>67.3</v>
       </c>
       <c r="K6" t="n">
-        <v>3.71</v>
+        <v>3.43</v>
       </c>
       <c r="L6" t="n">
-        <v>2.95</v>
+        <v>2.68</v>
       </c>
       <c r="M6" t="n">
         <v>59.6</v>
       </c>
       <c r="N6" t="n">
-        <v>3.92</v>
+        <v>3.63</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -19289,43 +20689,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C7" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D7" t="n">
-        <v>52.1</v>
+        <v>55.3</v>
       </c>
       <c r="E7" t="n">
-        <v>1.32</v>
+        <v>1.72</v>
       </c>
       <c r="F7" t="n">
-        <v>0.82</v>
+        <v>1.13</v>
       </c>
       <c r="G7" t="n">
-        <v>43.7</v>
+        <v>46.1</v>
       </c>
       <c r="H7" t="n">
-        <v>1.3</v>
+        <v>1.69</v>
       </c>
       <c r="I7" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J7" t="n">
-        <v>61.2</v>
+        <v>63.5</v>
       </c>
       <c r="K7" t="n">
-        <v>2.09</v>
+        <v>2.58</v>
       </c>
       <c r="L7" t="n">
-        <v>1.38</v>
+        <v>1.87</v>
       </c>
       <c r="M7" t="n">
-        <v>59.2</v>
+        <v>61.5</v>
       </c>
       <c r="N7" t="n">
-        <v>2.27</v>
+        <v>2.72</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-07
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q529"/>
+  <dimension ref="A1:Q552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12145,7 +12145,7 @@
         </is>
       </c>
       <c r="G239" t="n">
-        <v>-8.68</v>
+        <v>-8.69</v>
       </c>
       <c r="H239" t="inlineStr">
         <is>
@@ -12160,10 +12160,10 @@
         <v>-7.87</v>
       </c>
       <c r="N239" t="n">
-        <v>-9.42</v>
+        <v>-9.43</v>
       </c>
       <c r="O239" t="n">
-        <v>-9.390000000000001</v>
+        <v>-9.4</v>
       </c>
     </row>
     <row r="240">
@@ -12830,6 +12830,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G253" t="n">
+        <v>-5.48</v>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K253" t="inlineStr"/>
       <c r="L253" t="n">
         <v>-2.7</v>
@@ -12837,6 +12845,12 @@
       <c r="M253" t="n">
         <v>-4.7</v>
       </c>
+      <c r="N253" t="n">
+        <v>-6.7</v>
+      </c>
+      <c r="O253" t="n">
+        <v>-6.79</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -12861,6 +12875,14 @@
         <v>2.46</v>
       </c>
       <c r="F254" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G254" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="H254" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -12872,6 +12894,12 @@
       <c r="M254" t="n">
         <v>3.5</v>
       </c>
+      <c r="N254" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="O254" t="n">
+        <v>6.86</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -12896,6 +12924,14 @@
         <v>-4.81</v>
       </c>
       <c r="F255" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G255" t="n">
+        <v>-2.08</v>
+      </c>
+      <c r="H255" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -12907,6 +12943,12 @@
       <c r="M255" t="n">
         <v>-4.31</v>
       </c>
+      <c r="N255" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="O255" t="n">
+        <v>-1.57</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -12933,6 +12975,14 @@
       <c r="F256" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G256" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K256" t="inlineStr"/>
@@ -12942,6 +12992,12 @@
       <c r="M256" t="n">
         <v>1.03</v>
       </c>
+      <c r="N256" t="n">
+        <v>-1.89</v>
+      </c>
+      <c r="O256" t="n">
+        <v>-0.84</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -12968,6 +13024,14 @@
       <c r="F257" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G257" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K257" t="inlineStr"/>
@@ -12977,6 +13041,12 @@
       <c r="M257" t="n">
         <v>-1.24</v>
       </c>
+      <c r="N257" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="O257" t="n">
+        <v>2.47</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -13001,6 +13071,14 @@
         <v>-6.69</v>
       </c>
       <c r="F258" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>-10.2</v>
+      </c>
+      <c r="H258" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13012,6 +13090,12 @@
       <c r="M258" t="n">
         <v>-6.48</v>
       </c>
+      <c r="N258" t="n">
+        <v>-11.42</v>
+      </c>
+      <c r="O258" t="n">
+        <v>-10</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -13038,6 +13122,14 @@
       <c r="F259" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K259" t="inlineStr"/>
@@ -13047,6 +13139,12 @@
       <c r="M259" t="n">
         <v>-3.59</v>
       </c>
+      <c r="N259" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="O259" t="n">
+        <v>1.45</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -13073,6 +13171,14 @@
       <c r="F260" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K260" t="inlineStr"/>
@@ -13082,6 +13188,12 @@
       <c r="M260" t="n">
         <v>-6.68</v>
       </c>
+      <c r="N260" t="n">
+        <v>-1.57</v>
+      </c>
+      <c r="O260" t="n">
+        <v>-0</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -13108,6 +13220,14 @@
       <c r="F261" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K261" t="inlineStr"/>
@@ -13117,6 +13237,12 @@
       <c r="M261" t="n">
         <v>2.06</v>
       </c>
+      <c r="N261" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="O261" t="n">
+        <v>8.34</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -13141,6 +13267,14 @@
         <v>4.09</v>
       </c>
       <c r="F262" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="H262" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -13152,6 +13286,12 @@
       <c r="M262" t="n">
         <v>1.64</v>
       </c>
+      <c r="N262" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="O262" t="n">
+        <v>2.16</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -13176,6 +13316,14 @@
         <v>1.27</v>
       </c>
       <c r="F263" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="H263" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -13187,6 +13335,12 @@
       <c r="M263" t="n">
         <v>2.74</v>
       </c>
+      <c r="N263" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="O263" t="n">
+        <v>6.78</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -13213,6 +13367,14 @@
       <c r="F264" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K264" t="inlineStr"/>
@@ -13222,6 +13384,12 @@
       <c r="M264" t="n">
         <v>1.49</v>
       </c>
+      <c r="N264" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="O264" t="n">
+        <v>8.98</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -13246,6 +13414,14 @@
         <v>-12.9</v>
       </c>
       <c r="F265" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>-11.48</v>
+      </c>
+      <c r="H265" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13257,6 +13433,12 @@
       <c r="M265" t="n">
         <v>-9.359999999999999</v>
       </c>
+      <c r="N265" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="O265" t="n">
+        <v>-7.89</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -13281,6 +13463,14 @@
         <v>-2.54</v>
       </c>
       <c r="F266" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>-3.08</v>
+      </c>
+      <c r="H266" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13292,6 +13482,12 @@
       <c r="M266" t="n">
         <v>-2.68</v>
       </c>
+      <c r="N266" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="O266" t="n">
+        <v>-3.22</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -13316,6 +13512,14 @@
         <v>-2.49</v>
       </c>
       <c r="F267" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="H267" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13327,6 +13531,12 @@
       <c r="M267" t="n">
         <v>-0.97</v>
       </c>
+      <c r="N267" t="n">
+        <v>-4.26</v>
+      </c>
+      <c r="O267" t="n">
+        <v>-1.54</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -13351,6 +13561,14 @@
         <v>-8.31</v>
       </c>
       <c r="F268" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G268" t="n">
+        <v>-10.74</v>
+      </c>
+      <c r="H268" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13362,6 +13580,12 @@
       <c r="M268" t="n">
         <v>-5.96</v>
       </c>
+      <c r="N268" t="n">
+        <v>-11.96</v>
+      </c>
+      <c r="O268" t="n">
+        <v>-8.449999999999999</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -13386,6 +13610,14 @@
         <v>5.74</v>
       </c>
       <c r="F269" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G269" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H269" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -13397,6 +13629,12 @@
       <c r="M269" t="n">
         <v>6.53</v>
       </c>
+      <c r="N269" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="O269" t="n">
+        <v>8.699999999999999</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -13423,6 +13661,14 @@
       <c r="F270" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G270" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K270" t="inlineStr"/>
@@ -13432,6 +13678,12 @@
       <c r="M270" t="n">
         <v>1.36</v>
       </c>
+      <c r="N270" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="O270" t="n">
+        <v>3.53</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -16428,7 +16680,7 @@
         <v>184.1</v>
       </c>
       <c r="E356" t="n">
-        <v>-1.65</v>
+        <v>-1.66</v>
       </c>
       <c r="F356" t="inlineStr">
         <is>
@@ -16437,10 +16689,10 @@
       </c>
       <c r="K356" t="inlineStr"/>
       <c r="L356" t="n">
-        <v>-3.61</v>
+        <v>-3.62</v>
       </c>
       <c r="M356" t="n">
-        <v>-2.17</v>
+        <v>-2.18</v>
       </c>
     </row>
     <row r="357">
@@ -16848,7 +17100,7 @@
         <v>184.1</v>
       </c>
       <c r="E368" t="n">
-        <v>-1.65</v>
+        <v>-1.66</v>
       </c>
       <c r="F368" t="inlineStr">
         <is>
@@ -16857,10 +17109,10 @@
       </c>
       <c r="K368" t="inlineStr"/>
       <c r="L368" t="n">
-        <v>-3.61</v>
+        <v>-3.62</v>
       </c>
       <c r="M368" t="n">
-        <v>-2.17</v>
+        <v>-2.18</v>
       </c>
     </row>
     <row r="369">
@@ -17442,7 +17694,21 @@
       <c r="D385" t="n">
         <v>239.94</v>
       </c>
+      <c r="E385" t="n">
+        <v>-3.02</v>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K385" t="inlineStr"/>
+      <c r="L385" t="n">
+        <v>-4.92</v>
+      </c>
+      <c r="M385" t="n">
+        <v>-5.48</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -17463,7 +17729,21 @@
       <c r="D386" t="n">
         <v>229.57</v>
       </c>
+      <c r="E386" t="n">
+        <v>-2.19</v>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K386" t="inlineStr"/>
+      <c r="L386" t="n">
+        <v>-4.09</v>
+      </c>
+      <c r="M386" t="n">
+        <v>-4.66</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -17484,7 +17764,21 @@
       <c r="D387" t="n">
         <v>725.1799999999999</v>
       </c>
+      <c r="E387" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K387" t="inlineStr"/>
+      <c r="L387" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="M387" t="n">
+        <v>-1.11</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -17505,7 +17799,21 @@
       <c r="D388" t="n">
         <v>134.01</v>
       </c>
+      <c r="E388" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K388" t="inlineStr"/>
+      <c r="L388" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M388" t="n">
+        <v>-0.96</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -17526,7 +17834,21 @@
       <c r="D389" t="n">
         <v>28.52</v>
       </c>
+      <c r="E389" t="n">
+        <v>-1.86</v>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K389" t="inlineStr"/>
+      <c r="L389" t="n">
+        <v>-3.76</v>
+      </c>
+      <c r="M389" t="n">
+        <v>-1.72</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -17547,7 +17869,21 @@
       <c r="D390" t="n">
         <v>187.05</v>
       </c>
+      <c r="E390" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K390" t="inlineStr"/>
+      <c r="L390" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="M390" t="n">
+        <v>1.99</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -17568,7 +17904,21 @@
       <c r="D391" t="n">
         <v>184.04</v>
       </c>
+      <c r="E391" t="n">
+        <v>-3.76</v>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K391" t="inlineStr"/>
+      <c r="L391" t="n">
+        <v>-5.66</v>
+      </c>
+      <c r="M391" t="n">
+        <v>-4.45</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -17589,7 +17939,21 @@
       <c r="D392" t="n">
         <v>487.38</v>
       </c>
+      <c r="E392" t="n">
+        <v>5.22</v>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K392" t="inlineStr"/>
+      <c r="L392" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="M392" t="n">
+        <v>4.98</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -17610,7 +17974,21 @@
       <c r="D393" t="n">
         <v>199.42</v>
       </c>
+      <c r="E393" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K393" t="inlineStr"/>
+      <c r="L393" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="M393" t="n">
+        <v>5.34</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -17631,7 +18009,21 @@
       <c r="D394" t="n">
         <v>333.02</v>
       </c>
+      <c r="E394" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K394" t="inlineStr"/>
+      <c r="L394" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="M394" t="n">
+        <v>1.91</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -17652,7 +18044,21 @@
       <c r="D395" t="n">
         <v>99.62</v>
       </c>
+      <c r="E395" t="n">
+        <v>-10.34</v>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K395" t="inlineStr"/>
+      <c r="L395" t="n">
+        <v>-12.24</v>
+      </c>
+      <c r="M395" t="n">
+        <v>-10.44</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -17673,7 +18079,21 @@
       <c r="D396" t="n">
         <v>537.95</v>
       </c>
+      <c r="E396" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K396" t="inlineStr"/>
+      <c r="L396" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M396" t="n">
+        <v>6.9</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -17694,7 +18114,21 @@
       <c r="D397" t="n">
         <v>153.76</v>
       </c>
+      <c r="E397" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K397" t="inlineStr"/>
+      <c r="L397" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="M397" t="n">
+        <v>5.96</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -17715,7 +18149,21 @@
       <c r="D398" t="n">
         <v>344.08</v>
       </c>
+      <c r="E398" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K398" t="inlineStr"/>
+      <c r="L398" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="M398" t="n">
+        <v>-0.22</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -17736,7 +18184,21 @@
       <c r="D399" t="n">
         <v>112.5</v>
       </c>
+      <c r="E399" t="n">
+        <v>-2.65</v>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K399" t="inlineStr"/>
+      <c r="L399" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="M399" t="n">
+        <v>-2.38</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -17757,7 +18219,21 @@
       <c r="D400" t="n">
         <v>10.14</v>
       </c>
+      <c r="E400" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K400" t="inlineStr"/>
+      <c r="L400" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="M400" t="n">
+        <v>4.79</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -17778,7 +18254,21 @@
       <c r="D401" t="n">
         <v>134.01</v>
       </c>
+      <c r="E401" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K401" t="inlineStr"/>
+      <c r="L401" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M401" t="n">
+        <v>-0.96</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -17799,7 +18289,21 @@
       <c r="D402" t="n">
         <v>184.04</v>
       </c>
+      <c r="E402" t="n">
+        <v>-3.76</v>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K402" t="inlineStr"/>
+      <c r="L402" t="n">
+        <v>-5.66</v>
+      </c>
+      <c r="M402" t="n">
+        <v>-4.45</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -17820,7 +18324,21 @@
       <c r="D403" t="n">
         <v>1739.89</v>
       </c>
+      <c r="E403" t="n">
+        <v>-2.71</v>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K403" t="inlineStr"/>
+      <c r="L403" t="n">
+        <v>-4.61</v>
+      </c>
+      <c r="M403" t="n">
+        <v>-2.55</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -17841,7 +18359,21 @@
       <c r="D404" t="n">
         <v>339.56</v>
       </c>
+      <c r="E404" t="n">
+        <v>-2.03</v>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K404" t="inlineStr"/>
+      <c r="L404" t="n">
+        <v>-3.93</v>
+      </c>
+      <c r="M404" t="n">
+        <v>-2.71</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -17862,7 +18394,21 @@
       <c r="D405" t="n">
         <v>179.29</v>
       </c>
+      <c r="E405" t="n">
+        <v>9.18</v>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K405" t="inlineStr"/>
+      <c r="L405" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="M405" t="n">
+        <v>6.45</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -17883,7 +18429,21 @@
       <c r="D406" t="n">
         <v>31.57</v>
       </c>
+      <c r="E406" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K406" t="inlineStr"/>
+      <c r="L406" t="n">
+        <v>5</v>
+      </c>
+      <c r="M406" t="n">
+        <v>5.27</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -17904,7 +18464,21 @@
       <c r="D407" t="n">
         <v>99.62</v>
       </c>
+      <c r="E407" t="n">
+        <v>-10.34</v>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K407" t="inlineStr"/>
+      <c r="L407" t="n">
+        <v>-12.24</v>
+      </c>
+      <c r="M407" t="n">
+        <v>-10.44</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -17925,7 +18499,21 @@
       <c r="D408" t="n">
         <v>1811.67</v>
       </c>
+      <c r="E408" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K408" t="inlineStr"/>
+      <c r="L408" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="M408" t="n">
+        <v>0.21</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -17946,7 +18534,21 @@
       <c r="D409" t="n">
         <v>77.41</v>
       </c>
+      <c r="E409" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K409" t="inlineStr"/>
+      <c r="L409" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="M409" t="n">
+        <v>2.18</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -17967,7 +18569,21 @@
       <c r="D410" t="n">
         <v>276.98</v>
       </c>
+      <c r="E410" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K410" t="inlineStr"/>
+      <c r="L410" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="M410" t="n">
+        <v>2.21</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -17988,7 +18604,21 @@
       <c r="D411" t="n">
         <v>155.25</v>
       </c>
+      <c r="E411" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K411" t="inlineStr"/>
+      <c r="L411" t="n">
+        <v>-3.96</v>
+      </c>
+      <c r="M411" t="n">
+        <v>-2.97</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -18009,7 +18639,21 @@
       <c r="D412" t="n">
         <v>971.26</v>
       </c>
+      <c r="E412" t="n">
+        <v>14.41</v>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K412" t="inlineStr"/>
+      <c r="L412" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="M412" t="n">
+        <v>13.29</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -18030,7 +18674,21 @@
       <c r="D413" t="n">
         <v>192.57</v>
       </c>
+      <c r="E413" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K413" t="inlineStr"/>
+      <c r="L413" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="M413" t="n">
+        <v>5.19</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -18051,7 +18709,21 @@
       <c r="D414" t="n">
         <v>512.9</v>
       </c>
+      <c r="E414" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K414" t="inlineStr"/>
+      <c r="L414" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="M414" t="n">
+        <v>1.76</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -18072,7 +18744,21 @@
       <c r="D415" t="n">
         <v>235.88</v>
       </c>
+      <c r="E415" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K415" t="inlineStr"/>
+      <c r="L415" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="M415" t="n">
+        <v>0.28</v>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -18093,7 +18779,21 @@
       <c r="D416" t="n">
         <v>307.82</v>
       </c>
+      <c r="E416" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K416" t="inlineStr"/>
+      <c r="L416" t="n">
+        <v>-3.01</v>
+      </c>
+      <c r="M416" t="n">
+        <v>-3.75</v>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -18114,7 +18814,21 @@
       <c r="D417" t="n">
         <v>40.34</v>
       </c>
+      <c r="E417" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K417" t="inlineStr"/>
+      <c r="L417" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="M417" t="n">
+        <v>3.02</v>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -19855,7 +20569,7 @@
         </is>
       </c>
       <c r="D500" t="n">
-        <v>181.06</v>
+        <v>181.04</v>
       </c>
       <c r="K500" t="inlineStr"/>
     </row>
@@ -20002,7 +20716,7 @@
         </is>
       </c>
       <c r="D507" t="n">
-        <v>181.06</v>
+        <v>181.04</v>
       </c>
       <c r="K507" t="inlineStr"/>
     </row>
@@ -20082,11 +20796,11 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>AAOI</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="D511" t="n">
-        <v>130.16</v>
+        <v>300.16</v>
       </c>
       <c r="K511" t="inlineStr"/>
     </row>
@@ -20103,11 +20817,11 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="D512" t="n">
-        <v>300.16</v>
+        <v>443.66</v>
       </c>
       <c r="K512" t="inlineStr"/>
     </row>
@@ -20124,11 +20838,11 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D513" t="n">
-        <v>443.66</v>
+        <v>287.19</v>
       </c>
       <c r="K513" t="inlineStr"/>
     </row>
@@ -20145,11 +20859,11 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D514" t="n">
-        <v>287.19</v>
+        <v>64.36</v>
       </c>
       <c r="K514" t="inlineStr"/>
     </row>
@@ -20166,11 +20880,11 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="D515" t="n">
-        <v>249.78</v>
+        <v>160.48</v>
       </c>
       <c r="K515" t="inlineStr"/>
     </row>
@@ -20182,16 +20896,16 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>Breakout Watch (EOD)</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>BUG</t>
         </is>
       </c>
       <c r="D516" t="n">
-        <v>64.36</v>
+        <v>48.73</v>
       </c>
       <c r="K516" t="inlineStr"/>
     </row>
@@ -20203,16 +20917,16 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>Breakout Watch (EOD)</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>HACK</t>
         </is>
       </c>
       <c r="D517" t="n">
-        <v>18.57</v>
+        <v>127.61</v>
       </c>
       <c r="K517" t="inlineStr"/>
     </row>
@@ -20224,16 +20938,16 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>Breakout Watch (EOD)</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>BOT</t>
         </is>
       </c>
       <c r="D518" t="n">
-        <v>160.48</v>
+        <v>30.66</v>
       </c>
       <c r="K518" t="inlineStr"/>
     </row>
@@ -20245,16 +20959,16 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>AAOI</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="D519" t="n">
-        <v>130.16</v>
+        <v>443.66</v>
       </c>
       <c r="K519" t="inlineStr"/>
     </row>
@@ -20266,16 +20980,16 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>BUG</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D520" t="n">
-        <v>48.73</v>
+        <v>287.19</v>
       </c>
       <c r="K520" t="inlineStr"/>
     </row>
@@ -20287,16 +21001,16 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D521" t="n">
-        <v>338.35</v>
+        <v>64.36</v>
       </c>
       <c r="K521" t="inlineStr"/>
     </row>
@@ -20308,165 +21022,648 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Performance: Buy</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>FOTO</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D522" t="n">
-        <v>20.53</v>
+        <v>25.8</v>
       </c>
       <c r="K522" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>Performance: Strong Buy</t>
+          <t>Uptrend MA50</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>HACK</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="D523" t="n">
-        <v>127.61</v>
+        <v>807.6</v>
       </c>
       <c r="K523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>BOT</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="D524" t="n">
-        <v>30.66</v>
+        <v>232.7</v>
       </c>
       <c r="K524" t="inlineStr"/>
     </row>
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="D525" t="n">
-        <v>443.66</v>
+        <v>224.55</v>
       </c>
       <c r="K525" t="inlineStr"/>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>LYTE</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D526" t="n">
-        <v>26.91</v>
+        <v>721.15</v>
       </c>
       <c r="K526" t="inlineStr"/>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="D527" t="n">
-        <v>287.19</v>
+        <v>27.99</v>
       </c>
       <c r="K527" t="inlineStr"/>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Golden Cross</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D528" t="n">
-        <v>64.36</v>
+        <v>177.12</v>
       </c>
       <c r="K528" t="inlineStr"/>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>512.83</v>
+      </c>
+      <c r="K529" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>213.68</v>
+      </c>
+      <c r="K530" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>294.37</v>
+      </c>
+      <c r="K531" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>291.2</v>
+      </c>
+      <c r="K532" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>EWY</t>
+        </is>
+      </c>
+      <c r="D533" t="n">
+        <v>183.6</v>
+      </c>
+      <c r="K533" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D534" t="n">
+        <v>721.15</v>
+      </c>
+      <c r="K534" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D535" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="K535" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D536" t="n">
+        <v>137.85</v>
+      </c>
+      <c r="K536" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D537" t="n">
+        <v>177.12</v>
+      </c>
+      <c r="K537" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="D538" t="n">
+        <v>1692.74</v>
+      </c>
+      <c r="K538" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D539" t="n">
+        <v>332.67</v>
+      </c>
+      <c r="K539" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D540" t="n">
+        <v>72.61</v>
+      </c>
+      <c r="K540" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D541" t="n">
+        <v>512.83</v>
+      </c>
+      <c r="K541" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>AAOI</t>
+        </is>
+      </c>
+      <c r="D542" t="n">
+        <v>122.55</v>
+      </c>
+      <c r="K542" t="inlineStr"/>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D543" t="n">
+        <v>645.83</v>
+      </c>
+      <c r="K543" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D544" t="n">
+        <v>47.84</v>
+      </c>
+      <c r="K544" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>COHR</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>334.71</v>
+      </c>
+      <c r="K545" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
           <t>Performance: Buy</t>
         </is>
       </c>
-      <c r="C529" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D529" t="n">
-        <v>25.8</v>
-      </c>
-      <c r="K529" t="inlineStr"/>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>265.35</v>
+      </c>
+      <c r="K546" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>FPS</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="K547" t="inlineStr"/>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>125.66</v>
+      </c>
+      <c r="K548" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>LYTE</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>26.52</v>
+      </c>
+      <c r="K549" t="inlineStr"/>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>196.49</v>
+      </c>
+      <c r="K550" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>284.73</v>
+      </c>
+      <c r="K551" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>72.61</v>
+      </c>
+      <c r="K552" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20591,7 +21788,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
         <v>8</v>
@@ -20640,43 +21837,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C3" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="D3" t="n">
-        <v>47.2</v>
+        <v>47</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.4</v>
+        <v>-0.31</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.95</v>
+        <v>-0.96</v>
       </c>
       <c r="G3" t="n">
-        <v>37.4</v>
+        <v>37.9</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.51</v>
+        <v>-0.52</v>
       </c>
       <c r="I3" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="J3" t="n">
-        <v>52.6</v>
+        <v>51.2</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.06</v>
+        <v>-0.19</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.83</v>
+        <v>-1</v>
       </c>
       <c r="M3" t="n">
-        <v>46.2</v>
+        <v>43</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.52</v>
+        <v>-0.57</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -20689,43 +21886,43 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="C4" t="n">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="D4" t="n">
-        <v>69.7</v>
+        <v>68.2</v>
       </c>
       <c r="E4" t="n">
-        <v>3.08</v>
+        <v>2.8</v>
       </c>
       <c r="F4" t="n">
-        <v>2.37</v>
+        <v>1.92</v>
       </c>
       <c r="G4" t="n">
-        <v>64.5</v>
+        <v>61.4</v>
       </c>
       <c r="H4" t="n">
-        <v>2.81</v>
+        <v>2.46</v>
       </c>
       <c r="I4" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J4" t="n">
-        <v>75.59999999999999</v>
+        <v>77.3</v>
       </c>
       <c r="K4" t="n">
-        <v>5.6</v>
+        <v>5.57</v>
       </c>
       <c r="L4" t="n">
-        <v>4.74</v>
+        <v>4.68</v>
       </c>
       <c r="M4" t="n">
-        <v>73.2</v>
+        <v>75</v>
       </c>
       <c r="N4" t="n">
-        <v>5.4</v>
+        <v>5.42</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -20738,25 +21935,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D5" t="n">
-        <v>66.7</v>
+        <v>68.2</v>
       </c>
       <c r="E5" t="n">
-        <v>3.18</v>
+        <v>3.35</v>
       </c>
       <c r="F5" t="n">
-        <v>2.44</v>
+        <v>2.55</v>
       </c>
       <c r="G5" t="n">
-        <v>66.7</v>
+        <v>68.2</v>
       </c>
       <c r="H5" t="n">
-        <v>1.99</v>
+        <v>2.14</v>
       </c>
       <c r="I5" t="n">
         <v>20</v>
@@ -20787,43 +21984,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C6" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D6" t="n">
-        <v>62</v>
+        <v>60.7</v>
       </c>
       <c r="E6" t="n">
-        <v>1.56</v>
+        <v>1.41</v>
       </c>
       <c r="F6" t="n">
-        <v>0.79</v>
+        <v>0.57</v>
       </c>
       <c r="G6" t="n">
-        <v>53.2</v>
+        <v>52.4</v>
       </c>
       <c r="H6" t="n">
-        <v>1.82</v>
+        <v>1.61</v>
       </c>
       <c r="I6" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J6" t="n">
-        <v>67.3</v>
+        <v>65.5</v>
       </c>
       <c r="K6" t="n">
-        <v>3.43</v>
+        <v>3.09</v>
       </c>
       <c r="L6" t="n">
-        <v>2.68</v>
+        <v>2.31</v>
       </c>
       <c r="M6" t="n">
-        <v>59.6</v>
+        <v>58.2</v>
       </c>
       <c r="N6" t="n">
-        <v>3.63</v>
+        <v>3.4</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -20836,43 +22033,43 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C7" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D7" t="n">
-        <v>55.3</v>
+        <v>57.3</v>
       </c>
       <c r="E7" t="n">
-        <v>1.72</v>
+        <v>1.87</v>
       </c>
       <c r="F7" t="n">
-        <v>1.13</v>
+        <v>1.18</v>
       </c>
       <c r="G7" t="n">
-        <v>46.1</v>
+        <v>47.6</v>
       </c>
       <c r="H7" t="n">
-        <v>1.69</v>
+        <v>1.81</v>
       </c>
       <c r="I7" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="J7" t="n">
-        <v>63.5</v>
+        <v>62.5</v>
       </c>
       <c r="K7" t="n">
-        <v>2.58</v>
+        <v>2.31</v>
       </c>
       <c r="L7" t="n">
-        <v>1.87</v>
+        <v>1.57</v>
       </c>
       <c r="M7" t="n">
-        <v>61.5</v>
+        <v>60.7</v>
       </c>
       <c r="N7" t="n">
-        <v>2.72</v>
+        <v>2.57</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-08
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q550"/>
+  <dimension ref="A1:Q574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,6 +539,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="I2" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>-5.69</v>
@@ -552,6 +560,12 @@
       <c r="O2" t="n">
         <v>-3.43</v>
       </c>
+      <c r="P2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -584,6 +598,14 @@
         <v>-2.1</v>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>-3.52</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -601,6 +623,12 @@
       <c r="O3" t="n">
         <v>-3.21</v>
       </c>
+      <c r="P3" t="n">
+        <v>-5.64</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>-4.62</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -633,6 +661,14 @@
         <v>5.24</v>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -650,6 +686,12 @@
       <c r="O4" t="n">
         <v>4.55</v>
       </c>
+      <c r="P4" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>3.48</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -682,6 +724,14 @@
         <v>5.88</v>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>8.27</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -699,6 +749,12 @@
       <c r="O5" t="n">
         <v>5.05</v>
       </c>
+      <c r="P5" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>7.43</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -731,6 +787,14 @@
         <v>1.11</v>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -748,6 +812,12 @@
       <c r="O6" t="n">
         <v>0.36</v>
       </c>
+      <c r="P6" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>5.36</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -780,6 +850,14 @@
         <v>5.04</v>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -797,6 +875,12 @@
       <c r="O7" t="n">
         <v>5.48</v>
       </c>
+      <c r="P7" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>6.97</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -829,6 +913,14 @@
         <v>2.75</v>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -846,6 +938,12 @@
       <c r="O8" t="n">
         <v>2.09</v>
       </c>
+      <c r="P8" t="n">
+        <v>-1.43</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -878,6 +976,14 @@
         <v>16.12</v>
       </c>
       <c r="H9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -895,6 +1001,12 @@
       <c r="O9" t="n">
         <v>14.47</v>
       </c>
+      <c r="P9" t="n">
+        <v>17.69</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>18.12</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -929,6 +1041,14 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -944,6 +1064,12 @@
       <c r="O10" t="n">
         <v>-1.43</v>
       </c>
+      <c r="P10" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>3.13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -978,6 +1104,14 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -993,6 +1127,12 @@
       <c r="O11" t="n">
         <v>-3.16</v>
       </c>
+      <c r="P11" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>-0.29</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1025,6 +1165,14 @@
         <v>7.26</v>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1042,6 +1190,12 @@
       <c r="O12" t="n">
         <v>7.74</v>
       </c>
+      <c r="P12" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>13.87</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1074,6 +1228,14 @@
         <v>14.76</v>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>18.03</v>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1091,6 +1253,12 @@
       <c r="O13" t="n">
         <v>14.07</v>
       </c>
+      <c r="P13" t="n">
+        <v>15.91</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>17.33</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1123,6 +1291,14 @@
         <v>24.33</v>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>25.91</v>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1140,6 +1316,12 @@
       <c r="O14" t="n">
         <v>24.72</v>
       </c>
+      <c r="P14" t="n">
+        <v>23.79</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>26.31</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1172,6 +1354,14 @@
         <v>-4.24</v>
       </c>
       <c r="H15" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>-6.25</v>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -1189,6 +1379,12 @@
       <c r="O15" t="n">
         <v>-5.61</v>
       </c>
+      <c r="P15" t="n">
+        <v>-8.369999999999999</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-7.6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1223,6 +1419,14 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K16" t="inlineStr"/>
@@ -1238,6 +1442,12 @@
       <c r="O16" t="n">
         <v>-1.85</v>
       </c>
+      <c r="P16" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>10.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1270,6 +1480,14 @@
         <v>1.11</v>
       </c>
       <c r="H17" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1287,6 +1505,12 @@
       <c r="O17" t="n">
         <v>0.36</v>
       </c>
+      <c r="P17" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>5.36</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1319,6 +1543,14 @@
         <v>15.31</v>
       </c>
       <c r="H18" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1336,6 +1568,12 @@
       <c r="O18" t="n">
         <v>14.61</v>
       </c>
+      <c r="P18" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>9.140000000000001</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1368,6 +1606,14 @@
         <v>16.12</v>
       </c>
       <c r="H19" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1385,6 +1631,12 @@
       <c r="O19" t="n">
         <v>14.47</v>
       </c>
+      <c r="P19" t="n">
+        <v>17.69</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>18.12</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1419,6 +1671,14 @@
       <c r="H20" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>-4.91</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -1434,6 +1694,12 @@
       <c r="O20" t="n">
         <v>2.24</v>
       </c>
+      <c r="P20" t="n">
+        <v>-7.03</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>-6.17</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1468,6 +1734,14 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -1483,6 +1757,12 @@
       <c r="O21" t="n">
         <v>-3.16</v>
       </c>
+      <c r="P21" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>-0.29</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1515,6 +1795,14 @@
         <v>7.26</v>
       </c>
       <c r="H22" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1532,6 +1820,12 @@
       <c r="O22" t="n">
         <v>7.74</v>
       </c>
+      <c r="P22" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>13.87</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1564,6 +1858,14 @@
         <v>5.4</v>
       </c>
       <c r="H23" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1581,6 +1883,12 @@
       <c r="O23" t="n">
         <v>4.44</v>
       </c>
+      <c r="P23" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>6.04</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1613,6 +1921,14 @@
         <v>2.86</v>
       </c>
       <c r="H24" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1630,6 +1946,12 @@
       <c r="O24" t="n">
         <v>2.49</v>
       </c>
+      <c r="P24" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>3.86</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1664,6 +1986,14 @@
       <c r="H25" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>-5.58</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -1679,6 +2009,12 @@
       <c r="O25" t="n">
         <v>6.49</v>
       </c>
+      <c r="P25" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>-5.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1711,6 +2047,14 @@
         <v>24.95</v>
       </c>
       <c r="H26" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>23.26</v>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -1728,6 +2072,12 @@
       <c r="O26" t="n">
         <v>23.11</v>
       </c>
+      <c r="P26" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>21.44</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1760,6 +2110,14 @@
         <v>-8.76</v>
       </c>
       <c r="H27" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>-11.37</v>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -1777,6 +2135,12 @@
       <c r="O27" t="n">
         <v>-15.24</v>
       </c>
+      <c r="P27" t="n">
+        <v>-13.49</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>-17.66</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1811,6 +2175,14 @@
       <c r="H28" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>-4.91</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -1826,6 +2198,12 @@
       <c r="O28" t="n">
         <v>2.24</v>
       </c>
+      <c r="P28" t="n">
+        <v>-7.03</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>-6.17</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13419,7 +13797,7 @@
         </is>
       </c>
       <c r="G265" t="n">
-        <v>-11.47</v>
+        <v>-11.48</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
@@ -13434,10 +13812,10 @@
         <v>-9.359999999999999</v>
       </c>
       <c r="N265" t="n">
-        <v>-12.69</v>
+        <v>-12.7</v>
       </c>
       <c r="O265" t="n">
-        <v>-7.87</v>
+        <v>-7.89</v>
       </c>
     </row>
     <row r="266">
@@ -13615,7 +13993,7 @@
         </is>
       </c>
       <c r="G269" t="n">
-        <v>7.88</v>
+        <v>7.9</v>
       </c>
       <c r="H269" t="inlineStr">
         <is>
@@ -13630,10 +14008,10 @@
         <v>6.53</v>
       </c>
       <c r="N269" t="n">
-        <v>6.66</v>
+        <v>6.68</v>
       </c>
       <c r="O269" t="n">
-        <v>8.68</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="270">
@@ -13712,6 +14090,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="G271" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K271" t="inlineStr"/>
       <c r="L271" t="n">
         <v>-0.23</v>
@@ -13719,6 +14105,12 @@
       <c r="M271" t="n">
         <v>-0.24</v>
       </c>
+      <c r="N271" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="O271" t="n">
+        <v>-4.02</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -13743,6 +14135,14 @@
         <v>-6.64</v>
       </c>
       <c r="F272" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G272" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="H272" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13754,6 +14154,12 @@
       <c r="M272" t="n">
         <v>-5.68</v>
       </c>
+      <c r="N272" t="n">
+        <v>-8.17</v>
+      </c>
+      <c r="O272" t="n">
+        <v>-6.34</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -13778,6 +14184,14 @@
         <v>2.99</v>
       </c>
       <c r="F273" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G273" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="H273" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -13789,6 +14203,12 @@
       <c r="M273" t="n">
         <v>2.66</v>
       </c>
+      <c r="N273" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="O273" t="n">
+        <v>4.64</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -13815,6 +14235,14 @@
       <c r="F274" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K274" t="inlineStr"/>
@@ -13824,6 +14252,12 @@
       <c r="M274" t="n">
         <v>0.27</v>
       </c>
+      <c r="N274" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="O274" t="n">
+        <v>1.71</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -13848,6 +14282,14 @@
         <v>-1.02</v>
       </c>
       <c r="F275" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G275" t="n">
+        <v>-2.01</v>
+      </c>
+      <c r="H275" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13859,6 +14301,12 @@
       <c r="M275" t="n">
         <v>-1.26</v>
       </c>
+      <c r="N275" t="n">
+        <v>-2.88</v>
+      </c>
+      <c r="O275" t="n">
+        <v>-2.24</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -13885,6 +14333,14 @@
       <c r="F276" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K276" t="inlineStr"/>
@@ -13894,6 +14350,12 @@
       <c r="M276" t="n">
         <v>-1.49</v>
       </c>
+      <c r="N276" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="O276" t="n">
+        <v>3.02</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -13918,6 +14380,14 @@
         <v>-6.26</v>
       </c>
       <c r="F277" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G277" t="n">
+        <v>-9.380000000000001</v>
+      </c>
+      <c r="H277" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -13929,6 +14399,12 @@
       <c r="M277" t="n">
         <v>-6.73</v>
       </c>
+      <c r="N277" t="n">
+        <v>-10.26</v>
+      </c>
+      <c r="O277" t="n">
+        <v>-9.84</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -13955,6 +14431,14 @@
       <c r="F278" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G278" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K278" t="inlineStr"/>
@@ -13964,6 +14448,12 @@
       <c r="M278" t="n">
         <v>-3.7</v>
       </c>
+      <c r="N278" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="O278" t="n">
+        <v>3.19</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -13990,6 +14480,14 @@
       <c r="F279" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G279" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K279" t="inlineStr"/>
@@ -13999,6 +14497,12 @@
       <c r="M279" t="n">
         <v>-3.6</v>
       </c>
+      <c r="N279" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="O279" t="n">
+        <v>5.15</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -14025,6 +14529,14 @@
       <c r="F280" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G280" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K280" t="inlineStr"/>
@@ -14034,6 +14546,12 @@
       <c r="M280" t="n">
         <v>2.73</v>
       </c>
+      <c r="N280" t="n">
+        <v>-1.74</v>
+      </c>
+      <c r="O280" t="n">
+        <v>-2.14</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -14058,6 +14576,14 @@
         <v>-8</v>
       </c>
       <c r="F281" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G281" t="n">
+        <v>-11.43</v>
+      </c>
+      <c r="H281" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14069,6 +14595,12 @@
       <c r="M281" t="n">
         <v>-8.720000000000001</v>
       </c>
+      <c r="N281" t="n">
+        <v>-12.3</v>
+      </c>
+      <c r="O281" t="n">
+        <v>-12.12</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -14093,6 +14625,14 @@
         <v>1.01</v>
       </c>
       <c r="F282" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G282" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="H282" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -14104,6 +14644,12 @@
       <c r="M282" t="n">
         <v>0.58</v>
       </c>
+      <c r="N282" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="O282" t="n">
+        <v>1.83</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -14128,6 +14674,14 @@
         <v>2.8</v>
       </c>
       <c r="F283" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G283" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="H283" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -14139,6 +14693,12 @@
       <c r="M283" t="n">
         <v>2.45</v>
       </c>
+      <c r="N283" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="O283" t="n">
+        <v>2.32</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -14163,6 +14723,14 @@
         <v>-1.13</v>
       </c>
       <c r="F284" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G284" t="n">
+        <v>-3.78</v>
+      </c>
+      <c r="H284" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14174,6 +14742,12 @@
       <c r="M284" t="n">
         <v>-2.72</v>
       </c>
+      <c r="N284" t="n">
+        <v>-4.65</v>
+      </c>
+      <c r="O284" t="n">
+        <v>-5.32</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -14198,6 +14772,14 @@
         <v>-2.15</v>
       </c>
       <c r="F285" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G285" t="n">
+        <v>-1.36</v>
+      </c>
+      <c r="H285" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14209,6 +14791,12 @@
       <c r="M285" t="n">
         <v>-3.06</v>
       </c>
+      <c r="N285" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="O285" t="n">
+        <v>-2.28</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -14233,6 +14821,14 @@
         <v>-4.57</v>
       </c>
       <c r="F286" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G286" t="n">
+        <v>-10.09</v>
+      </c>
+      <c r="H286" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14244,6 +14840,12 @@
       <c r="M286" t="n">
         <v>-8.31</v>
       </c>
+      <c r="N286" t="n">
+        <v>-10.96</v>
+      </c>
+      <c r="O286" t="n">
+        <v>-13.62</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -14270,6 +14872,14 @@
       <c r="F287" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G287" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K287" t="inlineStr"/>
@@ -14279,6 +14889,12 @@
       <c r="M287" t="n">
         <v>4.81</v>
       </c>
+      <c r="N287" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="O287" t="n">
+        <v>-1.36</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -14303,6 +14919,14 @@
         <v>-5.8</v>
       </c>
       <c r="F288" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G288" t="n">
+        <v>-15.9</v>
+      </c>
+      <c r="H288" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14314,6 +14938,12 @@
       <c r="M288" t="n">
         <v>-5.49</v>
       </c>
+      <c r="N288" t="n">
+        <v>-16.77</v>
+      </c>
+      <c r="O288" t="n">
+        <v>-15.62</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -14338,6 +14968,14 @@
         <v>-6.64</v>
       </c>
       <c r="F289" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G289" t="n">
+        <v>-7.3</v>
+      </c>
+      <c r="H289" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14349,6 +14987,12 @@
       <c r="M289" t="n">
         <v>-5.68</v>
       </c>
+      <c r="N289" t="n">
+        <v>-8.17</v>
+      </c>
+      <c r="O289" t="n">
+        <v>-6.34</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -14375,6 +15019,14 @@
       <c r="F290" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G290" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K290" t="inlineStr"/>
@@ -14384,6 +15036,12 @@
       <c r="M290" t="n">
         <v>-3.38</v>
       </c>
+      <c r="N290" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O290" t="n">
+        <v>0.85</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -14410,6 +15068,14 @@
       <c r="F291" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G291" t="n">
+        <v>-4.17</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K291" t="inlineStr"/>
@@ -14419,6 +15085,12 @@
       <c r="M291" t="n">
         <v>0.04</v>
       </c>
+      <c r="N291" t="n">
+        <v>-5.05</v>
+      </c>
+      <c r="O291" t="n">
+        <v>-5.61</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -14443,6 +15115,14 @@
         <v>-4.6</v>
       </c>
       <c r="F292" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G292" t="n">
+        <v>-9.75</v>
+      </c>
+      <c r="H292" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14454,6 +15134,12 @@
       <c r="M292" t="n">
         <v>-5.52</v>
       </c>
+      <c r="N292" t="n">
+        <v>-10.63</v>
+      </c>
+      <c r="O292" t="n">
+        <v>-10.63</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -14478,6 +15164,14 @@
         <v>-1.21</v>
       </c>
       <c r="F293" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G293" t="n">
+        <v>-4.52</v>
+      </c>
+      <c r="H293" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -14489,6 +15183,12 @@
       <c r="M293" t="n">
         <v>-2.7</v>
       </c>
+      <c r="N293" t="n">
+        <v>-5.39</v>
+      </c>
+      <c r="O293" t="n">
+        <v>-5.96</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -14515,6 +15215,14 @@
       <c r="F294" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G294" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K294" t="inlineStr"/>
@@ -14524,6 +15232,12 @@
       <c r="M294" t="n">
         <v>-1.49</v>
       </c>
+      <c r="N294" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="O294" t="n">
+        <v>3.02</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -18675,7 +19389,7 @@
         <v>192.57</v>
       </c>
       <c r="E413" t="n">
-        <v>2.02</v>
+        <v>2.04</v>
       </c>
       <c r="F413" t="inlineStr">
         <is>
@@ -18684,10 +19398,10 @@
       </c>
       <c r="K413" t="inlineStr"/>
       <c r="L413" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="M413" t="n">
-        <v>5.18</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="414">
@@ -18849,7 +19563,21 @@
       <c r="D418" t="n">
         <v>241.28</v>
       </c>
+      <c r="E418" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K418" t="inlineStr"/>
+      <c r="L418" t="n">
+        <v>-1.39</v>
+      </c>
+      <c r="M418" t="n">
+        <v>-0.92</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -18870,7 +19598,21 @@
       <c r="D419" t="n">
         <v>236.69</v>
       </c>
+      <c r="E419" t="n">
+        <v>-3.79</v>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K419" t="inlineStr"/>
+      <c r="L419" t="n">
+        <v>-5.08</v>
+      </c>
+      <c r="M419" t="n">
+        <v>-4.46</v>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -18891,7 +19633,21 @@
       <c r="D420" t="n">
         <v>725.9299999999999</v>
       </c>
+      <c r="E420" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K420" t="inlineStr"/>
+      <c r="L420" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M420" t="n">
+        <v>-1.79</v>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -18912,7 +19668,21 @@
       <c r="D421" t="n">
         <v>137.76</v>
       </c>
+      <c r="E421" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K421" t="inlineStr"/>
+      <c r="L421" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="M421" t="n">
+        <v>0.12</v>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -18933,7 +19703,21 @@
       <c r="D422" t="n">
         <v>28.12</v>
       </c>
+      <c r="E422" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K422" t="inlineStr"/>
+      <c r="L422" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="M422" t="n">
+        <v>-1.2</v>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -18954,7 +19738,21 @@
       <c r="D423" t="n">
         <v>190.04</v>
       </c>
+      <c r="E423" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K423" t="inlineStr"/>
+      <c r="L423" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="M423" t="n">
+        <v>2.85</v>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -18975,7 +19773,21 @@
       <c r="D424" t="n">
         <v>182.09</v>
       </c>
+      <c r="E424" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K424" t="inlineStr"/>
+      <c r="L424" t="n">
+        <v>-4.62</v>
+      </c>
+      <c r="M424" t="n">
+        <v>-5.83</v>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -18996,7 +19808,21 @@
       <c r="D425" t="n">
         <v>491.4</v>
       </c>
+      <c r="E425" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K425" t="inlineStr"/>
+      <c r="L425" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="M425" t="n">
+        <v>7.09</v>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -19017,7 +19843,21 @@
       <c r="D426" t="n">
         <v>198.78</v>
       </c>
+      <c r="E426" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K426" t="inlineStr"/>
+      <c r="L426" t="n">
+        <v>7.77</v>
+      </c>
+      <c r="M426" t="n">
+        <v>7.67</v>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -19038,7 +19878,21 @@
       <c r="D427" t="n">
         <v>330.32</v>
       </c>
+      <c r="E427" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K427" t="inlineStr"/>
+      <c r="L427" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="M427" t="n">
+        <v>2.05</v>
+      </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -19059,7 +19913,21 @@
       <c r="D428" t="n">
         <v>101.6</v>
       </c>
+      <c r="E428" t="n">
+        <v>-14.13</v>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K428" t="inlineStr"/>
+      <c r="L428" t="n">
+        <v>-15.43</v>
+      </c>
+      <c r="M428" t="n">
+        <v>-16.7</v>
+      </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -19080,7 +19948,21 @@
       <c r="D429" t="n">
         <v>277.58</v>
       </c>
+      <c r="E429" t="n">
+        <v>-1.78</v>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K429" t="inlineStr"/>
+      <c r="L429" t="n">
+        <v>-3.08</v>
+      </c>
+      <c r="M429" t="n">
+        <v>-4.1</v>
+      </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -19101,7 +19983,21 @@
       <c r="D430" t="n">
         <v>236.69</v>
       </c>
+      <c r="E430" t="n">
+        <v>-3.79</v>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K430" t="inlineStr"/>
+      <c r="L430" t="n">
+        <v>-5.08</v>
+      </c>
+      <c r="M430" t="n">
+        <v>-4.46</v>
+      </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -19122,7 +20018,21 @@
       <c r="D431" t="n">
         <v>541.74</v>
       </c>
+      <c r="E431" t="n">
+        <v>6.09</v>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K431" t="inlineStr"/>
+      <c r="L431" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="M431" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -19143,7 +20053,21 @@
       <c r="D432" t="n">
         <v>160.42</v>
       </c>
+      <c r="E432" t="n">
+        <v>-4.74</v>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K432" t="inlineStr"/>
+      <c r="L432" t="n">
+        <v>-6.04</v>
+      </c>
+      <c r="M432" t="n">
+        <v>-6.92</v>
+      </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -19164,7 +20088,21 @@
       <c r="D433" t="n">
         <v>10.37</v>
       </c>
+      <c r="E433" t="n">
+        <v>-2.22</v>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K433" t="inlineStr"/>
+      <c r="L433" t="n">
+        <v>-3.51</v>
+      </c>
+      <c r="M433" t="n">
+        <v>-4.44</v>
+      </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -19185,7 +20123,21 @@
       <c r="D434" t="n">
         <v>137.76</v>
       </c>
+      <c r="E434" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K434" t="inlineStr"/>
+      <c r="L434" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="M434" t="n">
+        <v>0.12</v>
+      </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -19206,7 +20158,21 @@
       <c r="D435" t="n">
         <v>182.09</v>
       </c>
+      <c r="E435" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K435" t="inlineStr"/>
+      <c r="L435" t="n">
+        <v>-4.62</v>
+      </c>
+      <c r="M435" t="n">
+        <v>-5.83</v>
+      </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -19227,7 +20193,21 @@
       <c r="D436" t="n">
         <v>1787.69</v>
       </c>
+      <c r="E436" t="n">
+        <v>-9.970000000000001</v>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K436" t="inlineStr"/>
+      <c r="L436" t="n">
+        <v>-11.26</v>
+      </c>
+      <c r="M436" t="n">
+        <v>-9.33</v>
+      </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -19248,7 +20228,21 @@
       <c r="D437" t="n">
         <v>319.19</v>
       </c>
+      <c r="E437" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K437" t="inlineStr"/>
+      <c r="L437" t="n">
+        <v>-6.58</v>
+      </c>
+      <c r="M437" t="n">
+        <v>-4.6</v>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -19269,7 +20263,21 @@
       <c r="D438" t="n">
         <v>19.24</v>
       </c>
+      <c r="E438" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K438" t="inlineStr"/>
+      <c r="L438" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="M438" t="n">
+        <v>-3.15</v>
+      </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -19290,7 +20298,21 @@
       <c r="D439" t="n">
         <v>101.6</v>
       </c>
+      <c r="E439" t="n">
+        <v>-14.13</v>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K439" t="inlineStr"/>
+      <c r="L439" t="n">
+        <v>-15.43</v>
+      </c>
+      <c r="M439" t="n">
+        <v>-16.7</v>
+      </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -19311,7 +20333,21 @@
       <c r="D440" t="n">
         <v>81.81</v>
       </c>
+      <c r="E440" t="n">
+        <v>-12.35</v>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K440" t="inlineStr"/>
+      <c r="L440" t="n">
+        <v>-13.64</v>
+      </c>
+      <c r="M440" t="n">
+        <v>-13.7</v>
+      </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -19332,7 +20368,21 @@
       <c r="D441" t="n">
         <v>19.24</v>
       </c>
+      <c r="E441" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K441" t="inlineStr"/>
+      <c r="L441" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="M441" t="n">
+        <v>-3.15</v>
+      </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -19353,7 +20403,21 @@
       <c r="D442" t="n">
         <v>1045.78</v>
       </c>
+      <c r="E442" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>FLAT</t>
+        </is>
+      </c>
       <c r="K442" t="inlineStr"/>
+      <c r="L442" t="n">
+        <v>-1.03</v>
+      </c>
+      <c r="M442" t="n">
+        <v>-0.54</v>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -19374,7 +20438,21 @@
       <c r="D443" t="n">
         <v>319.19</v>
       </c>
+      <c r="E443" t="n">
+        <v>-5.28</v>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K443" t="inlineStr"/>
+      <c r="L443" t="n">
+        <v>-6.58</v>
+      </c>
+      <c r="M443" t="n">
+        <v>-4.6</v>
+      </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -19395,7 +20473,21 @@
       <c r="D444" t="n">
         <v>987.45</v>
       </c>
+      <c r="E444" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K444" t="inlineStr"/>
+      <c r="L444" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="M444" t="n">
+        <v>-0.58</v>
+      </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -19416,7 +20508,21 @@
       <c r="D445" t="n">
         <v>151.77</v>
       </c>
+      <c r="E445" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K445" t="inlineStr"/>
+      <c r="L445" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M445" t="n">
+        <v>-0.12</v>
+      </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -19437,7 +20543,21 @@
       <c r="D446" t="n">
         <v>268.08</v>
       </c>
+      <c r="E446" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K446" t="inlineStr"/>
+      <c r="L446" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="M446" t="n">
+        <v>-1.32</v>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -19458,7 +20578,21 @@
       <c r="D447" t="n">
         <v>314.88</v>
       </c>
+      <c r="E447" t="n">
+        <v>-7.04</v>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K447" t="inlineStr"/>
+      <c r="L447" t="n">
+        <v>-8.34</v>
+      </c>
+      <c r="M447" t="n">
+        <v>-11.1</v>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -19479,7 +20613,21 @@
       <c r="D448" t="n">
         <v>1787.69</v>
       </c>
+      <c r="E448" t="n">
+        <v>-9.970000000000001</v>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K448" t="inlineStr"/>
+      <c r="L448" t="n">
+        <v>-11.26</v>
+      </c>
+      <c r="M448" t="n">
+        <v>-9.33</v>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -19500,7 +20648,21 @@
       <c r="D449" t="n">
         <v>44.78</v>
       </c>
+      <c r="E449" t="n">
+        <v>-1.52</v>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K449" t="inlineStr"/>
+      <c r="L449" t="n">
+        <v>-2.81</v>
+      </c>
+      <c r="M449" t="n">
+        <v>-4.04</v>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -19521,7 +20683,21 @@
       <c r="D450" t="n">
         <v>32.4</v>
       </c>
+      <c r="E450" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K450" t="inlineStr"/>
+      <c r="L450" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="M450" t="n">
+        <v>1.09</v>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
@@ -21220,7 +22396,7 @@
         </is>
       </c>
       <c r="D531" t="n">
-        <v>294.41</v>
+        <v>294.37</v>
       </c>
       <c r="K531" t="inlineStr"/>
     </row>
@@ -21279,11 +22455,11 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D534" t="n">
-        <v>109.52</v>
+        <v>721.15</v>
       </c>
       <c r="K534" t="inlineStr"/>
     </row>
@@ -21300,11 +22476,11 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="D535" t="n">
-        <v>721.15</v>
+        <v>10.62</v>
       </c>
       <c r="K535" t="inlineStr"/>
     </row>
@@ -21321,11 +22497,11 @@
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="D536" t="n">
-        <v>342.82</v>
+        <v>137.85</v>
       </c>
       <c r="K536" t="inlineStr"/>
     </row>
@@ -21342,11 +22518,11 @@
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>NOK</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="D537" t="n">
-        <v>10.62</v>
+        <v>177.12</v>
       </c>
       <c r="K537" t="inlineStr"/>
     </row>
@@ -21363,11 +22539,11 @@
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="D538" t="n">
-        <v>137.85</v>
+        <v>1692.74</v>
       </c>
       <c r="K538" t="inlineStr"/>
     </row>
@@ -21384,11 +22560,11 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="D539" t="n">
-        <v>177.12</v>
+        <v>332.67</v>
       </c>
       <c r="K539" t="inlineStr"/>
     </row>
@@ -21400,16 +22576,16 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>Bull Flag Watch</t>
+          <t>Breakout Watch (EOD)</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D540" t="n">
-        <v>1692.74</v>
+        <v>72.61</v>
       </c>
       <c r="K540" t="inlineStr"/>
     </row>
@@ -21421,16 +22597,16 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>Bull Flag Watch</t>
+          <t>Breakout Watch (EOD)</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>SPOT</t>
         </is>
       </c>
       <c r="D541" t="n">
-        <v>332.67</v>
+        <v>512.83</v>
       </c>
       <c r="K541" t="inlineStr"/>
     </row>
@@ -21442,16 +22618,16 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Breakout Watch (EOD)</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>AAOI</t>
         </is>
       </c>
       <c r="D542" t="n">
-        <v>72.61</v>
+        <v>122.55</v>
       </c>
       <c r="K542" t="inlineStr"/>
     </row>
@@ -21468,11 +22644,11 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>AAOI</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D543" t="n">
-        <v>122.55</v>
+        <v>645.83</v>
       </c>
       <c r="K543" t="inlineStr"/>
     </row>
@@ -21594,11 +22770,11 @@
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>LYTE</t>
         </is>
       </c>
       <c r="D549" t="n">
-        <v>196.46</v>
+        <v>26.52</v>
       </c>
       <c r="K549" t="inlineStr"/>
     </row>
@@ -21615,13 +22791,517 @@
       </c>
       <c r="C550" t="inlineStr">
         <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>196.49</v>
+      </c>
+      <c r="K550" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>284.73</v>
+      </c>
+      <c r="K551" t="inlineStr"/>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
           <t>PENG</t>
         </is>
       </c>
-      <c r="D550" t="n">
+      <c r="D552" t="n">
         <v>72.61</v>
       </c>
-      <c r="K550" t="inlineStr"/>
+      <c r="K552" t="inlineStr"/>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Uptrend MA50</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>774.96</v>
+      </c>
+      <c r="K553" t="inlineStr"/>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>241.06</v>
+      </c>
+      <c r="K554" t="inlineStr"/>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>227.73</v>
+      </c>
+      <c r="K555" t="inlineStr"/>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>720.84</v>
+      </c>
+      <c r="K556" t="inlineStr"/>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
+      <c r="D557" t="n">
+        <v>27.84</v>
+      </c>
+      <c r="K557" t="inlineStr"/>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>176.03</v>
+      </c>
+      <c r="K558" t="inlineStr"/>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D559" t="n">
+        <v>216.81</v>
+      </c>
+      <c r="K559" t="inlineStr"/>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>272.64</v>
+      </c>
+      <c r="K560" t="inlineStr"/>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>574.73</v>
+      </c>
+      <c r="K561" t="inlineStr"/>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>348.3</v>
+      </c>
+      <c r="K562" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>139.73</v>
+      </c>
+      <c r="K563" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>340.42</v>
+      </c>
+      <c r="K564" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>47.98</v>
+      </c>
+      <c r="K565" t="inlineStr"/>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D566" t="n">
+        <v>574.73</v>
+      </c>
+      <c r="K566" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>125.3</v>
+      </c>
+      <c r="K567" t="inlineStr"/>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D568" t="n">
+        <v>197.2</v>
+      </c>
+      <c r="K568" t="inlineStr"/>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>274.61</v>
+      </c>
+      <c r="K569" t="inlineStr"/>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>71.56999999999999</v>
+      </c>
+      <c r="K570" t="inlineStr"/>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>198.72</v>
+      </c>
+      <c r="K571" t="inlineStr"/>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="K572" t="inlineStr"/>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>203.57</v>
+      </c>
+      <c r="K573" t="inlineStr"/>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>216.81</v>
+      </c>
+      <c r="K574" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21746,7 +23426,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="n">
         <v>8</v>
@@ -21785,7 +23465,22 @@
         <v>-1.06</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="P2" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="S2" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="3">
@@ -21795,46 +23490,61 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C3" t="n">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D3" t="n">
-        <v>47</v>
+        <v>46.8</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.31</v>
+        <v>-0.2</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.96</v>
+        <v>-0.88</v>
       </c>
       <c r="G3" t="n">
-        <v>37.9</v>
+        <v>38.3</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.52</v>
+        <v>-0.46</v>
       </c>
       <c r="I3" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="J3" t="n">
-        <v>51.2</v>
+        <v>51.6</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.19</v>
+        <v>-0.27</v>
       </c>
       <c r="L3" t="n">
-        <v>-1</v>
+        <v>-1.09</v>
       </c>
       <c r="M3" t="n">
-        <v>43</v>
+        <v>44.2</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.57</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="P3" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="R3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="S3" t="n">
+        <v>75</v>
+      </c>
+      <c r="T3" t="n">
+        <v>6.83</v>
       </c>
     </row>
     <row r="4">
@@ -21844,46 +23554,61 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C4" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="D4" t="n">
-        <v>68.2</v>
+        <v>64.3</v>
       </c>
       <c r="E4" t="n">
-        <v>2.8</v>
+        <v>2.21</v>
       </c>
       <c r="F4" t="n">
-        <v>1.92</v>
+        <v>1.29</v>
       </c>
       <c r="G4" t="n">
-        <v>61.4</v>
+        <v>58.2</v>
       </c>
       <c r="H4" t="n">
-        <v>2.46</v>
+        <v>1.74</v>
       </c>
       <c r="I4" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="J4" t="n">
-        <v>77.3</v>
+        <v>75</v>
       </c>
       <c r="K4" t="n">
-        <v>5.57</v>
+        <v>4.95</v>
       </c>
       <c r="L4" t="n">
-        <v>4.68</v>
+        <v>4.07</v>
       </c>
       <c r="M4" t="n">
-        <v>75</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>5.42</v>
+        <v>4.76</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="P4" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="R4" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="S4" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="T4" t="n">
+        <v>8.449999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -21893,25 +23618,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D5" t="n">
-        <v>68.2</v>
+        <v>62.5</v>
       </c>
       <c r="E5" t="n">
-        <v>3.35</v>
+        <v>2.81</v>
       </c>
       <c r="F5" t="n">
-        <v>2.55</v>
+        <v>1.98</v>
       </c>
       <c r="G5" t="n">
-        <v>68.2</v>
+        <v>62.5</v>
       </c>
       <c r="H5" t="n">
-        <v>2.14</v>
+        <v>1.64</v>
       </c>
       <c r="I5" t="n">
         <v>20</v>
@@ -21942,46 +23667,61 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C6" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D6" t="n">
-        <v>60.7</v>
+        <v>59.1</v>
       </c>
       <c r="E6" t="n">
-        <v>1.41</v>
+        <v>1.04</v>
       </c>
       <c r="F6" t="n">
-        <v>0.57</v>
+        <v>0.18</v>
       </c>
       <c r="G6" t="n">
-        <v>52.4</v>
+        <v>50</v>
       </c>
       <c r="H6" t="n">
-        <v>1.61</v>
+        <v>1.15</v>
       </c>
       <c r="I6" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="J6" t="n">
-        <v>65.5</v>
+        <v>60</v>
       </c>
       <c r="K6" t="n">
-        <v>3.09</v>
+        <v>2.3</v>
       </c>
       <c r="L6" t="n">
-        <v>2.31</v>
+        <v>1.51</v>
       </c>
       <c r="M6" t="n">
-        <v>58.2</v>
+        <v>53.3</v>
       </c>
       <c r="N6" t="n">
-        <v>3.4</v>
+        <v>2.48</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="P6" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-2.79</v>
+      </c>
+      <c r="S6" t="n">
+        <v>50</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-0.92</v>
       </c>
     </row>
     <row r="7">
@@ -21991,46 +23731,61 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C7" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="D7" t="n">
-        <v>57.3</v>
+        <v>56.7</v>
       </c>
       <c r="E7" t="n">
-        <v>1.87</v>
+        <v>1.51</v>
       </c>
       <c r="F7" t="n">
-        <v>1.18</v>
+        <v>0.77</v>
       </c>
       <c r="G7" t="n">
-        <v>47.6</v>
+        <v>46.7</v>
       </c>
       <c r="H7" t="n">
-        <v>1.81</v>
+        <v>1.32</v>
       </c>
       <c r="I7" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="J7" t="n">
-        <v>62.5</v>
+        <v>59.7</v>
       </c>
       <c r="K7" t="n">
-        <v>2.31</v>
+        <v>1.75</v>
       </c>
       <c r="L7" t="n">
-        <v>1.57</v>
+        <v>0.99</v>
       </c>
       <c r="M7" t="n">
-        <v>60.7</v>
+        <v>58.1</v>
       </c>
       <c r="N7" t="n">
-        <v>2.57</v>
+        <v>1.92</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="P7" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="S7" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="T7" t="n">
+        <v>-0.8</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
BCC tracker: session 2026-10-09
</commit_message>
<xml_diff>
--- a/bcc/data/BCC-tracker.xlsx
+++ b/bcc/data/BCC-tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q575"/>
+  <dimension ref="A1:Q614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2240,6 +2240,14 @@
           <t>DOWN</t>
         </is>
       </c>
+      <c r="I29" t="n">
+        <v>-3.45</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>-1.32</v>
@@ -2253,6 +2261,12 @@
       <c r="O29" t="n">
         <v>-2.02</v>
       </c>
+      <c r="P29" t="n">
+        <v>-5.31</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>-3.08</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2285,6 +2299,14 @@
         <v>-5.53</v>
       </c>
       <c r="H30" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>-7.52</v>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -2302,6 +2324,12 @@
       <c r="O30" t="n">
         <v>-8.6</v>
       </c>
+      <c r="P30" t="n">
+        <v>-9.390000000000001</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>-10.53</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2334,6 +2362,14 @@
         <v>4.42</v>
       </c>
       <c r="H31" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2351,6 +2387,12 @@
       <c r="O31" t="n">
         <v>2.26</v>
       </c>
+      <c r="P31" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>8.619999999999999</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2383,6 +2425,14 @@
         <v>4.14</v>
       </c>
       <c r="H32" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2400,6 +2450,12 @@
       <c r="O32" t="n">
         <v>3.74</v>
       </c>
+      <c r="P32" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>7.55</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2432,6 +2488,14 @@
         <v>2.33</v>
       </c>
       <c r="H33" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2449,6 +2513,12 @@
       <c r="O33" t="n">
         <v>-3.23</v>
       </c>
+      <c r="P33" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2481,6 +2551,14 @@
         <v>3.43</v>
       </c>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2498,6 +2576,12 @@
       <c r="O34" t="n">
         <v>2</v>
       </c>
+      <c r="P34" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.58</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2530,6 +2614,14 @@
         <v>13.42</v>
       </c>
       <c r="H35" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2547,6 +2639,12 @@
       <c r="O35" t="n">
         <v>11.67</v>
       </c>
+      <c r="P35" t="n">
+        <v>23.15</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>23.1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2579,6 +2677,14 @@
         <v>2.46</v>
       </c>
       <c r="H36" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2596,6 +2702,12 @@
       <c r="O36" t="n">
         <v>1.15</v>
       </c>
+      <c r="P36" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>2.02</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2630,6 +2742,14 @@
       <c r="H37" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -2645,6 +2765,12 @@
       <c r="O37" t="n">
         <v>-5.73</v>
       </c>
+      <c r="P37" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>-2.22</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2677,6 +2803,14 @@
         <v>4.47</v>
       </c>
       <c r="H38" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2694,6 +2828,12 @@
       <c r="O38" t="n">
         <v>0.68</v>
       </c>
+      <c r="P38" t="n">
+        <v>13.22</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>10.91</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2726,6 +2866,14 @@
         <v>21.96</v>
       </c>
       <c r="H39" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>33.04</v>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2743,6 +2891,12 @@
       <c r="O39" t="n">
         <v>15.03</v>
       </c>
+      <c r="P39" t="n">
+        <v>31.18</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>25.49</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2775,6 +2929,14 @@
         <v>1.58</v>
       </c>
       <c r="H40" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>19</v>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2792,6 +2954,12 @@
       <c r="O40" t="n">
         <v>9.279999999999999</v>
       </c>
+      <c r="P40" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>28.05</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2824,6 +2992,14 @@
         <v>10.94</v>
       </c>
       <c r="H41" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2841,6 +3017,12 @@
       <c r="O41" t="n">
         <v>21.28</v>
       </c>
+      <c r="P41" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>27.48</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2873,6 +3055,14 @@
         <v>4.14</v>
       </c>
       <c r="H42" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2890,6 +3080,12 @@
       <c r="O42" t="n">
         <v>3.74</v>
       </c>
+      <c r="P42" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>7.55</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2922,6 +3118,14 @@
         <v>13.42</v>
       </c>
       <c r="H43" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>25.02</v>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -2939,6 +3143,12 @@
       <c r="O43" t="n">
         <v>11.67</v>
       </c>
+      <c r="P43" t="n">
+        <v>23.15</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>23.1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2973,6 +3183,14 @@
       <c r="H44" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>-3.14</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
@@ -2988,6 +3206,12 @@
       <c r="O44" t="n">
         <v>16.74</v>
       </c>
+      <c r="P44" t="n">
+        <v>-5.01</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>3.87</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3022,6 +3246,14 @@
       <c r="H45" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -3037,6 +3269,12 @@
       <c r="O45" t="n">
         <v>-5.73</v>
       </c>
+      <c r="P45" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>-2.22</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3071,6 +3309,14 @@
       <c r="H46" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
@@ -3086,6 +3332,12 @@
       <c r="O46" t="n">
         <v>-3.76</v>
       </c>
+      <c r="P46" t="n">
+        <v>7.78</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>8.140000000000001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3120,6 +3372,14 @@
       <c r="H47" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
@@ -3135,6 +3395,12 @@
       <c r="O47" t="n">
         <v>4.42</v>
       </c>
+      <c r="P47" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>8.779999999999999</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3167,6 +3433,14 @@
         <v>22.18</v>
       </c>
       <c r="H48" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>17.82</v>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -3184,6 +3458,12 @@
       <c r="O48" t="n">
         <v>29.58</v>
       </c>
+      <c r="P48" t="n">
+        <v>15.95</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>24.95</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3218,6 +3498,14 @@
       <c r="H49" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
@@ -3233,6 +3521,12 @@
       <c r="O49" t="n">
         <v>4.42</v>
       </c>
+      <c r="P49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>8.779999999999999</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3265,6 +3559,14 @@
         <v>-0.82</v>
       </c>
       <c r="H50" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>-6.09</v>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -3282,6 +3584,12 @@
       <c r="O50" t="n">
         <v>4.76</v>
       </c>
+      <c r="P50" t="n">
+        <v>-7.96</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>-0.82</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3314,6 +3622,14 @@
         <v>-5.81</v>
       </c>
       <c r="H51" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>-5.84</v>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -3331,6 +3647,12 @@
       <c r="O51" t="n">
         <v>3.94</v>
       </c>
+      <c r="P51" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>3.91</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3363,6 +3685,14 @@
         <v>1.58</v>
       </c>
       <c r="H52" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>19</v>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -3380,6 +3710,12 @@
       <c r="O52" t="n">
         <v>9.279999999999999</v>
       </c>
+      <c r="P52" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>28.05</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3412,6 +3748,14 @@
         <v>-6.65</v>
       </c>
       <c r="H53" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>-6.78</v>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -3429,6 +3773,12 @@
       <c r="O53" t="n">
         <v>3.39</v>
       </c>
+      <c r="P53" t="n">
+        <v>-8.65</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>3.24</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15266,6 +15616,14 @@
           <t>FLAT</t>
         </is>
       </c>
+      <c r="G295" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K295" t="inlineStr"/>
       <c r="L295" t="n">
         <v>0.51</v>
@@ -15273,6 +15631,12 @@
       <c r="M295" t="n">
         <v>4.22</v>
       </c>
+      <c r="N295" t="n">
+        <v>-3.04</v>
+      </c>
+      <c r="O295" t="n">
+        <v>1.73</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -15297,6 +15661,14 @@
         <v>-3.14</v>
       </c>
       <c r="F296" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G296" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H296" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -15308,6 +15680,12 @@
       <c r="M296" t="n">
         <v>-3.03</v>
       </c>
+      <c r="N296" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="O296" t="n">
+        <v>-4.29</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -15334,6 +15712,14 @@
       <c r="F297" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G297" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K297" t="inlineStr"/>
@@ -15343,6 +15729,12 @@
       <c r="M297" t="n">
         <v>2.29</v>
       </c>
+      <c r="N297" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="O297" t="n">
+        <v>5.76</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -15369,6 +15761,14 @@
       <c r="F298" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G298" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K298" t="inlineStr"/>
@@ -15378,6 +15778,12 @@
       <c r="M298" t="n">
         <v>3.43</v>
       </c>
+      <c r="N298" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="O298" t="n">
+        <v>8.42</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -15402,6 +15808,14 @@
         <v>-3.03</v>
       </c>
       <c r="F299" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G299" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="H299" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -15413,6 +15827,12 @@
       <c r="M299" t="n">
         <v>-2.97</v>
       </c>
+      <c r="N299" t="n">
+        <v>-2.33</v>
+      </c>
+      <c r="O299" t="n">
+        <v>-1.32</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -15439,6 +15859,14 @@
       <c r="F300" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G300" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K300" t="inlineStr"/>
@@ -15448,6 +15876,12 @@
       <c r="M300" t="n">
         <v>1.25</v>
       </c>
+      <c r="N300" t="n">
+        <v>9.289999999999999</v>
+      </c>
+      <c r="O300" t="n">
+        <v>12.16</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -15472,6 +15906,14 @@
         <v>-8.470000000000001</v>
       </c>
       <c r="F301" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G301" t="n">
+        <v>-13.08</v>
+      </c>
+      <c r="H301" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -15483,6 +15925,12 @@
       <c r="M301" t="n">
         <v>-7.28</v>
       </c>
+      <c r="N301" t="n">
+        <v>-14.01</v>
+      </c>
+      <c r="O301" t="n">
+        <v>-11.95</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -15509,6 +15957,14 @@
       <c r="F302" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G302" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K302" t="inlineStr"/>
@@ -15518,6 +15974,12 @@
       <c r="M302" t="n">
         <v>-6.83</v>
       </c>
+      <c r="N302" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O302" t="n">
+        <v>4.24</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -15542,6 +16004,14 @@
         <v>1.84</v>
       </c>
       <c r="F303" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G303" t="n">
+        <v>21.16</v>
+      </c>
+      <c r="H303" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -15553,6 +16023,12 @@
       <c r="M303" t="n">
         <v>3.98</v>
       </c>
+      <c r="N303" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="O303" t="n">
+        <v>23.72</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -15579,6 +16055,14 @@
       <c r="F304" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G304" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>FLAT</t>
         </is>
       </c>
       <c r="K304" t="inlineStr"/>
@@ -15588,6 +16072,12 @@
       <c r="M304" t="n">
         <v>6.34</v>
       </c>
+      <c r="N304" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="O304" t="n">
+        <v>1.48</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -15612,6 +16102,14 @@
         <v>-5.58</v>
       </c>
       <c r="F305" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G305" t="n">
+        <v>-8.67</v>
+      </c>
+      <c r="H305" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -15623,6 +16121,12 @@
       <c r="M305" t="n">
         <v>-4.58</v>
       </c>
+      <c r="N305" t="n">
+        <v>-9.6</v>
+      </c>
+      <c r="O305" t="n">
+        <v>-7.7</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -15647,6 +16151,14 @@
         <v>2.28</v>
       </c>
       <c r="F306" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G306" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="H306" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -15658,6 +16170,12 @@
       <c r="M306" t="n">
         <v>4.43</v>
       </c>
+      <c r="N306" t="n">
+        <v>5.29</v>
+      </c>
+      <c r="O306" t="n">
+        <v>8.449999999999999</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -15684,6 +16202,14 @@
       <c r="F307" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G307" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K307" t="inlineStr"/>
@@ -15693,6 +16219,12 @@
       <c r="M307" t="n">
         <v>3.43</v>
       </c>
+      <c r="N307" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="O307" t="n">
+        <v>8.42</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -15717,6 +16249,14 @@
         <v>3.95</v>
       </c>
       <c r="F308" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G308" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H308" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -15728,6 +16268,12 @@
       <c r="M308" t="n">
         <v>1.73</v>
       </c>
+      <c r="N308" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="O308" t="n">
+        <v>-0.28</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -15752,6 +16298,14 @@
         <v>1.52</v>
       </c>
       <c r="F309" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="G309" t="n">
+        <v>9.82</v>
+      </c>
+      <c r="H309" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
@@ -15763,6 +16317,12 @@
       <c r="M309" t="n">
         <v>6.47</v>
       </c>
+      <c r="N309" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="O309" t="n">
+        <v>15.18</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -15789,6 +16349,14 @@
       <c r="F310" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G310" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K310" t="inlineStr"/>
@@ -15798,6 +16366,12 @@
       <c r="M310" t="n">
         <v>3.07</v>
       </c>
+      <c r="N310" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="O310" t="n">
+        <v>13.46</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -15824,6 +16398,14 @@
       <c r="F311" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G311" t="n">
+        <v>-18.84</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K311" t="inlineStr"/>
@@ -15833,6 +16415,12 @@
       <c r="M311" t="n">
         <v>5.58</v>
       </c>
+      <c r="N311" t="n">
+        <v>-19.77</v>
+      </c>
+      <c r="O311" t="n">
+        <v>-16.59</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -15857,6 +16445,14 @@
         <v>-3.92</v>
       </c>
       <c r="F312" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G312" t="n">
+        <v>-6.19</v>
+      </c>
+      <c r="H312" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -15868,6 +16464,12 @@
       <c r="M312" t="n">
         <v>-1.78</v>
       </c>
+      <c r="N312" t="n">
+        <v>-7.12</v>
+      </c>
+      <c r="O312" t="n">
+        <v>-4.1</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -15892,6 +16494,14 @@
         <v>-0.91</v>
       </c>
       <c r="F313" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G313" t="n">
+        <v>-14.1</v>
+      </c>
+      <c r="H313" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -15903,6 +16513,12 @@
       <c r="M313" t="n">
         <v>0.44</v>
       </c>
+      <c r="N313" t="n">
+        <v>-15.04</v>
+      </c>
+      <c r="O313" t="n">
+        <v>-12.94</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -15929,6 +16545,14 @@
       <c r="F314" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G314" t="n">
+        <v>-13.3</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K314" t="inlineStr"/>
@@ -15938,6 +16562,12 @@
       <c r="M314" t="n">
         <v>12.1</v>
       </c>
+      <c r="N314" t="n">
+        <v>-14.23</v>
+      </c>
+      <c r="O314" t="n">
+        <v>-10.67</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -15964,6 +16594,14 @@
       <c r="F315" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G315" t="n">
+        <v>-2.91</v>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K315" t="inlineStr"/>
@@ -15973,6 +16611,12 @@
       <c r="M315" t="n">
         <v>2.25</v>
       </c>
+      <c r="N315" t="n">
+        <v>-3.84</v>
+      </c>
+      <c r="O315" t="n">
+        <v>-0.88</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -15999,6 +16643,14 @@
       <c r="F316" t="inlineStr">
         <is>
           <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G316" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K316" t="inlineStr"/>
@@ -16008,6 +16660,12 @@
       <c r="M316" t="n">
         <v>-2.74</v>
       </c>
+      <c r="N316" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="O316" t="n">
+        <v>15.18</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -16032,6 +16690,14 @@
         <v>-3.14</v>
       </c>
       <c r="F317" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G317" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H317" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -16043,6 +16709,12 @@
       <c r="M317" t="n">
         <v>-3.03</v>
       </c>
+      <c r="N317" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="O317" t="n">
+        <v>-4.29</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -16069,6 +16741,14 @@
       <c r="F318" t="inlineStr">
         <is>
           <t>FLAT</t>
+        </is>
+      </c>
+      <c r="G318" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>UP</t>
         </is>
       </c>
       <c r="K318" t="inlineStr"/>
@@ -16078,6 +16758,12 @@
       <c r="M318" t="n">
         <v>2.29</v>
       </c>
+      <c r="N318" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="O318" t="n">
+        <v>5.76</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -16102,6 +16788,14 @@
         <v>-0.68</v>
       </c>
       <c r="F319" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="G319" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H319" t="inlineStr">
         <is>
           <t>DOWN</t>
         </is>
@@ -16113,6 +16807,12 @@
       <c r="M319" t="n">
         <v>-0.2</v>
       </c>
+      <c r="N319" t="n">
+        <v>-5.93</v>
+      </c>
+      <c r="O319" t="n">
+        <v>-4.55</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -16139,6 +16839,14 @@
       <c r="F320" t="inlineStr">
         <is>
           <t>UP</t>
+        </is>
+      </c>
+      <c r="G320" t="n">
+        <v>-8.74</v>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="K320" t="inlineStr"/>
@@ -16148,6 +16856,12 @@
       <c r="M320" t="n">
         <v>1.39</v>
       </c>
+      <c r="N320" t="n">
+        <v>-9.67</v>
+      </c>
+      <c r="O320" t="n">
+        <v>-8.880000000000001</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -20718,7 +21432,21 @@
       <c r="D451" t="n">
         <v>237.69</v>
       </c>
+      <c r="E451" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K451" t="inlineStr"/>
+      <c r="L451" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="M451" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -20739,7 +21467,21 @@
       <c r="D452" t="n">
         <v>234.69</v>
       </c>
+      <c r="E452" t="n">
+        <v>-2.39</v>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K452" t="inlineStr"/>
+      <c r="L452" t="n">
+        <v>-3.55</v>
+      </c>
+      <c r="M452" t="n">
+        <v>-2.38</v>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -20760,7 +21502,21 @@
       <c r="D453" t="n">
         <v>728.08</v>
       </c>
+      <c r="E453" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K453" t="inlineStr"/>
+      <c r="L453" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="M453" t="n">
+        <v>-1.35</v>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -20781,7 +21537,21 @@
       <c r="D454" t="n">
         <v>134.38</v>
       </c>
+      <c r="E454" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K454" t="inlineStr"/>
+      <c r="L454" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="M454" t="n">
+        <v>4.07</v>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -20802,7 +21572,21 @@
       <c r="D455" t="n">
         <v>27.8</v>
       </c>
+      <c r="E455" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K455" t="inlineStr"/>
+      <c r="L455" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="M455" t="n">
+        <v>2.14</v>
+      </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -20823,7 +21607,21 @@
       <c r="D456" t="n">
         <v>188.75</v>
       </c>
+      <c r="E456" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K456" t="inlineStr"/>
+      <c r="L456" t="n">
+        <v>9.609999999999999</v>
+      </c>
+      <c r="M456" t="n">
+        <v>10.25</v>
+      </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -20844,7 +21642,21 @@
       <c r="D457" t="n">
         <v>184.87</v>
       </c>
+      <c r="E457" t="n">
+        <v>-5.04</v>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K457" t="inlineStr"/>
+      <c r="L457" t="n">
+        <v>-6.19</v>
+      </c>
+      <c r="M457" t="n">
+        <v>-5.24</v>
+      </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -20865,7 +21677,21 @@
       <c r="D458" t="n">
         <v>472.89</v>
       </c>
+      <c r="E458" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K458" t="inlineStr"/>
+      <c r="L458" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="M458" t="n">
+        <v>11.74</v>
+      </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -20886,7 +21712,21 @@
       <c r="D459" t="n">
         <v>196.6</v>
       </c>
+      <c r="E459" t="n">
+        <v>18.97</v>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K459" t="inlineStr"/>
+      <c r="L459" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="M459" t="n">
+        <v>18.55</v>
+      </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -20907,7 +21747,21 @@
       <c r="D460" t="n">
         <v>333.69</v>
       </c>
+      <c r="E460" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K460" t="inlineStr"/>
+      <c r="L460" t="n">
+        <v>-0.27</v>
+      </c>
+      <c r="M460" t="n">
+        <v>1.04</v>
+      </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -20928,7 +21782,21 @@
       <c r="D461" t="n">
         <v>289.15</v>
       </c>
+      <c r="E461" t="n">
+        <v>-3.06</v>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K461" t="inlineStr"/>
+      <c r="L461" t="n">
+        <v>-4.22</v>
+      </c>
+      <c r="M461" t="n">
+        <v>-3.44</v>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -20949,7 +21817,21 @@
       <c r="D462" t="n">
         <v>562.52</v>
       </c>
+      <c r="E462" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K462" t="inlineStr"/>
+      <c r="L462" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="M462" t="n">
+        <v>5.17</v>
+      </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -20970,7 +21852,21 @@
       <c r="D463" t="n">
         <v>184.87</v>
       </c>
+      <c r="E463" t="n">
+        <v>-5.04</v>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
       <c r="K463" t="inlineStr"/>
+      <c r="L463" t="n">
+        <v>-6.19</v>
+      </c>
+      <c r="M463" t="n">
+        <v>-5.24</v>
+      </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -20991,7 +21887,21 @@
       <c r="D464" t="n">
         <v>341.04</v>
       </c>
+      <c r="E464" t="n">
+        <v>8.17</v>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K464" t="inlineStr"/>
+      <c r="L464" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="M464" t="n">
+        <v>7.77</v>
+      </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -21012,7 +21922,21 @@
       <c r="D465" t="n">
         <v>196.6</v>
       </c>
+      <c r="E465" t="n">
+        <v>18.97</v>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K465" t="inlineStr"/>
+      <c r="L465" t="n">
+        <v>17.81</v>
+      </c>
+      <c r="M465" t="n">
+        <v>18.55</v>
+      </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -21033,7 +21957,21 @@
       <c r="D466" t="n">
         <v>61.36</v>
       </c>
+      <c r="E466" t="n">
+        <v>24.32</v>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K466" t="inlineStr"/>
+      <c r="L466" t="n">
+        <v>23.16</v>
+      </c>
+      <c r="M466" t="n">
+        <v>24.74</v>
+      </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -21054,7 +21992,21 @@
       <c r="D467" t="n">
         <v>46.92</v>
       </c>
+      <c r="E467" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K467" t="inlineStr"/>
+      <c r="L467" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="M467" t="n">
+        <v>6.57</v>
+      </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -21075,7 +22027,21 @@
       <c r="D468" t="n">
         <v>123.08</v>
       </c>
+      <c r="E468" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K468" t="inlineStr"/>
+      <c r="L468" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="M468" t="n">
+        <v>5.98</v>
+      </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -21096,7 +22062,21 @@
       <c r="D469" t="n">
         <v>1085.42</v>
       </c>
+      <c r="E469" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K469" t="inlineStr"/>
+      <c r="L469" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="M469" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -21117,7 +22097,21 @@
       <c r="D470" t="n">
         <v>61.36</v>
       </c>
+      <c r="E470" t="n">
+        <v>24.32</v>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K470" t="inlineStr"/>
+      <c r="L470" t="n">
+        <v>23.16</v>
+      </c>
+      <c r="M470" t="n">
+        <v>24.74</v>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -21138,7 +22132,21 @@
       <c r="D471" t="n">
         <v>25.06</v>
       </c>
+      <c r="E471" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="K471" t="inlineStr"/>
+      <c r="L471" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="M471" t="n">
+        <v>4.35</v>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -23022,11 +24030,11 @@
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="D561" t="n">
-        <v>348.3</v>
+        <v>139.73</v>
       </c>
       <c r="K561" t="inlineStr"/>
     </row>
@@ -23038,16 +24046,16 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Bull Flag Watch</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D562" t="n">
-        <v>139.73</v>
+        <v>340.42</v>
       </c>
       <c r="K562" t="inlineStr"/>
     </row>
@@ -23064,11 +24072,11 @@
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>BUG</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="D563" t="n">
-        <v>47.98</v>
+        <v>346.9</v>
       </c>
       <c r="K563" t="inlineStr"/>
     </row>
@@ -23085,11 +24093,11 @@
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>BUG</t>
         </is>
       </c>
       <c r="D564" t="n">
-        <v>574.73</v>
+        <v>47.98</v>
       </c>
       <c r="K564" t="inlineStr"/>
     </row>
@@ -23106,11 +24114,11 @@
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>HACK</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="D565" t="n">
-        <v>125.3</v>
+        <v>425.73</v>
       </c>
       <c r="K565" t="inlineStr"/>
     </row>
@@ -23122,16 +24130,16 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="D566" t="n">
-        <v>720.84</v>
+        <v>574.73</v>
       </c>
       <c r="K566" t="inlineStr"/>
     </row>
@@ -23143,16 +24151,16 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>HACK</t>
         </is>
       </c>
       <c r="D567" t="n">
-        <v>197.2</v>
+        <v>125.3</v>
       </c>
       <c r="K567" t="inlineStr"/>
     </row>
@@ -23164,16 +24172,16 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Performance: Buy</t>
+          <t>Performance: Strong Buy</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>IGV</t>
         </is>
       </c>
       <c r="D568" t="n">
-        <v>274.61</v>
+        <v>109.57</v>
       </c>
       <c r="K568" t="inlineStr"/>
     </row>
@@ -23190,11 +24198,11 @@
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>FOTO</t>
         </is>
       </c>
       <c r="D569" t="n">
-        <v>230.57</v>
+        <v>19.08</v>
       </c>
       <c r="K569" t="inlineStr"/>
     </row>
@@ -23211,11 +24219,11 @@
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D570" t="n">
-        <v>71.56999999999999</v>
+        <v>1048.6</v>
       </c>
       <c r="K570" t="inlineStr"/>
     </row>
@@ -23232,11 +24240,11 @@
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D571" t="n">
-        <v>198.72</v>
+        <v>720.84</v>
       </c>
       <c r="K571" t="inlineStr"/>
     </row>
@@ -23253,11 +24261,11 @@
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D572" t="n">
-        <v>25.41</v>
+        <v>197.2</v>
       </c>
       <c r="K572" t="inlineStr"/>
     </row>
@@ -23274,11 +24282,11 @@
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D573" t="n">
-        <v>203.57</v>
+        <v>274.61</v>
       </c>
       <c r="K573" t="inlineStr"/>
     </row>
@@ -23295,11 +24303,11 @@
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D574" t="n">
-        <v>156.17</v>
+        <v>230.57</v>
       </c>
       <c r="K574" t="inlineStr"/>
     </row>
@@ -23316,13 +24324,832 @@
       </c>
       <c r="C575" t="inlineStr">
         <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>71.56999999999999</v>
+      </c>
+      <c r="K575" t="inlineStr"/>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>198.72</v>
+      </c>
+      <c r="K576" t="inlineStr"/>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>747.5700000000001</v>
+      </c>
+      <c r="K577" t="inlineStr"/>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="K578" t="inlineStr"/>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>343.56</v>
+      </c>
+      <c r="K579" t="inlineStr"/>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>773.89</v>
+      </c>
+      <c r="K580" t="inlineStr"/>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>203.57</v>
+      </c>
+      <c r="K581" t="inlineStr"/>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
           <t>ZS</t>
         </is>
       </c>
-      <c r="D575" t="n">
+      <c r="D582" t="n">
         <v>216.81</v>
       </c>
-      <c r="K575" t="inlineStr"/>
+      <c r="K582" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Uptrend MA50</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>782.8099999999999</v>
+      </c>
+      <c r="K583" t="inlineStr"/>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>242.27</v>
+      </c>
+      <c r="K584" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>229.08</v>
+      </c>
+      <c r="K585" t="inlineStr"/>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>718.6</v>
+      </c>
+      <c r="K586" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>175.56</v>
+      </c>
+      <c r="K587" t="inlineStr"/>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Golden Cross</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>ZS</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>233.89</v>
+      </c>
+      <c r="K588" t="inlineStr"/>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>608.09</v>
+      </c>
+      <c r="K589" t="inlineStr"/>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>280.3</v>
+      </c>
+      <c r="K590" t="inlineStr"/>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>229.08</v>
+      </c>
+      <c r="K591" t="inlineStr"/>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>156.69</v>
+      </c>
+      <c r="K592" t="inlineStr"/>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>718.6</v>
+      </c>
+      <c r="K593" t="inlineStr"/>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>10.38</v>
+      </c>
+      <c r="K594" t="inlineStr"/>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>NOW</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>140.87</v>
+      </c>
+      <c r="K595" t="inlineStr"/>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Bull Flag Watch</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>SPOT</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>529.02</v>
+      </c>
+      <c r="K596" t="inlineStr"/>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>224.98</v>
+      </c>
+      <c r="K597" t="inlineStr"/>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>76.28</v>
+      </c>
+      <c r="K598" t="inlineStr"/>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>209.06</v>
+      </c>
+      <c r="K599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Breakout Watch (EOD)</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>368.92</v>
+      </c>
+      <c r="K600" t="inlineStr"/>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>50.13</v>
+      </c>
+      <c r="K601" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>CRWD</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>275.05</v>
+      </c>
+      <c r="K602" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>HACK</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>130.76</v>
+      </c>
+      <c r="K603" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>76.28</v>
+      </c>
+      <c r="K604" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Performance: Strong Buy</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>SNOW</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>368.92</v>
+      </c>
+      <c r="K605" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>LITE</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>1103.2</v>
+      </c>
+      <c r="K606" t="inlineStr"/>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>224.98</v>
+      </c>
+      <c r="K607" t="inlineStr"/>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>360.93</v>
+      </c>
+      <c r="K608" t="inlineStr"/>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>229.34</v>
+      </c>
+      <c r="K609" t="inlineStr"/>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D610" t="n">
+        <v>209.06</v>
+      </c>
+      <c r="K610" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D611" t="n">
+        <v>751.24</v>
+      </c>
+      <c r="K611" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D612" t="n">
+        <v>26.28</v>
+      </c>
+      <c r="K612" t="inlineStr"/>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="D613" t="n">
+        <v>206.81</v>
+      </c>
+      <c r="K613" t="inlineStr"/>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Performance: Buy</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>VST</t>
+        </is>
+      </c>
+      <c r="D614" t="n">
+        <v>161.46</v>
+      </c>
+      <c r="K614" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23447,7 +25274,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
         <v>8</v>
@@ -23486,22 +25313,22 @@
         <v>-1.06</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P2" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="Q2" t="n">
-        <v>1.08</v>
+        <v>-0.05</v>
       </c>
       <c r="R2" t="n">
-        <v>-1.04</v>
+        <v>-2.1</v>
       </c>
       <c r="S2" t="n">
-        <v>66.7</v>
+        <v>50</v>
       </c>
       <c r="T2" t="n">
-        <v>0.05</v>
+        <v>-0.73</v>
       </c>
     </row>
     <row r="3">
@@ -23511,61 +25338,61 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C3" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>46.8</v>
+        <v>48</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.2</v>
+        <v>0.09</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.89</v>
+        <v>-0.63</v>
       </c>
       <c r="G3" t="n">
-        <v>37.6</v>
+        <v>39.3</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.46</v>
+        <v>-0.18</v>
       </c>
       <c r="I3" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J3" t="n">
-        <v>51.6</v>
+        <v>51.9</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.27</v>
+        <v>-0.04</v>
       </c>
       <c r="L3" t="n">
-        <v>-1.09</v>
+        <v>-0.87</v>
       </c>
       <c r="M3" t="n">
-        <v>44.2</v>
+        <v>45.2</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.15</v>
       </c>
       <c r="O3" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="P3" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.37</v>
+        <v>7.21</v>
       </c>
       <c r="R3" t="n">
-        <v>5.25</v>
+        <v>5.23</v>
       </c>
       <c r="S3" t="n">
-        <v>75</v>
+        <v>76.5</v>
       </c>
       <c r="T3" t="n">
-        <v>6.83</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="4">
@@ -23575,61 +25402,61 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C4" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D4" t="n">
-        <v>64.3</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>2.21</v>
+        <v>2.31</v>
       </c>
       <c r="F4" t="n">
-        <v>1.29</v>
+        <v>1.38</v>
       </c>
       <c r="G4" t="n">
-        <v>58.2</v>
+        <v>57.7</v>
       </c>
       <c r="H4" t="n">
-        <v>1.74</v>
+        <v>1.86</v>
       </c>
       <c r="I4" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="J4" t="n">
-        <v>75</v>
+        <v>74.5</v>
       </c>
       <c r="K4" t="n">
-        <v>4.95</v>
+        <v>4.74</v>
       </c>
       <c r="L4" t="n">
-        <v>4.07</v>
+        <v>3.85</v>
       </c>
       <c r="M4" t="n">
-        <v>72.90000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="N4" t="n">
-        <v>4.76</v>
+        <v>4.86</v>
       </c>
       <c r="O4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="P4" t="n">
-        <v>81.8</v>
+        <v>84.2</v>
       </c>
       <c r="Q4" t="n">
-        <v>9.26</v>
+        <v>11.09</v>
       </c>
       <c r="R4" t="n">
-        <v>7.14</v>
+        <v>9.08</v>
       </c>
       <c r="S4" t="n">
-        <v>72.7</v>
+        <v>73.7</v>
       </c>
       <c r="T4" t="n">
-        <v>8.449999999999999</v>
+        <v>11.28</v>
       </c>
     </row>
     <row r="5">
@@ -23639,25 +25466,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" t="n">
-        <v>62.5</v>
+        <v>64</v>
       </c>
       <c r="E5" t="n">
-        <v>2.81</v>
+        <v>3.67</v>
       </c>
       <c r="F5" t="n">
-        <v>1.97</v>
+        <v>2.82</v>
       </c>
       <c r="G5" t="n">
-        <v>62.5</v>
+        <v>64</v>
       </c>
       <c r="H5" t="n">
-        <v>1.63</v>
+        <v>2.55</v>
       </c>
       <c r="I5" t="n">
         <v>20</v>
@@ -23678,7 +25505,22 @@
         <v>1.56</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S5" t="n">
+        <v>100</v>
+      </c>
+      <c r="T5" t="n">
+        <v>8.779999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -23688,61 +25530,61 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C6" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D6" t="n">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="E6" t="n">
-        <v>1.04</v>
+        <v>1.16</v>
       </c>
       <c r="F6" t="n">
-        <v>0.18</v>
+        <v>0.3</v>
       </c>
       <c r="G6" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="I6" t="n">
+        <v>66</v>
+      </c>
+      <c r="J6" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="M6" t="n">
         <v>50</v>
       </c>
-      <c r="H6" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="N6" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="O6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" t="n">
         <v>60</v>
       </c>
-      <c r="J6" t="n">
+      <c r="Q6" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="S6" t="n">
         <v>60</v>
       </c>
-      <c r="K6" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="M6" t="n">
-        <v>53.3</v>
-      </c>
-      <c r="N6" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="O6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P6" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>-0.67</v>
-      </c>
-      <c r="R6" t="n">
-        <v>-2.79</v>
-      </c>
-      <c r="S6" t="n">
-        <v>50</v>
-      </c>
       <c r="T6" t="n">
-        <v>-0.92</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="7">
@@ -23752,61 +25594,61 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C7" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D7" t="n">
-        <v>56.7</v>
+        <v>58.1</v>
       </c>
       <c r="E7" t="n">
-        <v>1.51</v>
+        <v>1.79</v>
       </c>
       <c r="F7" t="n">
-        <v>0.77</v>
+        <v>1.04</v>
       </c>
       <c r="G7" t="n">
-        <v>46.7</v>
+        <v>48.4</v>
       </c>
       <c r="H7" t="n">
-        <v>1.31</v>
+        <v>1.59</v>
       </c>
       <c r="I7" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J7" t="n">
-        <v>59.7</v>
+        <v>57.6</v>
       </c>
       <c r="K7" t="n">
-        <v>1.74</v>
+        <v>1.42</v>
       </c>
       <c r="L7" t="n">
-        <v>0.98</v>
+        <v>0.65</v>
       </c>
       <c r="M7" t="n">
-        <v>58.1</v>
+        <v>56.1</v>
       </c>
       <c r="N7" t="n">
-        <v>1.91</v>
+        <v>1.62</v>
       </c>
       <c r="O7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P7" t="n">
         <v>33.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>2.33</v>
+        <v>2.23</v>
       </c>
       <c r="R7" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="S7" t="n">
         <v>33.3</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.8</v>
+        <v>5.47</v>
       </c>
     </row>
     <row r="9">

</xml_diff>